<commit_message>
fix: light theme LivingBackground dimming only in dark mode
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2845FEF-0906-4AA1-80F0-30CDEDD8980B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A7EA4F-C085-4AEC-8F07-75BE160892B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1922" uniqueCount="841">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="847">
   <si>
     <t>Артикул</t>
   </si>
@@ -4946,6 +4946,78 @@
 Бренд: SMART DERMA
 Країна виробництва: 🇺🇦 Україна
 🌟 Arabica Coffee Eye Mask – твій must-have для сяючого та молодого погляду без темних кіл і набряків! 🌟</t>
+  </si>
+  <si>
+    <t>Інтелектуальна сироватка-елексир "БІОПЛАЗМА" з мультипептидами - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Bioplasma Peptide Elixir – концентрований інтелектуальний догляд! ✨
+🌿 Високотехнологічна формула для комплексного омолодження:
+💎 Відновлює пружність та еластичність завдяки комплексу пептидів
+💧 Забезпечує глибоке зволоження гіалуроновою кислотою
+🌸 Омега-насичена лляна олія живить та розгладжує
+🛡️ Активізує регенераційні процеси та захищає від стресу
+🌟 Дарує шкірі гладкість, сяйво та молодість
+💚 Результат – тонкі лінії та зморшки розгладжуються, шкіра виглядає здоровою та оновленою!
+📌 Ключові активні компоненти:
+🌱 Bioplasma™ FA та комплекс пептидів (Replexium, CAPS2GO™, Argireline, Agefinity™) – стимуляція синтезу колагену та регенерація
+💧 Гіалуронат натрію, Hyalurosmooth PW LS 8997, Hydagen® Aquaporin – глибоке зволоження та підтримка водного балансу
+🥥 Лляна олія, масла ши та авокадо – живлення та відновлення бар’єру
+🌸 Антарктицин, Easyliance, біотин трипептид-1 – ревіталізація та зміцнення шкіри
+⚡ Ацетил тетрапептид-2, ацетил гексапептид-1, олігопептиди та поліпептиди – омолодження та корекція зморшок
+📌 Показання до застосування:
+Щоденний догляд для уповільнення старіння
+Запобігання зморшкам
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація та знижений тонус
+Догляд після інвазивних процедур
+Вікова шкіра
+📌 Як застосовувати:  
+Нанеси кілька крапель еліксиру на очищену шкіру обличчя та шиї. Використовуй щодня для максимального ефекту омолодження.
+✔️ Характеристики продукту:
+Тип: Інтелектуальна антивікова сироватка-еліксир
+Об’єм: 50 мл
+Призначення: Омолодження, зволоження, відновлення, живлення
+Тип шкіри: Зріла, суха, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Bioplasma Peptide Elixir – твій must-have для молодої та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>704</t>
+  </si>
+  <si>
+    <t>Інтелектуального заповнювального Гідромісту – 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Intelligent HydroMist – багатофункціональне зволоження та anti-age догляд! ✨
+🌿 Інноваційна формула для щоденного відновлення:
+💧 Миттєве та пролонговане зволоження
+🌸 Нормалізація pH та вирівнювання тону шкіри
+💎 Зменшення глибини зморшок та профілактика їх появи
+🛡️ Захист від сухості та еритеми
+🌟 Ефект сяйва зсередини
+💚 Результат – свіжа, гладка та сяюча шкіра щодня!
+📌 Ключові активні компоненти:
+❄️ Antarcticine® – морський інгредієнт із криопротекторними властивостями
+💧 Гіалуронат натрію та Hydagen® Aquaporin – глибоке зволоження та підтримка водного балансу
+🌱 SPAR'AGE™ та морські мінерали – ревіталізація та захист
+🌸 Амінокислоти та пантенол – живлення, відновлення та зміцнення шкіри
+📌 Показання до застосування:
+Щоденний догляд за віковою шкірою
+Профілактика старіння
+Відновлення після косметологічних процедур
+Борьба з гіперпігментацією та зниженим тонусом
+✔️ Характеристики продукту:
+Тип: Інтелектуальний заповнювальний гідроміст
+Об’єм: 250 мл
+Призначення: Зволоження, омолодження, захист, сяйво
+Тип шкіри: Всі типи, особливо суха та зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Intelligent HydroMist – твій must-have для миттєвого зволоження та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>703</t>
   </si>
 </sst>
 </file>
@@ -7345,38 +7417,66 @@
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="12"/>
-      <c r="B63" s="8"/>
+      <c r="A63" s="12" t="s">
+        <v>843</v>
+      </c>
+      <c r="B63" s="8" t="s">
+        <v>841</v>
+      </c>
       <c r="C63" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D63" s="8"/>
+      <c r="D63" s="8">
+        <v>1140</v>
+      </c>
       <c r="E63" s="8"/>
       <c r="F63" s="8"/>
-      <c r="G63" s="8"/>
-      <c r="H63" s="8"/>
+      <c r="G63" s="8">
+        <v>16</v>
+      </c>
+      <c r="H63" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I63" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J63" s="8"/>
-      <c r="K63" s="18"/>
+      <c r="J63" s="8" t="s">
+        <v>842</v>
+      </c>
+      <c r="K63" s="18" t="s">
+        <v>843</v>
+      </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="12"/>
-      <c r="B64" s="8"/>
+      <c r="A64" s="12" t="s">
+        <v>846</v>
+      </c>
+      <c r="B64" s="8" t="s">
+        <v>844</v>
+      </c>
       <c r="C64" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D64" s="8"/>
+      <c r="D64" s="8">
+        <v>1000</v>
+      </c>
       <c r="E64" s="8"/>
       <c r="F64" s="8"/>
-      <c r="G64" s="8"/>
-      <c r="H64" s="8"/>
+      <c r="G64" s="8">
+        <v>19</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>672</v>
+      </c>
       <c r="I64" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J64" s="8"/>
-      <c r="K64" s="18"/>
+      <c r="J64" s="8" t="s">
+        <v>845</v>
+      </c>
+      <c r="K64" s="18" t="s">
+        <v>846</v>
+      </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" s="12"/>

</xml_diff>

<commit_message>
fix: light theme no dark flash on scroll; product description with proper paragraphs
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6A7EA4F-C085-4AEC-8F07-75BE160892B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD68DCB2-8C38-491A-B141-9C853EA50B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1932" uniqueCount="847">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="878">
   <si>
     <t>Артикул</t>
   </si>
@@ -5018,6 +5018,339 @@
   </si>
   <si>
     <t>703</t>
+  </si>
+  <si>
+    <t>Гель для вмивання "Активатор Енергії" з кислотами - 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Energy Activator Cleansing Gel – перезарядка для твоєї шкіри! ✨
+🌿 Інноваційна формула з кислотами та ензимами:
+⚡ Перезаряджає клітини шкіри на 27%
+💧 Відновлює pH-баланс та підтримує оптимальний рівень зволоження
+🌸 Комплекс із трьох кислот у розчині електролітів – м’яке, але ефективне очищення
+🛡️ Компонент OXY 229 PF активує мітохондріальне дихання для енергії клітин
+💎 Дарує свіжість, сяйво та рівний тон
+💚 Результат – чиста, енергійна та сяюча шкіра після кожного вмивання!
+📌 Ключові активні компоненти:
+🌱 Гліколева, піруватна та ферулова кислоти – ексфоліація та вирівнювання тону
+⚡ OXY 229 PF – активація клітинної енергії
+💧 Гіалуронат натрію, сечовина, Д-пантенол – глибоке зволоження та відновлення
+🌸 Екстракт гібіскуса, морські мінерали – антиоксидантний захист та тонізація
+🌟 Hydagen® Aquaporin, Lys'lastine™ V, Perlaura® – підтримка водного балансу та пружності
+📌 Показання до застосування:
+Уповільнення старіння без радикальних методів
+Запобігання появі зморшок
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Догляд після інвазивних процедур
+📌 Як застосовувати:  
+Нанеси невелику кількість гелю на вологу шкіру, розподіли по масажних лініях, легко промасажуй та змий теплою водою. Використовуй щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Інноваційний гель для вмивання
+Об’єм: 250 мл
+Призначення: Очищення, омолодження, відновлення енергії клітин
+Тип шкіри: Вікова, комбінована, проблемна
+Країна виробництва: 🇺🇦 Україна
+🌟 Energy Activator Cleansing Gel – твій must-have для щоденного енергетичного догляду! 🌟</t>
+  </si>
+  <si>
+    <t>700</t>
+  </si>
+  <si>
+    <t>SMART4DERMA Aquagen - Двоетапна система інтенсивного зволоження 2х75</t>
+  </si>
+  <si>
+    <t>2х75 мл</t>
+  </si>
+  <si>
+    <t>✨ SMART4DERMA Aquagen – інноваційна система догляду з урахуванням циркадних ритмів! ✨
+🌿 Двоетапна формула для глибокого зволоження, живлення та ревіталізації:
+💧 Відновлює баланс вологи та мікробіом шкіри
+🌸 Стимулює синтез колагену та забезпечує ліфтинг
+💎 Освітлює пігментацію та повертає природне сяйво
+🛡️ Захищає від зовнішніх факторів та фотостаріння
+💚 Результат – пружна, сяюча та здорова шкіра з ефектом перетворення!
+📌 Система включає дві маски:
+1️⃣ 4D Aqua Mask Vita C &amp; Probiotic (75 мл)
+Збагачена вітамінами та пребіотиками
+Містить чотири види гіалуронової кислоти
+Відновлює мікробіом, покращує тон та тургор
+Захищає від зовнішніх факторів
+2️⃣ Bakuchiol Mask Ceramides &amp; AA2G (75 мл)
+Глибоко зволожує та оздоровлює шкіру
+Розгладжує зморшки та освітлює пігментацію
+Повертає природне сяйво та еластичність
+📌 Активні інгредієнти:
+🌱 Крок 1: Сік алое, Hydagen® Aquaporin, 4D гіалуронова кислота, пребіотики, Д-пантенол, вітаміни В3 і С, кофеїн, біотин, Amitose 3GA
+🌸 Крок 2: Олії ши та оливки, бакухіол, сквалан, BIO CERAMIDYL PURE, гідролізовані протеїни пшениці, вівса, шовку та рису
+✔️ Характеристики продукту:
+Тип: Двоетапна система інтенсивного зволоження
+Об’єм: 2×75 мл
+Призначення: Зволоження, живлення, ліфтинг, освітлення
+Тип шкіри: Всі типи, особливо суха та зріла
+Бренд: SMART4DERMA
+Країна виробництва: 🇺🇦 Україна
+🌟 SMART4DERMA Aquagen – твій must-have для глибокого зволоження та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>520</t>
+  </si>
+  <si>
+    <t>Розкішний живильний крем з церамідами 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Luxury Ceramide Nourishing Cream – глибоке живлення та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Технологія подвійного зволоження – миттєвий та тривалий ефект
+🌸 Церамиди зміцнюють захисний бар’єр шкіри
+🥥 Комплекс Multifeel забезпечує інтенсивне живлення
+🌟 Пантенол заспокоює та відновлює
+💎 Зменшує глибину зморшок, підвищує пружність та еластичність
+💚 Результат – гладка, сяюча та здорова шкіра щодня!
+📌 Показання до застосування:
+Суха та зневоднена шкіра
+Зріла та чутлива шкіра
+Всі типи шкіри для щоденного догляду
+Відновлення після косметичних процедур
+✔️ Характеристики продукту:
+Тип: Живильний крем з церамідами
+Об’єм: 50 мл / 100 мл (залежно від упаковки)
+Призначення: Зволоження, живлення, відновлення, омолодження
+Тип шкіри: Всі типи, особливо суха та зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Ceramide Nourishing Cream – твій must-have для глибокого живлення та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>525</t>
+  </si>
+  <si>
+    <t>Невагомий Крем-гель SPF 50 - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Weightless SPF 50 Gel-Cream – щоденний захист та зволоження! ✨
+🌿 Інноваційна формула для комфортного щоденного догляду:
+☀️ Потужний УФ-захист: комплекс PolyFructol Plus та X50 Skin Barrier запобігає фотостарінню та передчасним зморшкам
+💧 Глибоке зволоження: технологія PatcH2O та Hydagen® Aquaporine працюють на клітинному рівні
+🛡️ Антиоксидантний захист: DN-Age нейтралізує вільні радикали та стрес
+🌸 Легка текстура: миттєво вбирається без липкості, даруючи комфорт
+💚 Результат – пружна, гладка та захищена шкіра з ефектом свіжості після кожного нанесення!
+📌 Показання до застосування:
+Щоденний догляд для всіх типів шкіри
+Захист від фото- та хроностаріння
+Профілактика зморшок та пігментації
+Зволоження та підтримка клітинного балансу
+📌 Як застосовувати:  
+Наносити на чисту, суху шкіру обличчя за 20 хвилин до виходу на сонце. Використовувати щодня для максимального захисту.
+✔️ Характеристики продукту:
+Тип: Крем-гель з SPF
+Об’єм: 50 мл / 230 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Всі типи
+Країна виробництва: 🇺🇦 Україна
+🌟 Weightless SPF 50 Gel-Cream – твій must-have для щоденного захисту та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>524</t>
+  </si>
+  <si>
+    <t>Постпроцедурний захисний регенерувальний спрей SPF50, 150 мл</t>
+  </si>
+  <si>
+    <t>518</t>
+  </si>
+  <si>
+    <t>✨ Post-Procedure Protective Spray SPF 50 – професійний догляд та відновлення! ✨
+🌿 Інноваційна формула для чутливої та пошкодженої шкіри:
+☀️ Максимальний захист SPF 50 від UVA/UVB-випромінювання
+💧 Відновлює оптимальний рівень зволоження без відчуття важкості
+🌸 Заспокоює подразнення та зменшує сухість
+🛡️ Сприяє регенерації та відновленню бар’єрної функції
+⚡ Зручний формат спрею для рівномірного нанесення
+💚 Результат – захищена, зволожена та відновлена шкіра після процедур!
+📌 Показання до застосування:
+Догляд після пілінгів, лазерних процедур, шліфування
+Суха та чутлива шкіра
+Роздратування та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Захисний регенерувальний спрей
+Об’єм: 150 мл
+Фактор захисту: SPF 50
+Спектр: UVA/UVB
+Водостійкий, гіпоалергенний
+Без вікових обмежень
+Країна виробництва: 🇺🇦 Україна
+🌟 Post-Procedure Protective Spray SPF 50 – твій must-have для безпечного та комфортного відновлення шкіри після процедур! 🌟</t>
+  </si>
+  <si>
+    <t>Сонцезахисний ультразволожувальний крем SPF50 з олією канабісу 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Cannabis Ultra-Hydrating Sunscreen SPF 50 – повний спектр захисту та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+☀️ SPF50 + широкоспектральний UVA/UVB-захист – профілактика фотостаріння та збереження колагену
+💧 Гіалуронова кислота + PolyFructol Plus – глибоке зволоження та підтримка водного балансу
+🌸 Екстракт азіатської центелли – заспокоює та відновлює бар’єрні функції
+🛡️ Токоферол ацетат та аскорбіл глюкозид – антиоксидантний захист від стресу та вільних радикалів
+🌟 Легка текстура з матуючим ефектом – без відчуття тяжкості
+💚 Результат – пружна, сяюча та захищена шкіра щодня!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Перші ознаки старіння
+Зниження бар’єрної функції
+📌 Як застосовувати:  
+Наносити на очищену шкіру обличчя вранці, за 20 хвилин до виходу на сонце. Використовувати щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Сонцезахисний крем з SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Cannabis Ultra-Hydrating Sunscreen SPF 50 – твій must-have для щоденного захисту та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>517</t>
+  </si>
+  <si>
+    <t>Ультразволожуючий бустер х50 "Поліфруктол", 30 мл</t>
+  </si>
+  <si>
+    <t>510</t>
+  </si>
+  <si>
+    <t>✨ Polyfructol x50 Ultra-Hydrating Booster – інноваційна енергія зволоження! ✨
+🌿 Передова дрон-молекулярна система доставки:
+💧 Миттєва, глибока та пролонгована гідратація
+🌸 Стимулює природне продукування гіалуронової кислоти
+🛡️ Відновлює водний баланс та бар’єрні функції шкіри
+⚡ Зменшує запальні процеси та подразнення
+🌟 Покращує текстуру та еластичність
+💚 Результат – шкіра стає свіжою, пружною та сяючою вже після першого застосування!
+📌 Ключові активні компоненти:
+🌱 Skin Barrier та Polyfructol Plus – захист та пролонговане зволоження
+🌿 Олія коноплі та екстракт зеленого чаю – антиоксидантний щит та живлення
+💧 Бета-глюкан, трегалоза, альгін – глибоке зволоження та відновлення
+🌸 Purisoft™ LS 9836 – детокс та захист від зовнішніх факторів
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Антиоксидантний ультразволожуючий бустер
+Об’єм: 30 мл
+Призначення: Зволоження, живлення, антиоксидантний захист
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Polyfructol x50 Booster – твій must-have для екстра зволоження та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Удосконалювало ний зволожувальний СС КРЕМ SPF30 - 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Advanced Moisturizing CC Cream SPF 30 – ідеальний тон та захист! ✨
+🌿 Мультифункціональна формула для щоденного догляду:
+💎 Пігменти в мікрокапсулах адаптуються до відтінку шкіри
+🌸 Вирівнює тон та дарує миттєвий ефект свіжості
+☀️ Захист від ультрафіолету завдяки SPF 30
+💧 Легка текстура – не забиває пори та забезпечує комфорт
+💚 Результат – рівний тон, сяйво та захищена шкіра щодня!
+📌 Ключові активні компоненти:
+🥥 Масло насіння жожоба та ши – живлення та м’якість
+🌿 Екстракт камелії – стимуляція регенерації
+💧 Гіалуронат натрію – інтенсивне зволоження
+🛡️ Оксид цинку – захист від UVA/UVB-променів
+🌸 Пчелиний віск – заспокоює та утримує вологу
+⚡ Ацетил гексапептид-8 – зменшення зморшок
+🌟 Вітамін Е та лецитин – антиоксидантний захист та баланс
+📌 Як застосовувати:  
+Нанеси крем на чисту шкіру обличчя, шиї та декольте масажними рухами. Використовуй щодня для рівного тону та захисту від сонця.
+✔️ Характеристики продукту:
+Тип: Зволожувальний СС крем з SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Тонування, зволоження, захист, омолодження
+Тип шкіри: Всі типи, особливо суха та чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced CC Cream SPF 30 – твій must-have для ідеального тону та щоденного захисту! 🌟</t>
+  </si>
+  <si>
+    <t>519</t>
+  </si>
+  <si>
+    <t>Екстразволожувальний крем із церамідами SPF30 суха та нормальна шкіра</t>
+  </si>
+  <si>
+    <t>✨ Ceramide Extra-Hydrating Cream SPF 30 – подвійний захист та зволоження! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Комплекс церамідів I–IV, VI – відновлює бар’єрну функцію та зміцнює шкіру
+🌸 Гіалуронова кислота + гліцерил глюкозид – пролонговане зволоження на клітинному рівні
+🛡️ Антиоксидантний щит – ферулова кислота, токоферол ацетат та екстракт зеленого чаю нейтралізують вільні радикали
+☀️ SPF 30 широкого спектру – невидимий сонцезахисний щит проти UVA/UVB
+🌟 PatcH20 та Hydagen® Aquaporin – підтримка водного балансу та пружності
+💚 Результат – гладка, сяюча та захищена шкіра без сухості та подразнень!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу та перші ознаки старіння
+Відновлення та захист бар’єрної функції
+📌 Активні компоненти:
+🌱 Оливкова олія, екстракт ромашки, центелла азіатська
+💧 Hydagen® Aquaporin, PatcH20, Д-пантенол
+🛡️ iActive Ceramide, X50 Skin Barrier, Phytosoothe LS 9766
+🌸 Токоферол ацетат, натрій аскорбіл фосфат, ферулова кислота, бісаболол
+✔️ Характеристики продукту:
+Тип: Екстразволожувальний крем із SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Зволоження, живлення, антиоксидантний захист, сонцезахист
+Тип шкіри: Суха, нормальна, чутлива
+Країна виробництва: 🇺🇦 Україна
+🌟 Ceramide Extra-Hydrating Cream SPF 30 – твій must-have для щоденного зволоження та захисту шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>506</t>
+  </si>
+  <si>
+    <t>Крем-маска глибоке зволоження 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Deep Moisture Cream-Mask – миттєве та пролонговане зволоження! ✨
+🌿 Легка пептидна формула з системою доставки X50:
+💧 Створює депо вологи в шкірі для подвійного ефекту гідратації
+🌸 Відновлює бар’єрні функції завдяки комплексу церамідів
+🛡️ Заспокоює подразнення та зменшує сухість
+⚡ Підвищує тонус та еластичність шкіри
+🌟 Дарує свіжість і сяйво вже після першого застосування
+💚 Результат – шкіра стає пружною, гладкою та сяючою!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист шкіри
+📌 Ключові активні компоненти:
+💧 Hydagen® Aquaporin, гіалуронат натрію, PolyFructol Plus – інтенсивне зволоження
+🌱 Олія авокадо, примули, екстракт центелли – живлення та відновлення
+🌸 Д-пантенол, ніацинамід, бета-глюкан – заспокійливий та регенеруючий ефект
+🛡️ iActive Ceramide, X50 Skin Barrier, токоферол, ферулова кислота, убіхінон – антиоксидантний захист та зміцнення бар’єру
+⚡ Амінокислоти та магнезіум аскорбіл фосфат – стимуляція клітинного оновлення
+✔️ Характеристики продукту:
+Тип: Крем-маска для глибокого зволоження
+Об’єм: 300 мл
+Призначення: Зволоження, живлення, відновлення, антиоксидантний захист
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Deep Moisture Cream-Mask – твій must-have для миттєвого та тривалого зволоження! 🌟</t>
+  </si>
+  <si>
+    <t>514</t>
   </si>
 </sst>
 </file>
@@ -7479,260 +7812,448 @@
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="12"/>
-      <c r="B65" s="8"/>
+      <c r="A65" s="12" t="s">
+        <v>849</v>
+      </c>
+      <c r="B65" s="8" t="s">
+        <v>847</v>
+      </c>
       <c r="C65" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D65" s="8"/>
+      <c r="D65" s="8">
+        <v>780</v>
+      </c>
       <c r="E65" s="8"/>
       <c r="F65" s="8"/>
-      <c r="G65" s="8"/>
-      <c r="H65" s="8"/>
+      <c r="G65" s="8">
+        <v>16</v>
+      </c>
+      <c r="H65" s="8" t="s">
+        <v>672</v>
+      </c>
       <c r="I65" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J65" s="8"/>
-      <c r="K65" s="18"/>
+      <c r="J65" s="8" t="s">
+        <v>848</v>
+      </c>
+      <c r="K65" s="18" t="s">
+        <v>849</v>
+      </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="12"/>
-      <c r="B66" s="8"/>
+      <c r="A66" s="12" t="s">
+        <v>853</v>
+      </c>
+      <c r="B66" s="8" t="s">
+        <v>850</v>
+      </c>
       <c r="C66" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D66" s="8"/>
+      <c r="D66" s="8">
+        <v>1320</v>
+      </c>
       <c r="E66" s="8"/>
       <c r="F66" s="8"/>
-      <c r="G66" s="8"/>
-      <c r="H66" s="8"/>
+      <c r="G66" s="8">
+        <v>19</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>851</v>
+      </c>
       <c r="I66" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J66" s="8"/>
-      <c r="K66" s="18"/>
+      <c r="J66" s="8" t="s">
+        <v>852</v>
+      </c>
+      <c r="K66" s="18" t="s">
+        <v>853</v>
+      </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="12"/>
-      <c r="B67" s="8"/>
+      <c r="A67" s="12" t="s">
+        <v>856</v>
+      </c>
+      <c r="B67" s="8" t="s">
+        <v>854</v>
+      </c>
       <c r="C67" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D67" s="8"/>
+      <c r="D67" s="8">
+        <v>680</v>
+      </c>
       <c r="E67" s="8"/>
       <c r="F67" s="8"/>
-      <c r="G67" s="8"/>
-      <c r="H67" s="8"/>
+      <c r="G67" s="8">
+        <v>25</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I67" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J67" s="8"/>
-      <c r="K67" s="18"/>
+      <c r="J67" s="8" t="s">
+        <v>855</v>
+      </c>
+      <c r="K67" s="18" t="s">
+        <v>856</v>
+      </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="12"/>
-      <c r="B68" s="8"/>
+      <c r="A68" s="12" t="s">
+        <v>859</v>
+      </c>
+      <c r="B68" s="8" t="s">
+        <v>857</v>
+      </c>
       <c r="C68" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D68" s="8"/>
+      <c r="D68" s="8">
+        <v>980</v>
+      </c>
       <c r="E68" s="8"/>
       <c r="F68" s="8"/>
-      <c r="G68" s="8"/>
-      <c r="H68" s="8"/>
+      <c r="G68" s="8">
+        <v>17</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I68" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J68" s="8"/>
-      <c r="K68" s="18"/>
+      <c r="J68" s="8" t="s">
+        <v>858</v>
+      </c>
+      <c r="K68" s="18" t="s">
+        <v>859</v>
+      </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="12"/>
-      <c r="B69" s="8"/>
+      <c r="A69" s="12" t="s">
+        <v>861</v>
+      </c>
+      <c r="B69" s="8" t="s">
+        <v>860</v>
+      </c>
       <c r="C69" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D69" s="8"/>
+      <c r="D69" s="8">
+        <v>1260</v>
+      </c>
       <c r="E69" s="8"/>
       <c r="F69" s="8"/>
-      <c r="G69" s="8"/>
-      <c r="H69" s="8"/>
+      <c r="G69" s="8">
+        <v>21</v>
+      </c>
+      <c r="H69" s="8" t="s">
+        <v>695</v>
+      </c>
       <c r="I69" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J69" s="8"/>
-      <c r="K69" s="18"/>
+      <c r="J69" s="8" t="s">
+        <v>862</v>
+      </c>
+      <c r="K69" s="18" t="s">
+        <v>861</v>
+      </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="12"/>
-      <c r="B70" s="8"/>
+      <c r="A70" s="12" t="s">
+        <v>865</v>
+      </c>
+      <c r="B70" s="8" t="s">
+        <v>863</v>
+      </c>
       <c r="C70" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D70" s="8"/>
+      <c r="D70" s="8">
+        <v>1020</v>
+      </c>
       <c r="E70" s="8"/>
       <c r="F70" s="8"/>
-      <c r="G70" s="8"/>
-      <c r="H70" s="8"/>
-      <c r="I70" s="8"/>
-      <c r="J70" s="8"/>
-      <c r="K70" s="18"/>
+      <c r="G70" s="8">
+        <v>26</v>
+      </c>
+      <c r="H70" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I70" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J70" s="8" t="s">
+        <v>864</v>
+      </c>
+      <c r="K70" s="18" t="s">
+        <v>865</v>
+      </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="12"/>
-      <c r="B71" s="9"/>
-      <c r="C71" s="9"/>
-      <c r="D71" s="8"/>
+      <c r="A71" s="12" t="s">
+        <v>867</v>
+      </c>
+      <c r="B71" s="8" t="s">
+        <v>866</v>
+      </c>
+      <c r="C71" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D71" s="8">
+        <v>980</v>
+      </c>
       <c r="E71" s="8"/>
       <c r="F71" s="8"/>
-      <c r="G71" s="8"/>
-      <c r="H71" s="8"/>
-      <c r="I71" s="8"/>
-      <c r="J71" s="9"/>
-      <c r="K71" s="15"/>
+      <c r="G71" s="8">
+        <v>16</v>
+      </c>
+      <c r="H71" s="8" t="s">
+        <v>664</v>
+      </c>
+      <c r="I71" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J71" s="8" t="s">
+        <v>868</v>
+      </c>
+      <c r="K71" s="18" t="s">
+        <v>867</v>
+      </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="12"/>
-      <c r="B72" s="9"/>
-      <c r="C72" s="9"/>
-      <c r="D72" s="8"/>
+      <c r="A72" s="12" t="s">
+        <v>871</v>
+      </c>
+      <c r="B72" s="8" t="s">
+        <v>869</v>
+      </c>
+      <c r="C72" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D72" s="8">
+        <v>1220</v>
+      </c>
       <c r="E72" s="8"/>
       <c r="F72" s="8"/>
-      <c r="G72" s="8"/>
-      <c r="H72" s="8"/>
-      <c r="I72" s="8"/>
-      <c r="J72" s="9"/>
-      <c r="K72" s="15"/>
+      <c r="G72" s="8">
+        <v>17</v>
+      </c>
+      <c r="H72" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I72" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J72" s="8" t="s">
+        <v>870</v>
+      </c>
+      <c r="K72" s="18" t="s">
+        <v>871</v>
+      </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="12"/>
-      <c r="B73" s="9"/>
-      <c r="C73" s="9"/>
-      <c r="D73" s="8"/>
+      <c r="A73" s="12" t="s">
+        <v>874</v>
+      </c>
+      <c r="B73" s="8" t="s">
+        <v>872</v>
+      </c>
+      <c r="C73" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D73" s="8">
+        <v>1140</v>
+      </c>
       <c r="E73" s="8"/>
       <c r="F73" s="8"/>
-      <c r="G73" s="8"/>
-      <c r="H73" s="8"/>
-      <c r="I73" s="8"/>
-      <c r="J73" s="9"/>
-      <c r="K73" s="15"/>
+      <c r="G73" s="8">
+        <v>21</v>
+      </c>
+      <c r="H73" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I73" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J73" s="8" t="s">
+        <v>873</v>
+      </c>
+      <c r="K73" s="18" t="s">
+        <v>874</v>
+      </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="12"/>
-      <c r="B74" s="9"/>
-      <c r="C74" s="9"/>
-      <c r="D74" s="8"/>
+      <c r="A74" s="12" t="s">
+        <v>877</v>
+      </c>
+      <c r="B74" s="8" t="s">
+        <v>875</v>
+      </c>
+      <c r="C74" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D74" s="8">
+        <v>780</v>
+      </c>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
-      <c r="G74" s="8"/>
-      <c r="H74" s="8"/>
-      <c r="I74" s="8"/>
-      <c r="J74" s="9"/>
-      <c r="K74" s="15"/>
+      <c r="G74" s="8">
+        <v>24</v>
+      </c>
+      <c r="H74" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I74" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J74" s="8" t="s">
+        <v>876</v>
+      </c>
+      <c r="K74" s="18" t="s">
+        <v>877</v>
+      </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" s="12"/>
-      <c r="B75" s="9"/>
-      <c r="C75" s="9"/>
+      <c r="B75" s="8"/>
+      <c r="C75" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D75" s="8"/>
       <c r="E75" s="8"/>
       <c r="F75" s="8"/>
       <c r="G75" s="8"/>
       <c r="H75" s="8"/>
-      <c r="I75" s="8"/>
-      <c r="J75" s="9"/>
-      <c r="K75" s="15"/>
+      <c r="I75" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J75" s="8"/>
+      <c r="K75" s="18"/>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" s="12"/>
-      <c r="B76" s="9"/>
-      <c r="C76" s="9"/>
+      <c r="B76" s="8"/>
+      <c r="C76" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D76" s="8"/>
       <c r="E76" s="8"/>
       <c r="F76" s="8"/>
       <c r="G76" s="8"/>
       <c r="H76" s="8"/>
-      <c r="I76" s="8"/>
-      <c r="J76" s="9"/>
-      <c r="K76" s="15"/>
+      <c r="I76" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J76" s="8"/>
+      <c r="K76" s="18"/>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" s="12"/>
-      <c r="B77" s="9"/>
-      <c r="C77" s="9"/>
+      <c r="B77" s="8"/>
+      <c r="C77" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D77" s="8"/>
       <c r="E77" s="8"/>
       <c r="F77" s="8"/>
       <c r="G77" s="8"/>
       <c r="H77" s="8"/>
-      <c r="I77" s="8"/>
-      <c r="J77" s="9"/>
-      <c r="K77" s="15"/>
+      <c r="I77" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J77" s="8"/>
+      <c r="K77" s="18"/>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" s="12"/>
-      <c r="B78" s="9"/>
-      <c r="C78" s="9"/>
+      <c r="B78" s="8"/>
+      <c r="C78" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D78" s="8"/>
       <c r="E78" s="8"/>
       <c r="F78" s="8"/>
       <c r="G78" s="8"/>
       <c r="H78" s="8"/>
-      <c r="I78" s="8"/>
-      <c r="J78" s="9"/>
-      <c r="K78" s="15"/>
+      <c r="I78" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J78" s="8"/>
+      <c r="K78" s="18"/>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" s="12"/>
-      <c r="B79" s="9"/>
-      <c r="C79" s="9"/>
+      <c r="B79" s="8"/>
+      <c r="C79" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D79" s="8"/>
       <c r="E79" s="8"/>
       <c r="F79" s="8"/>
       <c r="G79" s="8"/>
       <c r="H79" s="8"/>
-      <c r="I79" s="8"/>
-      <c r="J79" s="9"/>
-      <c r="K79" s="15"/>
+      <c r="I79" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J79" s="8"/>
+      <c r="K79" s="18"/>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80" s="12"/>
-      <c r="B80" s="9"/>
-      <c r="C80" s="9"/>
+      <c r="B80" s="8"/>
+      <c r="C80" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D80" s="8"/>
       <c r="E80" s="8"/>
       <c r="F80" s="8"/>
       <c r="G80" s="8"/>
       <c r="H80" s="8"/>
-      <c r="I80" s="8"/>
-      <c r="J80" s="9"/>
-      <c r="K80" s="15"/>
+      <c r="I80" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J80" s="8"/>
+      <c r="K80" s="18"/>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81" s="12"/>
-      <c r="B81" s="9"/>
-      <c r="C81" s="9"/>
+      <c r="B81" s="8"/>
+      <c r="C81" s="8" t="s">
+        <v>653</v>
+      </c>
       <c r="D81" s="8"/>
       <c r="E81" s="8"/>
       <c r="F81" s="8"/>
       <c r="G81" s="8"/>
       <c r="H81" s="8"/>
-      <c r="I81" s="8"/>
-      <c r="J81" s="9"/>
-      <c r="K81" s="15"/>
+      <c r="I81" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J81" s="8"/>
+      <c r="K81" s="18"/>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82" s="12"/>
-      <c r="B82" s="9"/>
-      <c r="C82" s="9"/>
+      <c r="B82" s="8"/>
+      <c r="C82" s="8"/>
       <c r="D82" s="8"/>
       <c r="E82" s="8"/>
       <c r="F82" s="8"/>
       <c r="G82" s="8"/>
       <c r="H82" s="8"/>
-      <c r="I82" s="8"/>
-      <c r="J82" s="9"/>
-      <c r="K82" s="15"/>
+      <c r="I82" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J82" s="8"/>
+      <c r="K82" s="18"/>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" s="12"/>

</xml_diff>

<commit_message>
feat: product detail - cutout image, beautiful description with notes/ingredients tables
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD68DCB2-8C38-491A-B141-9C853EA50B9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C81592AE-E6FD-4959-B8DD-B468DE8D66AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2006" uniqueCount="878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2016" uniqueCount="884">
   <si>
     <t>Артикул</t>
   </si>
@@ -5351,6 +5351,76 @@
   </si>
   <si>
     <t>514</t>
+  </si>
+  <si>
+    <t>Зволожувальний дренажний крем від темних кіл та набряків 30 мл</t>
+  </si>
+  <si>
+    <t>✨ Drainage Moisturizing Eye Cream – свіжий та сяючий погляд! ✨
+🌿 Активна формула для зони навколо очей:
+💧 Інтенсивне зволоження та відновлення бар’єрної функції
+🌸 Освітлення темних кіл завдяки екстракту водоростей
+🛡️ Зменшення набряків завдяки рутину та ескуліну
+⚡ Комплекс інкапсульованих пептидів – стимуляція синтезу білків для пружності
+🌟 Живлення та захист завдяки олії авокадо та примули
+💚 Результат – зменшені набряки, світліший тон та пружна шкіра навколо очей!
+📌 Активні компоненти:
+🌱 Екстракт водоростей – покращує кровообіг та освітлює темні кола
+🌸 Рутин + ескулін – протинабрякова дія
+💧 Інулін – підвищує пружність та еластичність
+⚡ Інкапсульовані пептиди – стимулюють синтез кератину, філагрину та лорекину
+🥥 Олія авокадо та примули вечірньої – живлення та захист
+🌟 Токоферол + магнезіум аскорбіл фосфат – антиоксидантний щит
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Зволожувальний дренажний крем для очей
+Об’єм: 30 мл
+Призначення: Зволоження, протинабрякова дія, освітлення темних кіл
+Тип шкіри: Суха, чутлива, зріла
+Країна виробництва: 🇺🇦 Україна
+🌟 Drainage Moisturizing Eye Cream – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>508</t>
+  </si>
+  <si>
+    <t>Дренажна освітлююча маска Глабрідин для очей 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Glabridin Eye Mask – професійний догляд для сяючого погляду! ✨
+🌿 Інноваційна формула для переорбітальної зони:
+💧 Зволожує та підвищує еластичність шкіри
+🌸 Освітлює темні кола та зменшує набряки нижніх повік
+🛡️ Зміцнює судини та покращує мікроциркуляцію
+⚡ Активізує виведення заліза та білірубіну, зменшуючи тьмяність
+🌟 Відновлює бар’єрну функцію та захищає від стресових факторів
+💚 Результат – свіжий, відпочилий та сяючий погляд!
+📌 Активні компоненти:
+🌱 Shadownyl, Рутин, Ескулін – зміцнення судин та протинабрякова дія
+🌸 Inoveol EGCG, екстракт зеленого чаю та каштана – антиоксидантний захист та покращення кровообігу
+💧 PolyFructol Plus, Hydagen® Aquaporin, інулін – глибоке зволоження та підтримка водного балансу
+🛡️ X50® Skin Barrier та комплекс пептидів – стимуляція синтезу кератину та філагрину, відновлення бар’єру
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист
+✔️ Характеристики продукту:
+Тип: Дренажна освітлююча маска для очей
+Об’єм: 50 мл
+Призначення: Зволоження, освітлення, протинабрякова дія, відновлення
+Бренд: Smart4Derma (Україна + Німеччина)
+Країна виробництва: 🇺🇦 Україна / 🇩🇪 Німеччина
+🌟 Smart4Derma Glabridin Eye Mask – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>512</t>
   </si>
 </sst>
 </file>
@@ -8122,38 +8192,66 @@
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="12"/>
-      <c r="B75" s="8"/>
+      <c r="A75" s="12" t="s">
+        <v>880</v>
+      </c>
+      <c r="B75" s="8" t="s">
+        <v>878</v>
+      </c>
       <c r="C75" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D75" s="8"/>
+      <c r="D75" s="8">
+        <v>660</v>
+      </c>
       <c r="E75" s="8"/>
       <c r="F75" s="8"/>
-      <c r="G75" s="8"/>
-      <c r="H75" s="8"/>
+      <c r="G75" s="8">
+        <v>13</v>
+      </c>
+      <c r="H75" s="8" t="s">
+        <v>664</v>
+      </c>
       <c r="I75" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J75" s="8"/>
-      <c r="K75" s="18"/>
+      <c r="J75" s="8" t="s">
+        <v>879</v>
+      </c>
+      <c r="K75" s="18" t="s">
+        <v>880</v>
+      </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="12"/>
-      <c r="B76" s="8"/>
+      <c r="A76" s="12" t="s">
+        <v>883</v>
+      </c>
+      <c r="B76" s="8" t="s">
+        <v>881</v>
+      </c>
       <c r="C76" s="8" t="s">
         <v>653</v>
       </c>
-      <c r="D76" s="8"/>
+      <c r="D76" s="8">
+        <v>1000</v>
+      </c>
       <c r="E76" s="8"/>
       <c r="F76" s="8"/>
-      <c r="G76" s="8"/>
-      <c r="H76" s="8"/>
+      <c r="G76" s="8">
+        <v>14</v>
+      </c>
+      <c r="H76" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I76" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J76" s="8"/>
-      <c r="K76" s="18"/>
+      <c r="J76" s="8" t="s">
+        <v>882</v>
+      </c>
+      <c r="K76" s="18" t="s">
+        <v>883</v>
+      </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" s="12"/>

</xml_diff>

<commit_message>
feat: working AI consultant (Groq) + catalog serums fixes
- add Next.js route POST /api/chat: Groq (openai/gpt-oss-120b/20b,
  json_object) with server-side top-15 candidate retrieval to fit the
  8000 TPM key limit, strict catalog-only validation, follow-up
  questions, and a localized keyword fallback (always 3 products)
- pass GROQ_API_KEY from root .env into the frontend container;
  exclude .env* from the Docker build context
- show per-product reason (💡) in chat bubbles
- catalog: retry server fetch x3, proper "load error + retry" state
  instead of "nothing found" when the backend is down, sync
  q/category/sale from URL on navigation (fixes stale filter state)
- refresh price.xlsx + product images, update screenshots, document
  live implementation notes in AI_CONSULTANT_PROMPT.md
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98587DFA-14EC-468C-B9CD-64BE232C5C74}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16B6B9B-0AC8-4E74-847B-DDFC89E7B5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2041" uniqueCount="899">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2291" uniqueCount="1014">
   <si>
     <t>Артикул</t>
   </si>
@@ -5423,6 +5423,9 @@
     <t>512</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>Екстразволожувальна Антиоксидантна сиворотка з центеллою 50 мл</t>
   </si>
   <si>
@@ -5584,6 +5587,1180 @@
   </si>
   <si>
     <t>410</t>
+  </si>
+  <si>
+    <t>Порозвужувальна себорегулювальна маска «босвелія» 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Boswellia Clay Mask Herbal Pore Control – чиста та збалансована шкіра! ✨
+🌿 Активна формула для проблемної шкіри:
+💧 Зменшує пори та контролює себум
+🌸 Знижує запалення, подразнення та почервоніння
+🛡️ Нормалізує мікробіом шкіри та створює антисептичний бар’єр
+⚡ Має тонізуючу та регенеруючу дію
+🌟 Покращує стан проблемної шкіри та дарує відчуття свіжості
+💚 Результат – матова, рівна та здорова шкіра без надлишку себуму!
+📌 Показання до застосування:
+Акне 1–3 ступеня, постакне
+Розширені пори, нерівний тон
+Атопічний дерматит, екзема, псоріаз
+Подразнення та свербіж
+📌 Активні компоненти:
+🌱 Олії виноградних та персикових кісточок – живлення та відновлення
+🌸 Каолін – глибоке очищення та себорегуляція
+💧 Д-пантенол, гліцерин, ніацинамід – зволоження та регенерація
+🛡️ Екстракти епілобіуму, прополісу, каштану та календули – протизапальна дія
+⚡ Кофеїн, Bosexil, Bix'Activ – контроль себуму та тонізуючий ефект
+🌟 Бісаболол, алантоїн, ацетил тетрапептид-15 – заспокоюють та відновлюють
+✔️ Характеристики продукту:
+Тип: Себорегулююча порозвужуюча маска
+Об’єм: 50 мл
+Призначення: Очищення, себорегуляція, протизапальна дія
+Тип шкіри: Проблемна, жирна, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Boswellia Clay Mask – твій must-have для чистої та збалансованої шкіри без недоліків! 🌟</t>
+  </si>
+  <si>
+    <t>408-1</t>
+  </si>
+  <si>
+    <t>Нічний себорегулювальний флюїд «азеламід» 50 мл</t>
+  </si>
+  <si>
+    <t>✨ Azelamid Night Fluid – нічна терапія проти акне! ✨
+🌿 Лікувальна формула для проблемної шкіри:
+💧 Глибоко очищає пори та зменшує виділення себуму
+🌸 Усуває запалення та почервоніння
+🛡️ Відновлює баланс мікробіому та бар’єрні функції
+⚡ Заспокоює подразнення та прискорює регенерацію
+🌟 Дарує рівний тон та здоровий вигляд шкіри
+💚 Результат – чиста, матова та спокійна шкіра вже після кількох застосувань!
+📌 Активні компоненти:
+🌱 Bix'Activ та прополіс – пригнічують P.Acne, забезпечують антибактеріальний ефект
+🌸 Екстракт епілобіуму – регулює активність сальних залоз та мікробіом
+💧 Азелаїнова та саліцилова кислоти – відлущують та очищають пори
+🛡️ Босвелія – покращує мікроциркуляцію та зменшує почервоніння
+🌟 Ніацинамід та D-пантенол – заспокоюють та стимулюють відновлення
+🌸 Екстракти ромашки, шавлії та каштана – протизапальна та тонізуюча дія
+📌 Показання до застосування:
+Акне 1–3 ступеня
+Постакне та розширені пори
+Нерівний тон шкіри
+Атопічний дерматит, псоріаз, екзема
+Подразнення та свербіж
+✔️ Характеристики продукту:
+Тип: Нічний себорегулюючий флюїд
+Об’єм: 50 мл
+Призначення: Лікування акне, себорегуляція, протизапальна дія
+Тип шкіри: Проблемна, жирна, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Azelamid Night Fluid – твій must-have для нічного догляду та боротьби з акне! 🌟</t>
+  </si>
+  <si>
+    <t>409</t>
+  </si>
+  <si>
+    <t>Трансдермальний санблок ꜱᴘꜰ 𝟥𝟢, 50 мл</t>
+  </si>
+  <si>
+    <t>407</t>
+  </si>
+  <si>
+    <t>✨ Therapeutic Sunscreen SPF 30 – комплексний догляд та захист! ✨
+🌿 Формула спеціально для проблемної шкіри з акне та себореєю:
+☀️ SPF 30 широкого спектру – надійний захист від UVA/UVB
+💧 Зменшує пори та контролює себум
+🌸 Лікує акне 1–3 ступеня та постакне
+🛡️ Бореться з дерматитом, псоріазом та екземою
+⚡ Вирівнює тон та зменшує почервоніння
+💚 Результат – здорова, матова та захищена шкіра без недоліків!
+📌 Активні компоненти:
+🌱 Ніацинамід – відновлює мікробіом та регулює себум
+🌸 Екстракт епілобіуму флешері – протизапальна дія
+💧 Бета-глюкан – відновлює та заспокоює
+🛡️ Екстракт бікс орлеана – зменшує пори та жирність
+🌟 Бісаболол, Д-пантенол, пантеніл триацетат – знімають подразнення та почервоніння
+⚡ Екстракт босвелії – ефективний при дерматиті та екземі
+🌸 Додатково: екстракти шавлії, алое, ромашки, прополіс, олії льону та винограду, токоферол ацетат
+📌 Показання до застосування:
+Акне 1–3 ступеня, постакне
+Себорея та розширені пори
+Атопічний дерматит, псоріаз, екзема
+Подразнення та свербіж
+Нерівний тон шкіри
+✔️ Характеристики продукту:
+Тип: Лікувальний сонцезахисний крем
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Захист, лікування акне, себорегуляція, відновлення
+Тип шкіри: Проблемна, жирна, комбінована
+Країна виробництва: 🇺🇦 Україна
+🌟 Therapeutic Sunscreen SPF 30 – твій must-have для комплексного догляду та захисту проблемної шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Мінеральний себорегулювальний тонер 250 мл</t>
+  </si>
+  <si>
+    <t>403</t>
+  </si>
+  <si>
+    <t>✨ MINERAL BHA-TONER DE-BLEMISH SOLUTION – твій мінеральний секрет чистої та сяючої шкіри! ✨
+🌿 Активний тонік-ексфоліант із мультимінеральним комплексом:
+🔄 Стимулює оновлення клітин та контролює себум
+⚖️ Балансує мікрофлору шкіри
+💎 Прискорює регенерацію та відновлення тканин
+💧 Глибоко зволожує та дарує еластичність
+💚 Показання:
+🌟 Акне 1–3 ступеня
+🌟 Постакне та розширені пори
+🌟 Нерівний тон шкіри
+🌟 Атопічний дерматит, псоріаз, екзема
+🌟 Подразнення та свербіж
+🌸 Активні компоненти:
+🔥 Азелаїнова та саліцилова кислоти
+✨ Ніацинамід та глюконолактон
+🌼 Екстракти ромашки, шавлії, епілобіуму
+🍯 Прополіс та Bosexil
+🪨 Мінерали: магній, калій, цинк, натрій, кальцій
+💎 Результат – чиста, свіжа та збалансована шкіра без недоліків! 🌟</t>
+  </si>
+  <si>
+    <t>Iнтенсивний очищувальний гель з босвелією 250 мл</t>
+  </si>
+  <si>
+    <t>✨ Boswellia Pro-Gel Deep Cleanse – твій ритуал чистоти та комфорту! ✨
+🌿 Інтенсивний очищаючий гель з босвелією – універсальний засіб для проблемної шкіри. 💎 Поєднання кислот, прополісу та екстракту босвелії дарує глибоке очищення та відновлення.
+🔥 Основні дії:
+✨ Усунення жирного блиску та гіперкератозу
+⚖️ Регуляція вироблення себуму
+🌸 Заспокоює та знімає подразнення
+🛡️ Відновлює бар’єрні функції епідермісу
+💚 Корегує прояви себореї та екземи
+🌟 Показання:
+🌿 Акне 1–3 ступеня та постакне
+🔍 Розширені пори
+🎨 Нерівний тон обличчя
+🧴 Атопічний дерматит, псоріаз, екзема
+😌 Подразнення та свербіж
+💧 Активні компоненти:
+🌼 Екстракт ромашки, 🌱 екстракт шавлії, 💎 сечовина, 🌿 Д-пантенол, 🌟 Bosexil, 🍯 прополіс, ⚡ азелаїнова кислота, 🌊 саліцилова кислота, ✨ ніацинамід, 🌰 екстракт кінського каштана.
+💚 Boswellia Pro-Gel Deep Cleanse – твій секрет чистої та здорової шкіри!</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>✨ Нічний крем CutiBiome Extra Regeneration 50 мл ✨
+🌙 Інтенсивний догляд для жирної та комбінованої шкіри з проявами акне!
+💎 Ліпосомальна формула забезпечує глибоке проникнення активних компонентів, даруючи шкірі відновлення та баланс.
+🔹 Показання до застосування:
+🌿 Жирна та комбінована шкіра
+🌸 Корекція акне 1–2 ступеня
+🌟 Зменшення слідів постакне
+✨ Вирівнювання тону обличчя
+🔍 Зменшення розширених пор
+💧 Заспокоєння запальних процесів
+💚 Основні переваги:
+⚖️ Нормалізація мікробіому шкіри
+🌿 Себорегуляція
+🌸 Зменшення слідів постакне
+🛡️ Антибактеріальна та протизапальна дія
+💦 Інтенсивне зволоження
+🌞 Матуючий ефект
+🌟 Активні компоненти:
+Олія виноградних та персикових кісточок, Д-пантенол, гліцерин, ніацинамід, Sebaryl FL LS 9088, екстракти лайма, зеленого чаю та чайного дерева, лактобіонова кислота, CutiBiome CLR™, Skinasensyl, алантоїн.
+📦 Об’єм: 50 мл
+🏢 Виробник: Smart4Derma</t>
+  </si>
+  <si>
+    <t>Нічний крем Кутибіом Extra Regeneration 50 мл для жирної шкіри</t>
+  </si>
+  <si>
+    <t>308</t>
+  </si>
+  <si>
+    <t>✨ Smart Derma Total Protect BB Cream SPF 30 – матовість та захист! ✨
+🌿 Багатофункціональна формула для жирної та комбінованої шкіри:
+☀️ SPF 30 UVA/UVB-захист – профілактика фотопошкоджень
+💧 Матуючий ефект без жирного блиску
+🌸 Вирівнює тон та зменшує сліди постакне
+🛡️ CutiBiome CLR – нормалізація мікробіому та протизапальна дія
+⚡ Довготривала гідратація та себорегуляція
+💚 Результат – рівний тон, матова та здорова шкіра щодня!
+📌 Активні компоненти:
+🌱 Олія виноградних та персикових кісточок – живлення та відновлення
+🌸 Екстракти зеленого чаю, лайма та чайного дерева – антибактеріальна дія
+💧 Ніацинамід та Д-пантенол – зволоження та регенерація
+🛡️ Лактобіонова кислота – м’яке відлущення та вирівнювання тону
+🌟 Алантоїн – заспокоює та знімає подразнення
+📌 Показання до застосування:
+Жирна та комбінована шкіра
+Акне 1–2 ступеня та постакне
+Нерівний тон обличчя
+Розширені пори
+Запальні процеси
+✔️ Характеристики продукту:
+Тип: Матуючий BB крем з SPF
+Об’єм: 50 мл
+Рівень захисту: SPF 30
+Призначення: Матування, тонування, захист, себорегуляція
+Тип шкіри: Жирна, комбінована, проблемна
+Бренд: Smart Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart Derma Total Protect BB Cream SPF 30 – твій must-have для матової та доглянутої шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>Матуючий ВВ крем SPF 30 Smart Derma Total Protect</t>
+  </si>
+  <si>
+    <t>310</t>
+  </si>
+  <si>
+    <t>✨ Sebo-Mask Manuka – контроль себуму та чиста шкіра! ✨
+🌿 Спеціалізована формула для жирної та комбінованої шкіри:
+💧 Нормалізує роботу сальних залоз та зменшує секрецію себуму
+🌸 Пригнічує розмноження бактерій Propionibacterium acnes
+🛡️ Заспокоює запальні процеси та зменшує почервоніння
+⚡ Вирівнює тон та зменшує сліди постакне
+🌟 Дарує матовість без жирного блиску
+💚 Результат – чиста, матова та здорова шкіра без недоліків!
+📌 Основні переваги:
+Нормалізація мікробіому шкіри
+Себорегуляція та матуючий ефект
+Зменшення слідів постакне
+Антибактеріальна та протизапальна дія
+Зволоження без жирного блиску
+Звуження пор
+📌 Активні компоненти:
+🌱 Олія персика та кокоса – живлення та відновлення
+🌸 Екстракти зеленого чаю, календули та кропиви – антиоксидантна та заспокійлива дія
+💧 Ніацинамід – контроль себуму та вирівнювання тону
+🛡️ Sebaryl – регуляція роботи сальних залоз
+⚡ Гідролат лайма – тонізуючий ефект
+🌟 Екстракт чайного дерева – антибактеріальна дія
+✔️ Характеристики продукту:
+Тип: Себорегулююча маска для жирної шкіри
+Об’єм: 50 мл
+Призначення: Контроль себуму, лікування акне, матування
+Тип шкіри: Жирна, комбінована, проблемна
+Країна виробництва: 🇺🇦 Україна
+🌟 Sebo-Mask Manuka – твій must-have для догляду за жирною та проблемною шкірою! 🌟</t>
+  </si>
+  <si>
+    <t>Манукі маска для жирної шкіри та акне Sebo-Mask 50 мл</t>
+  </si>
+  <si>
+    <t>306-1</t>
+  </si>
+  <si>
+    <t>Ліпосомальна сироватка з феруловою кислотою BHA-PHA Control 50 мл</t>
+  </si>
+  <si>
+    <t>✨ BHA-PHA Control Serum – інтенсивна терапія для проблемної шкіри! ✨
+🌿 Спеціалізована формула для жирної та комбінованої шкіри:
+💧 Нормалізує мікробіом та пригнічує ріст бактерій P. Acnes
+🌸 Зменшує сліди постакне та вирівнює тон
+🛡️ Забезпечує себорегуляцію та матуючий ефект
+⚡ Має антибактеріальну та протизапальну дію
+🌟 Дарує зволоження без жирного блиску
+💚 Результат – чиста, матова та здорова шкіра з рівним тоном!
+📌 Основні активні компоненти:
+🌱 Азелаїнова кислота – потужна антибактеріальна дія
+🌸 Ферулова кислота – антиоксидантний захист
+💧 Ніацинамід – себорегуляція та зволоження
+🛡️ Лактобіонова кислота – делікатне відлущування
+🌟 Екстракти алоє, ромашки, чайного дерева та зеленого чаю – заспокоюють та знімають запалення
+📌 Показання до застосування:
+Жирна та комбінована шкіра
+Акне 1–2 ступеня
+Постакне та розширені пори
+Нерівний тон обличчя
+Запальні процеси
+✔️ Характеристики продукту:
+Тип: Ліпосомальна сироватка для проблемної шкіри
+Об’єм: 50 мл
+Призначення: Лікування акне, себорегуляція, антиоксидантний захист
+Тип шкіри: Жирна, комбінована, проблемна
+Країна виробництва: 🇺🇦 Україна
+🌟 BHA-PHA Control Serum – твій must-have для догляду за проблемною шкірою та контролю акне! 🌟</t>
+  </si>
+  <si>
+    <t>312</t>
+  </si>
+  <si>
+    <t>Манукі маска для жирної шкіри та акне Sebo-Mask 230 мл</t>
+  </si>
+  <si>
+    <t>230 мл</t>
+  </si>
+  <si>
+    <t>✨ Sebo-Mask Manuka – контроль себуму та чиста шкіра! ✨
+🌿 Спеціалізована формула для жирної та комбінованої шкіри:
+💧 Нормалізує роботу сальних залоз та зменшує секрецію себуму
+🌸 Пригнічує розмноження бактерій Propionibacterium acnes
+🛡️ Заспокоює запальні процеси та зменшує почервоніння
+⚡ Вирівнює тон та зменшує сліди постакне
+🌟 Дарує матовість без жирного блиску
+💚 Результат – чиста, матова та здорова шкіра без недоліків!
+📌 Основні переваги:
+Нормалізація мікробіому шкіри
+Себорегуляція та матуючий ефект
+Зменшення слідів постакне
+Антибактеріальна та протизапальна дія
+Зволоження без жирного блиску
+Звуження пор
+📌 Активні компоненти:
+🌱 Олія персика та кокоса – живлення та відновлення
+🌸 Екстракти зеленого чаю, календули та кропиви – антиоксидантна та заспокійлива дія
+💧 Ніацинамід – контроль себуму та вирівнювання тону
+🛡️ Sebaryl – регуляція роботи сальних залоз
+⚡ Гідролат лайма – тонізуючий ефект
+🌟 Екстракт чайного дерева – антибактеріальна дія
+✔️ Характеристики продукту:
+Тип: Себорегулююча маска для жирної шкіри
+Об’єм: 230 мл
+Призначення: Контроль себуму, лікування акне, матування
+Тип шкіри: Жирна, комбінована, проблемна
+Країна виробництва: 🇺🇦 Україна
+🌟 Sebo-Mask Manuka – твій must-have для догляду за жирною та проблемною шкірою! 🌟</t>
+  </si>
+  <si>
+    <t>306</t>
+  </si>
+  <si>
+    <t>Ензимна пудра Smart4Derma з вулканічним пилом для жирної шкіри 120 г</t>
+  </si>
+  <si>
+    <t>120 г</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Enzyme Powder – глибоке очищення та контроль себуму! ✨
+🌿 Професійна формула для жирної та комбінованої шкіри:
+💧 Ефективно розчиняє сальні пробки та очищає пори
+🌸 Зменшує їх розмір та нормалізує себорегуляцію
+🛡️ Має антибактеріальну та протизапальну дію
+⚡ Дарує матуючий ефект без пересушування
+🌟 Стимулює регенерацію та вирівнює тон шкіри
+💚 Результат – чиста, матова та здорова шкіра з рівним тоном!
+📌 Активні компоненти:
+🌱 Ніацинамід – контроль роботи сальних залоз
+🌸 Комплекс кислот (лактобіонова, винна) – делікатне відлущування
+💧 Папаїн – ензимне очищення
+🛡️ Вулканічний пил – регуляція себуму та глибоке очищення
+⚡ Цинк глюканат – протизапальна дія
+🌟 Кофеїн – тонізує та активізує мікроциркуляцію
+📌 Показання до застосування:
+Жирна та комбінована шкіра
+Акне 1–2 ступеня
+Постакне та нерівний тон
+Розширені пори
+Запальні процеси
+✔️ Характеристики продукту:
+Тип: Ензимна пудра для очищення
+Об’єм: 120 г
+Лінійка: Acne Balance
+Призначення: Глибоке очищення, себорегуляція, матування
+Тип шкіри: Жирна, комбінована, проблемна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma Enzyme Powder – твій must-have для глибокого очищення та сяючої шкіри без недоліків! 🌟</t>
+  </si>
+  <si>
+    <t>301</t>
+  </si>
+  <si>
+    <t>Себорегулюючий мультикислотний тонер CUTIBIOME TONER BHA-PHA CONTROL</t>
+  </si>
+  <si>
+    <t>✨ CUTIBIOME TONER – контроль себуму та рівний тон! ✨
+🌿 Інтенсивна терапія для проблемної шкіри:
+💧 Зволожує та нормалізує рН
+🌸 Вирівнює тон та зменшує сліди постакне
+🛡️ Має виражену антибактеріальну та протизапальну дію
+⚡ Нормалізує мікробіом та регулює роботу сальних залоз
+🌟 Дарує матуючий ефект без пересушування
+💚 Результат – чиста, матова та здорова шкіра з рівним тоном!
+📌 Показання до застосування:
+Жирна та комбінована шкіра
+Акне 1–2 ступеня
+Постакне та розширені пори
+Нерівний тон обличчя
+Запальні процеси
+📌 Активні компоненти:
+🌱 Кислотний комплекс BHA + PHA (саліцилова та лактобіонова кислоти) – очищення та делікатне відлущування
+🌸 Азелаїнова кислота – протизапальна та антибактеріальна дія
+💧 Ніацинамід та цинк глюканат – себорегуляція та зволоження
+🛡️ Екстракти алоє та ромашки – заспокоюють та знімають подразнення
+⚡ Кофеїн – тонізує та активізує мікроциркуляцію
+🌟 Ефірні олії чайного дерева та лайма, CutiBiome CLR – нормалізація мікробіому та антисептичний ефект
+✔️ Характеристики продукту:
+Тип: Себорегулюючий мультикислотний тонер
+Об’єм: 100 мл
+Призначення: Зволоження, себорегуляція, антибактеріальна дія
+Тип шкіри: Жирна, комбінована, проблемна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 CUTIBIOME TONER – твій must-have для догляду за проблемною шкірою та контролю акне!</t>
+  </si>
+  <si>
+    <t>304</t>
+  </si>
+  <si>
+    <t>Очищающая мультикислотная пенка для жирной, комбинированной и кожи из акне 80 мл</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma AHA-BHA-PHA Foam – глибоке очищення та контроль акне! ✨
+🌿 Спеціальна формула для жирної та проблемної шкіри:
+💧 Делікатно, але ефективно видаляє забруднення, себум та залишки макіяжу
+🌸 Регулює вироблення себуму та зменшує пори
+🛡️ Має антибактеріальну та заспокійливу дію
+⚡ Підтримує мікробіом шкіри завдяки PHA-кислотам
+🌟 Робить шкіру гладкою, матовою та свіжою
+💚 Результат – чиста, матова та здорова шкіра без недоліків!
+📌 Основні властивості:
+Регуляція себуму та зменшення пор (ніацинамід, азелаїнова та гліколева кислоти)
+Антибактеріальна та заспокійлива дія (олії чайного дерева та лайма)
+Підтримка мікробіому (PHA-кислоти)
+📌 Активні компоненти:
+🌱 AHA, BHA, PHA кислоти (гліколева, молочна, винна, яблучна, лактобіонова, саліцилова)
+🌸 Азелаїнова кислота – протизапальна дія
+💧 Ніацинамід – себорегуляція та зволоження
+🛡️ Олії лайма та чайного дерева – антисептичний ефект
+⚡ Кофеїн та цинк – тонізуюча та протизапальна дія
+📌 Застосування:  
+Нанести на вологу шкіру, помасажувати 1–2 хвилини та змити. Використовувати двічі на день.
+✔️ Характеристики продукту:
+Тип: Очищувальна пінка для обличчя
+Призначення: Очищення, себорегуляція, антибактеріальна дія
+Тип шкіри: Жирна, комбінована, проблемна
+Лінійка: Acne Balance
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma AHA-BHA-PHA Foam – твій must-have для щоденного контролю акне та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Маска-гоммаж Smart4Derma з молочними протеїнами та ферментами 100 мл</t>
+  </si>
+  <si>
+    <t>240-1</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Enzyme Gommage – м’яке відлущування та сяйво! ✨
+🌿 Унікальна формула для делікатного догляду:
+💧 Дбайливо видаляє відмерлі клітини та сальні пробки
+🌸 Вирівнює текстуру та дарує гладкість
+🛡️ Зберігає гідроліпідний баланс шкіри
+⚡ Стимулює регенерацію та оновлення клітин
+🌟 Робить шкіру сяючою та свіжою після кожного застосування
+💚 Результат – м’яка, рівна та сяюча шкіра без подразнень!
+📌 Активні інгредієнти:
+🌱 Молочні протеїни та ферменти (актинідин, бромелайн, трипсин, хримотрипсин, фіцин, сутілайн) – ензимне очищення та ексфоліація
+🌸 Екстракти розмарину, ламінарії, кори верби, обліпихи та горобини – антиоксидантна та протизапальна дія
+💧 Олії пінника лугового, солодкого мигдалю та грецького горіха – живлення та відновлення
+🛡️ Prozymex® та X-pressin – стимуляція регенерації та оновлення клітин
+📌 Спосіб застосування:  
+Нанести на чисту вологу шкіру, легкими масажними рухами скочувати засіб, видаляючи відмерлі клітини. Змити водою.
+✔️ Характеристики продукту:
+Тип: Очищувальна маска-гоммаж
+Об’єм: 100 мл
+Призначення: Ексфоліація, очищення, сяйво
+Тип шкіри: Усі типи, особливо тьмяна та проблемна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma Enzyme Gommage – твій must-have для м’якого відлущування та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Освітлювальний пілінг для делікатних зон Smart4Derma Intimate Harmony Peel 30 мл</t>
+  </si>
+  <si>
+    <t>✨ Intimate Harmony Peel – ніжне освітлення та догляд! ✨
+🌿 Спеціально створений для делікатних зон:
+💧 Освітлює та вирівнює тон шкіри
+🌸 Зменшує пігментацію та нерівності текстури
+🛡️ Уповільнює ріст волосся та запобігає його вростанню
+⚡ Підтримує пружність та еластичність
+🌟 Дарує гладку, світлу та доглянуту шкіру навіть у найчутливіших ділянках
+💚 Результат – бездоганна шкіра без дискомфорту!
+📌 Активні інгредієнти та їх дія:
+🌱 Мигдальна кислота (20%) – м’яке відлущування та освітлення
+🌸 Транексамова кислота (15%) – боротьба з пігментними плямами
+💧 Молочна кислота (10%) – зволоження та вирівнювання текстури
+🛡️ Лактобіонова кислота (7%) – антиоксидантна та омолоджуюча дія
+⚡ Лимонна кислота та папаїн – посилюють освітлення та очищають пори
+🌟 Саліцилова кислота – запобігає вростанню волосся
+📌 Спосіб використання:  
+Нанести 1–2 мл засобу на чисту, суху шкіру делікатних зон (пахви, зона бікіні, внутрішня поверхня стегон, ареоли), уникаючи слизових оболонок.
+Залишити на 5–10 хвилин, після чого ретельно змити теплою водою.
+Рекомендований курс: 6–8 процедур з інтервалом 7–10 днів.
+✔️ Характеристики продукту:
+Тип: Освітлювальний пілінг для делікатних зон
+Об’єм: 50 мл
+Призначення: Освітлення, вирівнювання тону, профілактика вростання волосся
+Тип шкіри: Усі типи, особливо чутлива та схильна до пігментації
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Intimate Harmony Peel – твій must-have для ніжного догляду та рівного тону шкіри у делікатних зонах! 🌟</t>
+  </si>
+  <si>
+    <t>681</t>
+  </si>
+  <si>
+    <t>681(1)</t>
+  </si>
+  <si>
+    <t>Антиоксидантний ультразахисний крем SPF 80 для жирної шкіри Smart4Derma QC Sunblock Oil-Free 230 мл</t>
+  </si>
+  <si>
+    <t>✨ QC Sunblock Oil-Free SPF 80 – ультра-захист та молодість шкіри! ✨
+🌿 Формула для щоденного використання:
+☀️ SPF 80 широкого спектра UVA/UVB – максимальний захист від сонячних променів
+🌸 Коензим Q10 та вітамін С – потужний антиоксидантний комплекс проти вільних радикалів
+🛡️ Запобігає появі зморшок та пігментних плям
+💧 Некомедогенна формула – зволожує без жирного блиску
+⚡ Створює рівномірне та гладке покриття
+💚 Результат – захищена, свіжа та доглянута шкіра щодня!
+📌 Переваги:
+Максимальний сонцезахисний ефект
+Антиоксидантний захист
+Некомедогенна формула
+Зволоження та протизапальна дія
+📌 Активні компоненти:
+🌱 Емоленти – живлення та м’якість
+🌸 Бісаболол – заспокоює та знімає подразнення
+💧 Вітамін С – антиоксидантний захист
+🛡️ Коензим Q10 – уповільнює старіння
+☀️ Сонцезахисні фільтри – UVA/UVB-захист
+📌 Спосіб використання:  
+Нанести тонким рівномірним шаром на очищену шкіру обличчя за 15–20 хвилин до виходу на сонце.
+Для тривалого перебування на сонці – оновлювати кожні 2–3 години.
+✔️ Характеристики продукту:
+Тип: Сонцезахисний крем
+Об’єм: 50 мл / 100 мл (залежно від упаковки)
+Рівень захисту: SPF 80
+Призначення: Захист, антиоксидантний догляд, профілактика старіння
+Тип шкіри: Усі типи, особливо схильна до фотостаріння
+Бренд: QC
+Країна виробництва: 🇺🇦 Україна
+🌟 QC Sunblock Oil-Free SPF 80 – твій must-have для щоденного ультра-захисту та молодості шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>849(1)</t>
+  </si>
+  <si>
+    <t>849</t>
+  </si>
+  <si>
+    <t>Денний крем SPF 35 проти пігментації для всіх типів шкіри Smart4Derma Marguerite Cream Power Defence SPF 35 - 230 мл</t>
+  </si>
+  <si>
+    <t>841</t>
+  </si>
+  <si>
+    <t>841(1)</t>
+  </si>
+  <si>
+    <t>✨ Marguerite Cream Power Defence SPF 35 – освітлення та захист! ✨
+🌿 Універсальна формула для всіх типів шкіри:
+☀️ SPF 35 – надійний захист від UVA/UVB
+🌸 Освітлює та вирівнює тон, зменшує пігментацію
+🛡️ Знижує продукування меланіну та запобігає появі нових плям
+⚡ Коригує вже наявні дефекти шкіри
+🌟 Заспокоює подразнення та зменшує запальні реакції
+💚 Результат – рівний, світлий та здоровий тон шкіри щодня!
+📌 Переваги:
+Висококонцентрована формула
+Сонцезахисний ефект
+Вирівнювання тону та зменшення гіперпігментації
+Антиоксидантна дія
+Зволоження та живлення
+📌 Активні компоненти:
+🌱 Амарантова олія, арбутин, бісаболол
+🌸 Вітамін C, глутатіон, токоферол
+💧 Екстракти маргаритки, солодки, ячменю, гадючника в’язолистого, кресу
+🛡️ Ізофлавони сої, лецитин, ліноленова кислота
+⚡ Олії бабассу, бораго, виноградної кісточки
+🌟 Пептиди та освітлюючий комплекс
+☀️ Сонцезахисні фільтри
+📌 Спосіб використання:  
+Щоранку нанести невелику кількість крему на очищену шкіру обличчя та шиї.
+Рівномірно розподілити легкими рухами до повного вбирання.
+Для максимального ефекту – використовувати щоденно.
+✔️ Характеристики продукту:
+Тип: Освітлювальний сонцезахисний крем
+Об’єм: 50 мл
+Рівень захисту: SPF 35
+Призначення: Освітлення, захист, антиоксидантний догляд
+Тип шкіри: Усі типи, включно з чутливою
+Бренд: Marguerite
+Країна виробництва: 🇺🇦 Україна
+🌟 Marguerite Cream Power Defence SPF 35 – твій must-have для рівного тону та захисту шкіри від сонця! 🌟</t>
+  </si>
+  <si>
+    <t>Освітлюючий крем SPF 15 «Сяючий погляд» Smart4Derma Eye Cream B-White Contour SPF 15 - 100 мл</t>
+  </si>
+  <si>
+    <t>844</t>
+  </si>
+  <si>
+    <t>844(1)</t>
+  </si>
+  <si>
+    <t>✨ B-White Eye Cream SPF 15 – сяйво та молодість погляду! ✨
+🌿 Формула для ніжної шкіри навколо очей:
+💧 Освітлює темні кола та зменшує набряки
+🌸 Вирівнює тон та усуває пігментацію
+🛡️ Захищає від фотостаріння та оксидативного стресу
+⚡ Заспокоює подразнення та знижує запальні процеси
+🌟 Підтримує пружність та еластичність шкіри
+💚 Результат – сяючий, свіжий та молодий погляд щодня!
+📌 Переваги:
+Зволоження та живлення
+Поліпшення мікроциркуляції
+Антиоксидантний захист
+Освітлення та вирівнювання тону
+Захист від UVA/UVB (SPF 15)
+📌 Активні компоненти:
+🌱 Shadownyl – антивіковий комплекс для зменшення темних кіл
+🌸 EGCG детокс-комплекс – антиоксидантна дія
+💧 β‑White пептид та арбутин – освітлення та контроль меланіну
+🛡️ Вітамін С та Brightenyl – боротьба з пігментацією
+⚡ Гіалуронова кислота, Aquaporin комплекс – інтенсивне зволоження
+🌟 Ескулін, есцин, рутина, пептиди Rubixyl – покращення мікроциркуляції та тонусу
+🌸 Олії авокадо та пасіфлори – живлення та відновлення
+📌 Спосіб використання:  
+Наносити щодня вранці та ввечері на очищену шкіру навколо очей легкими рухами по масажних лініях до повного поглинання.
+Підходить для всіх типів шкіри, особливо схильної до пігментації та втрати тонусу.
+✔️ Характеристики продукту:
+Тип: Освітлювальний антивіковий крем для очей
+Об’єм: 30 мл
+Рівень захисту: SPF 15
+Призначення: Освітлення, антиоксидантний захист, зволоження
+Тип шкіри: Усі типи, особливо делікатна та схильна до пігментації
+Бренд: B-White
+Країна виробництва: 🇺🇦 Україна
+🌟 Eye Cream B-White Contour SPF 15 – твій must-have для сяючого та молодого погляду без темних кіл! 🌟</t>
+  </si>
+  <si>
+    <t>Оптично-відбілююча реепітелізуюча маска Smart4Derma Opti-White Mask DGA Re-Epithelium 300 мл</t>
+  </si>
+  <si>
+    <t>300 мл</t>
+  </si>
+  <si>
+    <t>847</t>
+  </si>
+  <si>
+    <t>847(1)</t>
+  </si>
+  <si>
+    <t>✨ Opti-White Mask – сяйво та рівний тон! ✨
+🌿 Висококонцентрована формула для боротьби з пігментацією:
+💧 Зменшує вираженість постакне, вікових та пігментних плям
+🌸 Усуває тьмяність та неоднорідний тон
+🛡️ Нейтралізує вільні радикали та захищає від оксидативного стресу
+⚡ Інтенсивно зволожує, усуває сухість та стягнутість
+🌟 Відновлює пружність, еластичність та природне сяйво
+💚 Результат – гладка, свіжа та сяюча шкіра без недоліків!
+📌 Властивості:
+Освітлення та вирівнювання тону
+Висококонцентрований склад
+Антиоксидантний захист
+Поліпшення тургору та пружності
+Інтенсивне зволоження
+📌 Активні компоненти:
+🌱 Вітамін С (3 стабільні форми) – освітлення та антиоксидантна дія
+🌸 Нанопептид-1 – повертає сяйво та вдосконалює мікрорельєф
+💧 Гіалуронова кислота – глибоке зволоження
+🛡️ Бісаболол – заспокоює та знімає подразнення
+🌟 Лецитин та пептиди – відновлення та зміцнення шкіри
+📌 Спосіб використання:  
+Нанести маску на чисту шкіру обличчя, рівномірно розподілити та залишити для дії. Використовувати регулярно для максимального ефекту освітлення та відновлення.
+✔️ Характеристики продукту:
+Тип: Освітлювальна концентрована маска
+Призначення: Освітлення, зволоження, антиоксидантний захист
+Тип шкіри: Нормальна, суха, комбінована, чутлива
+Вік: 25+, 30+, 40+, 50+
+Країна виробництва: 🇺🇦 Україна
+🌟 Opti-White Mask – твій must-have для сяючої та доглянутої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Интеллектуальный осветляющий Бустер-Концентрат тройного действия Smart Booster 3D Whitening Smart4Derma 10 ml</t>
+  </si>
+  <si>
+    <t>10 ml</t>
+  </si>
+  <si>
+    <t>843</t>
+  </si>
+  <si>
+    <t>843(1)</t>
+  </si>
+  <si>
+    <t>✨ Brightenyl Concentrate – рівний тон та сяйво шкіри! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Коригує меланогенез за трьома напрямками:
+• зменшує утворення ендотеліну-1 (ЕТ-1)
+• скорочує біосинтез меланіну, індукований УФ-випромінюванням
+• регулює активність тирозинази та α-MSH
+🌸 Освітлює пігментні плями різного генезу
+🛡️ Запобігає фотостарінню та оксидативному стресу клітин
+⚡ Вирівнює тон та текстуру шкіри
+🌟 Дарує сяйво та здоровий вигляд
+💚 Результат – світла, рівна та доглянута шкіра без пігментації!
+📌 Показання:
+Пігментні плями різного походження (сонячні, вікові, постакне, післязапальні)
+Нерівний тон та тьмяність
+Профілактика фотостаріння
+Лікування будь-якої гіперхромії
+📌 Активні інгредієнти:
+🌱 Екстракт маргаритки та кресу садового – освітлення та регуляція меланогенезу
+🌸 Гіалуронова кислота – глибоке зволоження
+💧 Лецитин та ізофлавони сої – відновлення та антиоксидантний захист
+🛡️ Аміноетилфосфінова кислота – контроль пігментації
+⚡ Екстракт софори японської та бурої водорості – протизапальна дія
+🌟 BRIGHTENYL®, арбутин, глутатіон, аскорбіл пальмітат – потужний освітлюючий комплекс
+✨ Нанопептид-1 – відновлення сяйва та пружності
+📌 Спосіб застосування:  
+Нанести невелику кількість препарату на очищену шкіру обличчя, шиї та декольте.
+Масажувати круговими рухами до повного поглинання.
+Рекомендується щоденне використання.
+✔️ Характеристики продукту:
+Тип: Освітлюючий концентрат для корекції пігментації
+Об’єм: 30 мл
+Призначення: Освітлення, профілактика фотостаріння, антиоксидантний захист
+Тип шкіри: Усі типи, особливо схильна до пігментації
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Brightenyl Concentrate – твій must-have для рівного тону та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Освітлювальний молекулярний тонік з ніацинамідом та глутатіоном Smart4Derma N-glutation Tonic Molecular Glow 500 мл</t>
+  </si>
+  <si>
+    <t>500 мл</t>
+  </si>
+  <si>
+    <t>855</t>
+  </si>
+  <si>
+    <t>855(1)</t>
+  </si>
+  <si>
+    <t>✨ Illuminating Toner – рівний тон та сяйво! ✨
+🌿 Формула для щоденного догляду:
+💧 Освітлює сліди постакне та рубці
+🌸 Зміцнює захисний бар’єр та протидіє вільним радикалам
+🛡️ Запобігає появі пігментних плям
+⚡ Гідратує та робить шкіру м’якою й гладкою
+🌟 Вирівнює колір та текстуру шкіри
+💚 Результат – здорова, сяюча та доглянута шкіра без недоліків!
+📌 Переваги:
+Вирівнювання тону
+Усунення пігментації
+Покращення тургору
+Зміцнення захисної функції
+📌 Активні компоненти:
+🌱 Арбутин – освітлення та профілактика пігментації
+🌸 Вітамін C та глутатіон – антиоксидантний захист
+💧 Диглюкозид галової кислоти – відновлення та зміцнення
+🌼 Екстракти маргаритки та толокнянки – природне освітлення
+🌿 Олія Шуінко – живлення та захист
+⚡ Папаїн – м’яке відлущування та оновлення
+📌 Спосіб використання:  
+Нанести тонік на очищену шкіру обличчя вранці та ввечері за допомогою ватного диска.
+М’яко масажувати круговими рухами для кращого проникнення активних компонентів.
+✔️ Характеристики продукту:
+Тип: Освітлювальний тонік
+Об’єм: 150 мл
+Призначення: Освітлення, вирівнювання тону, антиоксидантний захист
+Тип шкіри: Нормальна, комбінована, проблемна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Illuminating Toner – твій must-have для сяючої та доглянутої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Освітлювальна ензимна пудра Smart4Derma Glow Enzyme Powder 10% Vitamin C &amp; Q10 120 грам</t>
+  </si>
+  <si>
+    <t>120 грам</t>
+  </si>
+  <si>
+    <t>852</t>
+  </si>
+  <si>
+    <t>852(1)</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Enzyme Powder – сяйво та рівний тон! ✨
+🌿 Формула для боротьби з пігментацією та тьмяністю:
+💧 Видаляє ороговілі клітини та сальні пробки
+🌸 Освітлює пігментні плями та сліди постакне
+🛡️ Зміцнює захисний бар’єр та протидіє вільним радикалам
+⚡ Вирівнює тон та текстуру шкіри
+🌟 Дарує свіжість, гладкість та сяйво
+💚 Результат – чиста, світла та доглянута шкіра без недоліків!
+📌 Переваги продукту:
+Ефективне видалення ороговілих клітин
+Освітлення пігментації та постакне
+Звуження пор та вирівнювання тону
+Підтримка шкіри в ідеальному стані
+📌 Активні компоненти:
+🌱 Арбутин та койєва кислота – освітлення та профілактика пігментації
+🌸 Вітамін С та коензим Q10 – антиоксидантний захист
+💧 Алантоїн та фолієва кислота – зволоження та відновлення
+🛡️ Бромелайн, папаїн, протеаза – ензимне очищення та ексфоліація
+⚡ Аргінін та винна кислота – регенерація та вирівнювання текстури
+📌 Спосіб використання:  
+Змішати невелику кількість пудри з водою до утворення піни.
+Нанести на вологу шкіру, м’яко масажувати та змити водою.
+Рекомендується використовувати 2–3 рази на тиждень.
+✔️ Характеристики продукту:
+Тип: Освітлювальна ензимна пудра
+Об’єм: 100 г
+Призначення: Освітлення, ексфоліація, антиоксидантний захист
+Тип шкіри: Усі типи, особливо схильна до пігментації та постакне
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma Enzyme Powder – твій must-have для сяючої та рівної шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>480 мл</t>
+  </si>
+  <si>
+    <t>Освітлювальна пінка з вітаміном C та глутатіоном Smart4Derma C-glutation Mousse Glow Cleanser 480 мл</t>
+  </si>
+  <si>
+    <t>853(1)</t>
+  </si>
+  <si>
+    <t>853</t>
+  </si>
+  <si>
+    <t>✨ Сила вітаміну С та глутатіону – сяюча шкіра щодня! ✨
+🌿 Інноваційна формула для комплексного догляду:
+💧 Дбайливо видаляє макіяж, забруднення та надлишки себуму
+🌸 Освітлює пігментні плями та сліди постакне
+🛡️ Забезпечує потужний антиоксидантний захист
+⚡ Інтенсивно гідратує та зберігає еластичність
+🌟 Звужує пори, вирівнює мікрорельєф та запобігає висипанням
+💚 Результат – чиста, сяюча та доглянута шкіра без подразнень!
+📌 Переваги:
+Ефективне очищення
+Освітлення пігментних плям
+Гідратування та захист
+Себорегуляція
+📌 Активні компоненти:
+🌱 Арбутин – освітлення та профілактика пігментації
+☀️ Вітамін C – антиоксидантний захист та вирівнювання тону
+💎 Глутатіон – потужний антиоксидант, зволоження та еластичність
+🌸 Диглюкозид галової кислоти – регенерація та зміцнення
+💧 Пантенол – інтенсивне зволоження та заспокоєння
+📌 Спосіб використання:  
+Нанести невелику кількість пінки на вологу шкіру, легко помасажувати та змити теплою водою.
+Використовувати регулярно для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Освітлювальна пінка для вмивання
+Призначення: Очищення, освітлення, антиоксидантний захист
+Тип шкіри: Нормальна, жирна, комбінована, проблемна
+Вік: 20+, 30+, 40+, 50+
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma C-Glutation Mousse – твій must-have для сяючої та рівної шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>Зміцнювальний Нічний крем для чутливої шкіри та куперозом 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Therapeutic Night Cream – нічний догляд для міцних капілярів! ✨
+🌿 Формула для чутливої та куперозної шкіри:
+💧 Зміцнює судини та капіляри
+🌸 Підтримує стабільну циркуляцію крові
+🛡️ Освітлює пігментацію та знімає подразнення
+⚡ Зменшує набряки та реактивність шкіри
+🌟 Відновлює ліпідний баланс та дарує комфорт
+💚 Результат – спокійна, рівна та доглянута шкіра щоранку!
+📌 Активні компоненти:
+🌺 Екстракт магнолії – протизапальна дія, зменшення подразнень
+🌱 Поліпептидний комплекс – активізує обмін речовин та зміцнює тканини
+💧 Гіалуронова кислота – глибоке зволоження та еластичність
+🥑 Олія авокадо та жожоба – живлення та відновлення бар’єру
+📌 Показання до застосування:
+Купероз та розацеа
+Судинна сітка та почервоніння
+Реактивна та суха шкіра
+Порушення мікроциркуляції
+📌 Спосіб використання:  
+Нанести крем на очищену шкіру обличчя перед сном. Рівномірно розподілити по всій поверхні для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Нічний крем для чутливої шкіри
+Об’єм: 230 мл
+Призначення: Зміцнення судин, зволоження, освітлення пігментації, зняття подразнень
+Тип шкіри: Чутлива, суха, куперозна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Therapeutic Night Cream – твій must-have для міцних капілярів та спокійної шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>802-1</t>
+  </si>
+  <si>
+    <t>802-1(1)</t>
+  </si>
+  <si>
+    <t>Зміцнювальний Денний крем для чутливої, куперозної шкіри SPF 20 - 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Strengthening Day Cream SPF 20 – щоденний захист та комфорт! ✨
+🌿 Професійна формула для проблемної шкіри:
+☀️ Захист від UVA/UVB-променів завдяки SPF 20
+🌸 Зміцнює капіляри та судини
+💧 Зменшує почервоніння та подразнення
+🛡️ Натуральні екстракти магнолії та шафрану для комплексного догляду
+⚡ Відновлює ліпідний баланс та підтримує мікроциркуляцію
+💚 Результат – спокійна, рівна та доглянута шкіра протягом дня!
+📌 Показання до застосування:
+Купероз та розацеа
+Судинні сітки та зірочки
+Реактивна та суха шкіра
+Приливний рум’янець
+Порушення мікроциркуляції
+Локальні запалення
+📌 Активні компоненти:
+🌺 Екстракт магнолії та шафрану – протизапальна та освітлююча дія
+☀️ Комплекс UVA/UVB-фільтрів – сонцезахисний ефект
+🥑 Олії ши, аргани та нони – живлення та відновлення бар’єру
+🌿 Escin ß-Sitosterol Phtosome®, ескулін, рутин – зміцнення судинної системи
+💧 Гіалуронова кислота та пептиди – зволоження та підвищення еластичності
+⚡ Кофеїн та CM-Naringenin-Chalcone – стимуляція мікроциркуляції
+📌 Спосіб використання:  
+Нанести крем на очищену шкіру обличчя щоранку. Рівномірно розподілити по всій поверхні, уникаючи зони навколо очей.
+✔️ Характеристики продукту:
+Тип: Денний крем для чутливої шкіри
+Об’єм: 230 мл
+Призначення: Зміцнення судин, зменшення почервонінь, освітлення пігментації, захист SPF 20
+Тип шкіри: Чутлива, суха, куперозна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Strengthening Day Cream SPF 20 – твій must-have для щоденного захисту та здорової шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>801</t>
+  </si>
+  <si>
+    <t>801(1)</t>
+  </si>
+  <si>
+    <t>Інтенсивна зміцнювальний маска "розкішна магнолія" 300 мл</t>
+  </si>
+  <si>
+    <t>807(1)</t>
+  </si>
+  <si>
+    <t>807</t>
+  </si>
+  <si>
+    <t>✨ Luxury Magnolia Mask – інтенсивне зміцнення та комфорт! ✨
+🌿 Формула для чутливої та схильної до почервоніння шкіри:
+💧 Заспокоює реактивну та роздратовану шкіру
+🌸 Зміцнює судинну стінку та знижує їх реактивність
+🛡️ Відновлює гідроліпідну мантію та бар’єрні функції
+⚡ Виражено зволожує та тонізує
+🌟 Сприяє загоєнню дрібних тріщин та мікропошкоджень
+💚 Результат – спокійна, міцна та сяюча шкіра після кожного застосування!
+📌 Показання до застосування:
+Купероз та розацеа
+Судинна сітка та зірочки
+Почервоніння та приливний рум’янець
+Порушення мікроциркуляції
+Суха та чутлива шкіра
+📌 Активні компоненти:
+🌺 MAXnolia та гідролат гамамелісу – протизапальна та заспокійлива дія
+🌱 Escin ß-Sitosterol Phtosome, ескулін, рутин – зміцнення судин
+💧 Unisooth ST-32, бета-глюкан, д-пантеніл триацетат – зволоження та відновлення
+🌸 Ацетил-тетрапептиди та пальмітол трипептид-8 – регенерація та підвищення еластичності
+🛡️ Екстракти імбиру, лакриці та гарпагофітуму – антиоксидантна та протизапальна дія
+⚡ PINOLUMIN PWD, CM-Naringenin-Chalcone – освітлення та вирівнювання тону
+📌 Спосіб використання:  
+Нанести маску на чисту шкіру обличчя, залишити на 10–15 хвилин, після чого змити теплою водою. Використовувати 1–2 рази на тиждень.
+✔️ Характеристики продукту:
+Тип: Зміцнювальна маска для обличчя
+Об’єм: 300 мл
+Призначення: Зміцнення судин, зволоження, заспокоєння, освітлення
+Тип шкіри: Чутлива, суха, куперозна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Magnolia Mask – твій must-have для міцної та сяючої шкіри без почервонінь! 🌟</t>
+  </si>
+  <si>
+    <t>Нейроседативний бустер для чутливої та куперозної шкіри 10 мл</t>
+  </si>
+  <si>
+    <t>10 мл</t>
+  </si>
+  <si>
+    <t>804</t>
+  </si>
+  <si>
+    <t>804(1)</t>
+  </si>
+  <si>
+    <t>✨ Neuro-Calm Booster – інтенсивна підтримка судин та спокій шкіри! ✨
+🌿 Висококонцентрована формула для проблемної та реактивної шкіри:
+💧 Зменшує нервову реакцію на зовнішні подразники
+🌸 Усуває нейрогенне запалення та почервоніння
+🛡️ Зміцнює стінки судин та зменшує їх проникність
+⚡ Покращує мікроциркуляцію крові та лімфовідтік
+🌟 Відновлює еластичність та міцність судин
+💚 Результат – спокійна, рівна та доглянута шкіра без судинних проявів!
+📌 Показання до застосування:
+Купероз та розацеа
+Судинна сітка та зірочки
+Почервоніння та роздратована шкіра
+Реактивна та чутлива шкіра
+Приливний рум’янець
+Порушення мікроциркуляції
+📌 Активні компоненти:
+🌺 MAXnolia та Anasensyl LS 9322 – заспокійлива та протизапальна дія
+🌱 Escin ß-Sitosterol Phtosome, ескулін, рутин – зміцнення судинної системи
+💧 Гіалуронова кислота та бета-глюкан – глибоке зволоження та відновлення
+⚡ Endothelyol та кофеїн – стимуляція мікроциркуляції
+🌸 Ацетил-тетрапептиди та пальмітол трипептид-8 – регенерація та підвищення еластичності
+🌟 CM-Naringenin-Chalcone та PINOLUMIN PWD – зменшення реактивності та освітлення тону
+📌 Спосіб використання:  
+Нанести кілька крапель бустера на очищену шкіру обличчя, особливо на ділянки з судинними проявами. Використовувати щодня перед нанесенням крему.
+✔️ Характеристики продукту:
+Тип: Інтенсивна сироватка-бустер
+Об’єм: 10 мл
+Призначення: Зміцнення судин, зменшення почервонінь, заспокоєння
+Тип шкіри: Чутлива, куперозна, реактивна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Neuro-Calm Booster – твій must-have для боротьби з куперозом та відновлення спокою шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>Зміцнювалиний 2х-фазний Тонер для чутливої та куперозної шкіри 500 мл</t>
+  </si>
+  <si>
+    <t>✨ Strengthening 2-Phase Toner – щоденний догляд та комфорт! ✨
+🌿 Формула без спирту для делікатної шкіри:
+💧 Швидко заспокоює подразнення та зменшує почервоніння
+🌸 Знімає набряки та відновлює бар’єр шкіри
+🛡️ Зміцнює судини та капіляри
+⚡ Вирівнює тон та підтримує баланс мікробіому
+🌟 Дарує свіжість та здоровий вигляд щодня
+💚 Результат – спокійна, рівна та доглянута шкіра без куперозу!
+📌 Ключові компоненти:
+🌱 Гідролізат гамамелісу + квіткова вода – заспокоює та звужує пори
+⚡ Есцин + кофеїн – покращують мікроциркуляцію та знімають набряки
+💧 Пантенол + бісаболол – зволоження та відновлення
+🌸 Ніацинамід – вирівнює тон шкіри
+🌿 Пребіотики – підтримують баланс мікробіому
+🌺 Екстракт камелії – додаткове заспокоєння
+📌 Переваги:
+Зміцнення судин та зменшення куперозу
+Усунення набряків та почервонінь
+Відновлення захисного бар’єру
+📌 Спосіб використання:  
+Перед застосуванням струсити. Нанести тонер на ватний диск та протерти обличчя вранці й ввечері після очищення.
+✔️ Характеристики продукту:
+Тип: Двофазний тонер для обличчя
+Об’єм: 500 мл
+Призначення: Заспокоєння, зміцнення судин, зменшення почервонінь
+Тип шкіри: Чутлива, суха, куперозна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Strengthening 2-Phase Toner – твій must-have для щоденного комфорту та здорової шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>810</t>
+  </si>
+  <si>
+    <t>810(1)</t>
+  </si>
+  <si>
+    <t>Міцелярний очищувальний крем-гель для чутливої, куперозної шкіри 500 мл</t>
+  </si>
+  <si>
+    <t>✨ Smart4Derma Micellar Cream-Gel – ніжне очищення та захист! ✨
+🌿 Формула для делікатного догляду:
+💧 Дбайливо очищує та видаляє макіяж без подразнень
+🌸 Заспокоює та зменшує почервоніння
+🛡️ Захищає від окислювального стресу
+⚡ Стимулює синтез колагену та підтримує пружність
+🌟 Зберігає природний гідроліпідний баланс
+💚 Результат – чиста, свіжа та доглянута шкіра щодня!
+📌 Переваги:
+М’яке очищення та видалення макіяжу
+Заспокійлива та антиоксидантна дія
+Стимуляція синтезу колагену
+Підтримка природного балансу шкіри
+📌 Активні компоненти:
+🌺 Водорозчинна арганова олія – делікатне очищення
+🌸 Екстракт магнолії (Maxnolia) – антиоксидантний захист
+🌱 Пептид Skinasensyl – зменшення чутливості
+☕ Кофеїн – стимуляція мікроциркуляції
+🌼 Екстракти женьшеню, ромашки та інші фітоекстракти – живлення та відновлення
+💧 Вітамін Е та гліцерин – зволоження та еластичність
+📌 Спосіб використання:  
+Нанести на вологу шкіру, легко помасажувати та змити водою. Використовувати вранці та ввечері.
+✔️ Характеристики продукту:
+Тип: Міцелярний очищувальний крем-гель
+Об’єм: 500 мл
+Призначення: Очищення, заспокоєння, зміцнення судин, антиоксидантний захист
+Тип шкіри: Чутлива, суха, куперозна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Smart4Derma Micellar Cream-Gel – твій must-have для ніжного очищення та здорової шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>808</t>
+  </si>
+  <si>
+    <t>808(1)</t>
+  </si>
+  <si>
+    <t>Вдосконалювальний Крем з ретинолом та церамідами 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Advanced Retinol &amp; Ceramide Cream – нічне відновлення та омолодження! ✨
+🌿 Передова антивікова формула:
+💎 Мікрокапсульований ретинол – контрольована нічна ексфоліація без подразнень
+🌸 Цераміди – відновлення епідермального бар’єру та захист від втрати вологи
+💧 Гіалуронат натрію та рослинні олії – глибоке зволоження та живлення
+🛡️ ПДРН та Lipobelle Soyaglycone – стимуляція регенерації та синтезу колагену
+🌟 RetiSTAR та рослинний ретинол – потужна антивікова дія
+💚 Результат – пружна, гладка та сяюча шкіра щоранку!
+📌 Дія крему:
+Розгладжує статичні та мімічні зморшки
+Відновлює пружність та еластичність
+Покращує колір обличчя та коригує постакне
+Забезпечує оптимальне зволоження
+Зміцнює дерма-епідермальне сполучення
+📌 Показання:
+Фото- та хроностаріння
+Зморшки та знижений тонус
+Тьмяний колір та гіперпігментація
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Спосіб використання:  
+Рекомендовано для нічного застосування на віковій шкірі. Нанести на очищене обличчя та шию перед сном, рівномірно розподілити легкими рухами.
+✔️ Характеристики продукту:
+Тип: Антивіковий нічний крем
+Об’єм: 230 мл
+Призначення: Омолодження, освітлення, зволоження, відновлення бар’єру
+Тип шкіри: Зріла, суха, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced Retinol &amp; Ceramide Cream – твій must-have для молодої та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>731-1</t>
+  </si>
+  <si>
+    <t>731-1(1)</t>
   </si>
 </sst>
 </file>
@@ -5717,9 +6894,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="49" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -5731,9 +6905,6 @@
     <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5743,12 +6914,186 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Відсотковий" xfId="1" builtinId="5"/>
     <cellStyle name="Звичайний" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="24">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9EAD3"/>
+          <bgColor rgb="FFD9EAD3"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+          <bgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF4CCCC"/>
+          <bgColor rgb="FFF4CCCC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -6033,25 +7378,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K93"/>
+  <dimension ref="A1:K158"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12" style="13" customWidth="1"/>
-    <col min="2" max="2" width="74.77734375" style="10" customWidth="1"/>
-    <col min="3" max="3" width="16" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.88671875" style="10" customWidth="1"/>
-    <col min="5" max="5" width="20.5546875" style="10" customWidth="1"/>
-    <col min="6" max="6" width="13.6640625" style="10" customWidth="1"/>
-    <col min="7" max="7" width="12" style="10" customWidth="1"/>
-    <col min="8" max="8" width="18.88671875" style="10" customWidth="1"/>
-    <col min="9" max="9" width="21.109375" style="10" customWidth="1"/>
-    <col min="10" max="10" width="44" style="10" customWidth="1"/>
-    <col min="11" max="11" width="18" style="13" customWidth="1"/>
-    <col min="12" max="16384" width="8.88671875" style="10"/>
+    <col min="1" max="1" width="12" style="12" customWidth="1"/>
+    <col min="2" max="2" width="37.44140625" style="9" customWidth="1"/>
+    <col min="3" max="3" width="16" style="9" customWidth="1"/>
+    <col min="4" max="4" width="14.88671875" style="9" customWidth="1"/>
+    <col min="5" max="5" width="12.77734375" style="9" customWidth="1"/>
+    <col min="6" max="6" width="13.6640625" style="9" customWidth="1"/>
+    <col min="7" max="7" width="12" style="9" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" style="9" customWidth="1"/>
+    <col min="9" max="9" width="21.109375" style="9" customWidth="1"/>
+    <col min="10" max="10" width="56" style="9" customWidth="1"/>
+    <col min="11" max="11" width="18" style="12" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="9"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" s="7" customFormat="1" ht="34.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
@@ -6081,18 +7426,18 @@
       <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="11" t="s">
+      <c r="K1" s="10" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>649</v>
       </c>
-      <c r="B2" s="16" t="s">
+      <c r="B2" s="14" t="s">
         <v>650</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="14" t="s">
         <v>653</v>
       </c>
       <c r="D2" s="8">
@@ -6105,27 +7450,27 @@
       <c r="G2" s="8">
         <v>10</v>
       </c>
-      <c r="H2" s="16" t="s">
+      <c r="H2" s="14" t="s">
         <v>652</v>
       </c>
-      <c r="I2" s="16" t="s">
+      <c r="I2" s="14" t="s">
         <v>657</v>
       </c>
-      <c r="J2" s="16" t="s">
+      <c r="J2" s="14" t="s">
         <v>651</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="15" t="s">
         <v>649</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="13" t="s">
         <v>655</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="14" t="s">
         <v>654</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="14" t="s">
         <v>658</v>
       </c>
       <c r="D3" s="8">
@@ -6138,27 +7483,27 @@
       <c r="G3" s="8">
         <v>25</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="14" t="s">
         <v>657</v>
       </c>
-      <c r="J3" s="16" t="s">
+      <c r="J3" s="14" t="s">
         <v>656</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="15" t="s">
         <v>655</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="13" t="s">
         <v>660</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="14" t="s">
         <v>659</v>
       </c>
-      <c r="C4" s="16" t="s">
+      <c r="C4" s="14" t="s">
         <v>658</v>
       </c>
       <c r="D4" s="8">
@@ -6171,27 +7516,27 @@
       <c r="G4" s="8">
         <v>35</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="I4" s="16" t="s">
+      <c r="I4" s="14" t="s">
         <v>657</v>
       </c>
-      <c r="J4" s="16" t="s">
+      <c r="J4" s="14" t="s">
         <v>661</v>
       </c>
-      <c r="K4" s="17" t="s">
+      <c r="K4" s="15" t="s">
         <v>660</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>663</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="14" t="s">
         <v>662</v>
       </c>
-      <c r="C5" s="16" t="s">
+      <c r="C5" s="14" t="s">
         <v>658</v>
       </c>
       <c r="D5" s="8">
@@ -6204,21 +7549,21 @@
       <c r="G5" s="8">
         <v>31</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="14" t="s">
         <v>664</v>
       </c>
-      <c r="I5" s="16" t="s">
+      <c r="I5" s="14" t="s">
         <v>657</v>
       </c>
-      <c r="J5" s="16" t="s">
+      <c r="J5" s="14" t="s">
         <v>665</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="15" t="s">
         <v>663</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="11" t="s">
         <v>668</v>
       </c>
       <c r="B6" s="8" t="s">
@@ -6246,12 +7591,12 @@
       <c r="J6" s="8" t="s">
         <v>667</v>
       </c>
-      <c r="K6" s="18" t="s">
+      <c r="K6" s="16" t="s">
         <v>668</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="11" t="s">
         <v>670</v>
       </c>
       <c r="B7" s="8" t="s">
@@ -6277,12 +7622,12 @@
       <c r="J7" s="8" t="s">
         <v>671</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="16" t="s">
         <v>670</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="11" t="s">
         <v>674</v>
       </c>
       <c r="B8" s="8" t="s">
@@ -6308,12 +7653,12 @@
       <c r="J8" s="8" t="s">
         <v>675</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="16" t="s">
         <v>674</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="11" t="s">
         <v>677</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -6339,12 +7684,12 @@
       <c r="J9" s="8" t="s">
         <v>678</v>
       </c>
-      <c r="K9" s="18" t="s">
+      <c r="K9" s="16" t="s">
         <v>677</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="11" t="s">
         <v>680</v>
       </c>
       <c r="B10" s="8" t="s">
@@ -6370,12 +7715,12 @@
       <c r="J10" s="8" t="s">
         <v>681</v>
       </c>
-      <c r="K10" s="18" t="s">
+      <c r="K10" s="16" t="s">
         <v>680</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="11" t="s">
         <v>683</v>
       </c>
       <c r="B11" s="8" t="s">
@@ -6401,12 +7746,12 @@
       <c r="J11" s="8" t="s">
         <v>684</v>
       </c>
-      <c r="K11" s="18" t="s">
+      <c r="K11" s="16" t="s">
         <v>683</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="11" t="s">
         <v>687</v>
       </c>
       <c r="B12" s="8" t="s">
@@ -6432,12 +7777,12 @@
       <c r="J12" s="8" t="s">
         <v>686</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="K12" s="16" t="s">
         <v>687</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="11" t="s">
         <v>689</v>
       </c>
       <c r="B13" s="8" t="s">
@@ -6463,12 +7808,12 @@
       <c r="J13" s="8" t="s">
         <v>690</v>
       </c>
-      <c r="K13" s="18" t="s">
+      <c r="K13" s="16" t="s">
         <v>689</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="12" t="s">
+      <c r="A14" s="11" t="s">
         <v>693</v>
       </c>
       <c r="B14" s="8" t="s">
@@ -6494,12 +7839,12 @@
       <c r="J14" s="8" t="s">
         <v>692</v>
       </c>
-      <c r="K14" s="18" t="s">
+      <c r="K14" s="16" t="s">
         <v>693</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="11" t="s">
         <v>696</v>
       </c>
       <c r="B15" s="8" t="s">
@@ -6525,12 +7870,12 @@
       <c r="J15" s="8" t="s">
         <v>697</v>
       </c>
-      <c r="K15" s="18" t="s">
+      <c r="K15" s="16" t="s">
         <v>696</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="11" t="s">
         <v>699</v>
       </c>
       <c r="B16" s="8" t="s">
@@ -6556,12 +7901,12 @@
       <c r="J16" s="8" t="s">
         <v>700</v>
       </c>
-      <c r="K16" s="18" t="s">
+      <c r="K16" s="16" t="s">
         <v>699</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="11" t="s">
         <v>702</v>
       </c>
       <c r="B17" s="8" t="s">
@@ -6587,12 +7932,12 @@
       <c r="J17" s="8" t="s">
         <v>703</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="K17" s="16" t="s">
         <v>702</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="11" t="s">
         <v>705</v>
       </c>
       <c r="B18" s="8" t="s">
@@ -6618,12 +7963,12 @@
       <c r="J18" s="8" t="s">
         <v>706</v>
       </c>
-      <c r="K18" s="18" t="s">
+      <c r="K18" s="16" t="s">
         <v>705</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" s="12" t="s">
+      <c r="A19" s="11" t="s">
         <v>708</v>
       </c>
       <c r="B19" s="8" t="s">
@@ -6649,12 +7994,12 @@
       <c r="J19" s="8" t="s">
         <v>709</v>
       </c>
-      <c r="K19" s="18" t="s">
+      <c r="K19" s="16" t="s">
         <v>708</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" s="12" t="s">
+      <c r="A20" s="11" t="s">
         <v>710</v>
       </c>
       <c r="B20" s="8" t="s">
@@ -6680,12 +8025,12 @@
       <c r="J20" s="8" t="s">
         <v>711</v>
       </c>
-      <c r="K20" s="18" t="s">
+      <c r="K20" s="16" t="s">
         <v>710</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>713</v>
       </c>
       <c r="B21" s="8" t="s">
@@ -6711,12 +8056,12 @@
       <c r="J21" s="8" t="s">
         <v>714</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="K21" s="16" t="s">
         <v>713</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>717</v>
       </c>
       <c r="B22" s="8" t="s">
@@ -6742,12 +8087,12 @@
       <c r="J22" s="8" t="s">
         <v>716</v>
       </c>
-      <c r="K22" s="18" t="s">
+      <c r="K22" s="16" t="s">
         <v>717</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>720</v>
       </c>
       <c r="B23" s="8" t="s">
@@ -6773,12 +8118,12 @@
       <c r="J23" s="8" t="s">
         <v>719</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="K23" s="16" t="s">
         <v>720</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" s="12" t="s">
+      <c r="A24" s="11" t="s">
         <v>722</v>
       </c>
       <c r="B24" s="8" t="s">
@@ -6804,12 +8149,12 @@
       <c r="J24" s="8" t="s">
         <v>723</v>
       </c>
-      <c r="K24" s="18" t="s">
+      <c r="K24" s="16" t="s">
         <v>722</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="11" t="s">
         <v>726</v>
       </c>
       <c r="B25" s="8" t="s">
@@ -6835,12 +8180,12 @@
       <c r="J25" s="8" t="s">
         <v>725</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="K25" s="16" t="s">
         <v>726</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="11" t="s">
         <v>728</v>
       </c>
       <c r="B26" s="8" t="s">
@@ -6866,12 +8211,12 @@
       <c r="J26" s="8" t="s">
         <v>729</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="K26" s="16" t="s">
         <v>728</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="11" t="s">
         <v>731</v>
       </c>
       <c r="B27" s="8" t="s">
@@ -6897,12 +8242,12 @@
       <c r="J27" s="8" t="s">
         <v>732</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="K27" s="16" t="s">
         <v>731</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="11" t="s">
         <v>734</v>
       </c>
       <c r="B28" s="8" t="s">
@@ -6928,12 +8273,12 @@
       <c r="J28" s="8" t="s">
         <v>735</v>
       </c>
-      <c r="K28" s="18" t="s">
+      <c r="K28" s="16" t="s">
         <v>734</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="11" t="s">
         <v>737</v>
       </c>
       <c r="B29" s="8" t="s">
@@ -6959,12 +8304,12 @@
       <c r="J29" s="8" t="s">
         <v>738</v>
       </c>
-      <c r="K29" s="18" t="s">
+      <c r="K29" s="16" t="s">
         <v>737</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="11" t="s">
         <v>741</v>
       </c>
       <c r="B30" s="8" t="s">
@@ -6990,12 +8335,12 @@
       <c r="J30" s="8" t="s">
         <v>740</v>
       </c>
-      <c r="K30" s="18" t="s">
+      <c r="K30" s="16" t="s">
         <v>741</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="11" t="s">
         <v>743</v>
       </c>
       <c r="B31" s="8" t="s">
@@ -7021,12 +8366,12 @@
       <c r="J31" s="8" t="s">
         <v>744</v>
       </c>
-      <c r="K31" s="18" t="s">
+      <c r="K31" s="16" t="s">
         <v>743</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="11" t="s">
         <v>746</v>
       </c>
       <c r="B32" s="8" t="s">
@@ -7052,12 +8397,12 @@
       <c r="J32" s="8" t="s">
         <v>747</v>
       </c>
-      <c r="K32" s="18" t="s">
+      <c r="K32" s="16" t="s">
         <v>746</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="11" t="s">
         <v>749</v>
       </c>
       <c r="B33" s="8" t="s">
@@ -7083,12 +8428,12 @@
       <c r="J33" s="8" t="s">
         <v>750</v>
       </c>
-      <c r="K33" s="18" t="s">
+      <c r="K33" s="16" t="s">
         <v>749</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="11" t="s">
         <v>753</v>
       </c>
       <c r="B34" s="8" t="s">
@@ -7114,12 +8459,12 @@
       <c r="J34" s="8" t="s">
         <v>752</v>
       </c>
-      <c r="K34" s="18" t="s">
+      <c r="K34" s="16" t="s">
         <v>754</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="11" t="s">
         <v>756</v>
       </c>
       <c r="B35" s="8" t="s">
@@ -7145,12 +8490,12 @@
       <c r="J35" s="8" t="s">
         <v>757</v>
       </c>
-      <c r="K35" s="18" t="s">
+      <c r="K35" s="16" t="s">
         <v>756</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="11" t="s">
         <v>760</v>
       </c>
       <c r="B36" s="8" t="s">
@@ -7176,12 +8521,12 @@
       <c r="J36" s="8" t="s">
         <v>759</v>
       </c>
-      <c r="K36" s="18" t="s">
+      <c r="K36" s="16" t="s">
         <v>760</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="11" t="s">
         <v>763</v>
       </c>
       <c r="B37" s="8" t="s">
@@ -7207,12 +8552,12 @@
       <c r="J37" s="8" t="s">
         <v>762</v>
       </c>
-      <c r="K37" s="18" t="s">
+      <c r="K37" s="16" t="s">
         <v>763</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A38" s="12" t="s">
+      <c r="A38" s="11" t="s">
         <v>766</v>
       </c>
       <c r="B38" s="8" t="s">
@@ -7238,12 +8583,12 @@
       <c r="J38" s="8" t="s">
         <v>765</v>
       </c>
-      <c r="K38" s="18" t="s">
+      <c r="K38" s="16" t="s">
         <v>766</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A39" s="12" t="s">
+      <c r="A39" s="11" t="s">
         <v>768</v>
       </c>
       <c r="B39" s="8" t="s">
@@ -7269,12 +8614,12 @@
       <c r="J39" s="8" t="s">
         <v>769</v>
       </c>
-      <c r="K39" s="18" t="s">
+      <c r="K39" s="16" t="s">
         <v>768</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A40" s="12" t="s">
+      <c r="A40" s="11" t="s">
         <v>771</v>
       </c>
       <c r="B40" s="8" t="s">
@@ -7300,12 +8645,12 @@
       <c r="J40" s="8" t="s">
         <v>772</v>
       </c>
-      <c r="K40" s="18" t="s">
+      <c r="K40" s="16" t="s">
         <v>771</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="11" t="s">
         <v>774</v>
       </c>
       <c r="B41" s="8" t="s">
@@ -7331,12 +8676,12 @@
       <c r="J41" s="8" t="s">
         <v>775</v>
       </c>
-      <c r="K41" s="18" t="s">
+      <c r="K41" s="16" t="s">
         <v>774</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A42" s="12" t="s">
+      <c r="A42" s="11" t="s">
         <v>777</v>
       </c>
       <c r="B42" s="8" t="s">
@@ -7362,12 +8707,12 @@
       <c r="J42" s="8" t="s">
         <v>778</v>
       </c>
-      <c r="K42" s="18" t="s">
+      <c r="K42" s="16" t="s">
         <v>777</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A43" s="12" t="s">
+      <c r="A43" s="11" t="s">
         <v>781</v>
       </c>
       <c r="B43" s="8" t="s">
@@ -7393,12 +8738,12 @@
       <c r="J43" s="8" t="s">
         <v>780</v>
       </c>
-      <c r="K43" s="18" t="s">
+      <c r="K43" s="16" t="s">
         <v>781</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
+      <c r="A44" s="11" t="s">
         <v>784</v>
       </c>
       <c r="B44" s="8" t="s">
@@ -7424,12 +8769,12 @@
       <c r="J44" s="8" t="s">
         <v>785</v>
       </c>
-      <c r="K44" s="18" t="s">
+      <c r="K44" s="16" t="s">
         <v>784</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="11" t="s">
         <v>787</v>
       </c>
       <c r="B45" s="8" t="s">
@@ -7455,12 +8800,12 @@
       <c r="J45" s="8" t="s">
         <v>788</v>
       </c>
-      <c r="K45" s="18" t="s">
+      <c r="K45" s="16" t="s">
         <v>787</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A46" s="12" t="s">
+      <c r="A46" s="11" t="s">
         <v>790</v>
       </c>
       <c r="B46" s="8" t="s">
@@ -7486,12 +8831,12 @@
       <c r="J46" s="8" t="s">
         <v>789</v>
       </c>
-      <c r="K46" s="18" t="s">
+      <c r="K46" s="16" t="s">
         <v>790</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A47" s="12" t="s">
+      <c r="A47" s="11" t="s">
         <v>791</v>
       </c>
       <c r="B47" s="8" t="s">
@@ -7517,12 +8862,12 @@
       <c r="J47" s="8" t="s">
         <v>792</v>
       </c>
-      <c r="K47" s="18" t="s">
+      <c r="K47" s="16" t="s">
         <v>791</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="11" t="s">
         <v>796</v>
       </c>
       <c r="B48" s="8" t="s">
@@ -7548,12 +8893,12 @@
       <c r="J48" s="8" t="s">
         <v>797</v>
       </c>
-      <c r="K48" s="18" t="s">
+      <c r="K48" s="16" t="s">
         <v>796</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A49" s="12" t="s">
+      <c r="A49" s="11" t="s">
         <v>799</v>
       </c>
       <c r="B49" s="8" t="s">
@@ -7579,12 +8924,12 @@
       <c r="J49" s="8" t="s">
         <v>800</v>
       </c>
-      <c r="K49" s="18" t="s">
+      <c r="K49" s="16" t="s">
         <v>799</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A50" s="12" t="s">
+      <c r="A50" s="11" t="s">
         <v>802</v>
       </c>
       <c r="B50" s="8" t="s">
@@ -7610,12 +8955,12 @@
       <c r="J50" s="8" t="s">
         <v>803</v>
       </c>
-      <c r="K50" s="18" t="s">
+      <c r="K50" s="16" t="s">
         <v>802</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="11" t="s">
         <v>805</v>
       </c>
       <c r="B51" s="8" t="s">
@@ -7641,12 +8986,12 @@
       <c r="J51" s="8" t="s">
         <v>806</v>
       </c>
-      <c r="K51" s="18" t="s">
+      <c r="K51" s="16" t="s">
         <v>805</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A52" s="12" t="s">
+      <c r="A52" s="11" t="s">
         <v>810</v>
       </c>
       <c r="B52" s="8" t="s">
@@ -7672,12 +9017,12 @@
       <c r="J52" s="8" t="s">
         <v>809</v>
       </c>
-      <c r="K52" s="18" t="s">
+      <c r="K52" s="16" t="s">
         <v>810</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
+      <c r="A53" s="11" t="s">
         <v>812</v>
       </c>
       <c r="B53" s="8" t="s">
@@ -7703,12 +9048,12 @@
       <c r="J53" s="8" t="s">
         <v>813</v>
       </c>
-      <c r="K53" s="18" t="s">
+      <c r="K53" s="16" t="s">
         <v>812</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A54" s="12" t="s">
+      <c r="A54" s="11" t="s">
         <v>816</v>
       </c>
       <c r="B54" s="8" t="s">
@@ -7734,12 +9079,12 @@
       <c r="J54" s="8" t="s">
         <v>815</v>
       </c>
-      <c r="K54" s="18" t="s">
+      <c r="K54" s="16" t="s">
         <v>816</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A55" s="12" t="s">
+      <c r="A55" s="11" t="s">
         <v>818</v>
       </c>
       <c r="B55" s="8" t="s">
@@ -7765,12 +9110,12 @@
       <c r="J55" s="8" t="s">
         <v>819</v>
       </c>
-      <c r="K55" s="18" t="s">
+      <c r="K55" s="16" t="s">
         <v>818</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A56" s="12" t="s">
+      <c r="A56" s="11" t="s">
         <v>822</v>
       </c>
       <c r="B56" s="8" t="s">
@@ -7796,12 +9141,12 @@
       <c r="J56" s="8" t="s">
         <v>821</v>
       </c>
-      <c r="K56" s="18" t="s">
+      <c r="K56" s="16" t="s">
         <v>822</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A57" s="12" t="s">
+      <c r="A57" s="11" t="s">
         <v>825</v>
       </c>
       <c r="B57" s="8" t="s">
@@ -7827,12 +9172,12 @@
       <c r="J57" s="8" t="s">
         <v>824</v>
       </c>
-      <c r="K57" s="18" t="s">
+      <c r="K57" s="16" t="s">
         <v>825</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A58" s="12" t="s">
+      <c r="A58" s="11" t="s">
         <v>828</v>
       </c>
       <c r="B58" s="8" t="s">
@@ -7858,12 +9203,12 @@
       <c r="J58" s="8" t="s">
         <v>827</v>
       </c>
-      <c r="K58" s="18" t="s">
+      <c r="K58" s="16" t="s">
         <v>828</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="11" t="s">
         <v>831</v>
       </c>
       <c r="B59" s="8" t="s">
@@ -7889,12 +9234,12 @@
       <c r="J59" s="8" t="s">
         <v>830</v>
       </c>
-      <c r="K59" s="18" t="s">
+      <c r="K59" s="16" t="s">
         <v>831</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A60" s="12" t="s">
+      <c r="A60" s="11" t="s">
         <v>834</v>
       </c>
       <c r="B60" s="8" t="s">
@@ -7920,12 +9265,12 @@
       <c r="J60" s="8" t="s">
         <v>833</v>
       </c>
-      <c r="K60" s="18" t="s">
+      <c r="K60" s="16" t="s">
         <v>834</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A61" s="12" t="s">
+      <c r="A61" s="11" t="s">
         <v>837</v>
       </c>
       <c r="B61" s="8" t="s">
@@ -7951,12 +9296,12 @@
       <c r="J61" s="8" t="s">
         <v>836</v>
       </c>
-      <c r="K61" s="18" t="s">
+      <c r="K61" s="16" t="s">
         <v>837</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A62" s="12" t="s">
+      <c r="A62" s="11" t="s">
         <v>839</v>
       </c>
       <c r="B62" s="8" t="s">
@@ -7982,12 +9327,12 @@
       <c r="J62" s="8" t="s">
         <v>840</v>
       </c>
-      <c r="K62" s="18" t="s">
+      <c r="K62" s="16" t="s">
         <v>839</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A63" s="12" t="s">
+      <c r="A63" s="11" t="s">
         <v>843</v>
       </c>
       <c r="B63" s="8" t="s">
@@ -8013,12 +9358,12 @@
       <c r="J63" s="8" t="s">
         <v>842</v>
       </c>
-      <c r="K63" s="18" t="s">
+      <c r="K63" s="16" t="s">
         <v>843</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A64" s="12" t="s">
+      <c r="A64" s="11" t="s">
         <v>846</v>
       </c>
       <c r="B64" s="8" t="s">
@@ -8044,12 +9389,12 @@
       <c r="J64" s="8" t="s">
         <v>845</v>
       </c>
-      <c r="K64" s="18" t="s">
+      <c r="K64" s="16" t="s">
         <v>846</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A65" s="12" t="s">
+      <c r="A65" s="11" t="s">
         <v>849</v>
       </c>
       <c r="B65" s="8" t="s">
@@ -8075,12 +9420,12 @@
       <c r="J65" s="8" t="s">
         <v>848</v>
       </c>
-      <c r="K65" s="18" t="s">
+      <c r="K65" s="16" t="s">
         <v>849</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A66" s="12" t="s">
+      <c r="A66" s="11" t="s">
         <v>853</v>
       </c>
       <c r="B66" s="8" t="s">
@@ -8106,12 +9451,12 @@
       <c r="J66" s="8" t="s">
         <v>852</v>
       </c>
-      <c r="K66" s="18" t="s">
+      <c r="K66" s="16" t="s">
         <v>853</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A67" s="12" t="s">
+      <c r="A67" s="11" t="s">
         <v>856</v>
       </c>
       <c r="B67" s="8" t="s">
@@ -8137,12 +9482,12 @@
       <c r="J67" s="8" t="s">
         <v>855</v>
       </c>
-      <c r="K67" s="18" t="s">
+      <c r="K67" s="16" t="s">
         <v>856</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A68" s="12" t="s">
+      <c r="A68" s="11" t="s">
         <v>859</v>
       </c>
       <c r="B68" s="8" t="s">
@@ -8168,12 +9513,12 @@
       <c r="J68" s="8" t="s">
         <v>858</v>
       </c>
-      <c r="K68" s="18" t="s">
+      <c r="K68" s="16" t="s">
         <v>859</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A69" s="12" t="s">
+      <c r="A69" s="11" t="s">
         <v>861</v>
       </c>
       <c r="B69" s="8" t="s">
@@ -8199,12 +9544,12 @@
       <c r="J69" s="8" t="s">
         <v>862</v>
       </c>
-      <c r="K69" s="18" t="s">
+      <c r="K69" s="16" t="s">
         <v>861</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A70" s="12" t="s">
+      <c r="A70" s="11" t="s">
         <v>865</v>
       </c>
       <c r="B70" s="8" t="s">
@@ -8230,12 +9575,12 @@
       <c r="J70" s="8" t="s">
         <v>864</v>
       </c>
-      <c r="K70" s="18" t="s">
+      <c r="K70" s="16" t="s">
         <v>865</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A71" s="12" t="s">
+      <c r="A71" s="11" t="s">
         <v>867</v>
       </c>
       <c r="B71" s="8" t="s">
@@ -8261,12 +9606,12 @@
       <c r="J71" s="8" t="s">
         <v>868</v>
       </c>
-      <c r="K71" s="18" t="s">
+      <c r="K71" s="16" t="s">
         <v>867</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A72" s="12" t="s">
+      <c r="A72" s="11" t="s">
         <v>871</v>
       </c>
       <c r="B72" s="8" t="s">
@@ -8292,12 +9637,12 @@
       <c r="J72" s="8" t="s">
         <v>870</v>
       </c>
-      <c r="K72" s="18" t="s">
+      <c r="K72" s="16" t="s">
         <v>871</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A73" s="12" t="s">
+      <c r="A73" s="11" t="s">
         <v>874</v>
       </c>
       <c r="B73" s="8" t="s">
@@ -8323,12 +9668,12 @@
       <c r="J73" s="8" t="s">
         <v>873</v>
       </c>
-      <c r="K73" s="18" t="s">
+      <c r="K73" s="16" t="s">
         <v>874</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A74" s="12" t="s">
+      <c r="A74" s="11" t="s">
         <v>877</v>
       </c>
       <c r="B74" s="8" t="s">
@@ -8354,12 +9699,12 @@
       <c r="J74" s="8" t="s">
         <v>876</v>
       </c>
-      <c r="K74" s="18" t="s">
+      <c r="K74" s="16" t="s">
         <v>877</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A75" s="12" t="s">
+      <c r="A75" s="11" t="s">
         <v>880</v>
       </c>
       <c r="B75" s="8" t="s">
@@ -8385,12 +9730,12 @@
       <c r="J75" s="8" t="s">
         <v>879</v>
       </c>
-      <c r="K75" s="18" t="s">
+      <c r="K75" s="16" t="s">
         <v>880</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A76" s="12" t="s">
+      <c r="A76" s="11" t="s">
         <v>883</v>
       </c>
       <c r="B76" s="8" t="s">
@@ -8416,16 +9761,16 @@
       <c r="J76" s="8" t="s">
         <v>882</v>
       </c>
-      <c r="K76" s="18" t="s">
+      <c r="K76" s="16" t="s">
         <v>883</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A77" s="12" t="s">
-        <v>886</v>
+      <c r="A77" s="11" t="s">
+        <v>887</v>
       </c>
       <c r="B77" s="8" t="s">
-        <v>884</v>
+        <v>885</v>
       </c>
       <c r="C77" s="8" t="s">
         <v>653</v>
@@ -8445,18 +9790,18 @@
         <v>657</v>
       </c>
       <c r="J77" s="8" t="s">
-        <v>885</v>
-      </c>
-      <c r="K77" s="18" t="s">
         <v>886</v>
       </c>
+      <c r="K77" s="16" t="s">
+        <v>887</v>
+      </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A78" s="12" t="s">
-        <v>889</v>
+      <c r="A78" s="11" t="s">
+        <v>890</v>
       </c>
       <c r="B78" s="8" t="s">
-        <v>887</v>
+        <v>888</v>
       </c>
       <c r="C78" s="8" t="s">
         <v>653</v>
@@ -8476,18 +9821,18 @@
         <v>657</v>
       </c>
       <c r="J78" s="8" t="s">
-        <v>888</v>
-      </c>
-      <c r="K78" s="18" t="s">
         <v>889</v>
       </c>
+      <c r="K78" s="16" t="s">
+        <v>890</v>
+      </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A79" s="12" t="s">
-        <v>892</v>
+      <c r="A79" s="11" t="s">
+        <v>893</v>
       </c>
       <c r="B79" s="8" t="s">
-        <v>890</v>
+        <v>891</v>
       </c>
       <c r="C79" s="8" t="s">
         <v>653</v>
@@ -8507,18 +9852,18 @@
         <v>657</v>
       </c>
       <c r="J79" s="8" t="s">
-        <v>891</v>
-      </c>
-      <c r="K79" s="18" t="s">
         <v>892</v>
       </c>
+      <c r="K79" s="16" t="s">
+        <v>893</v>
+      </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A80" s="12" t="s">
-        <v>895</v>
+      <c r="A80" s="11" t="s">
+        <v>896</v>
       </c>
       <c r="B80" s="8" t="s">
-        <v>893</v>
+        <v>894</v>
       </c>
       <c r="C80" s="8" t="s">
         <v>653</v>
@@ -8538,18 +9883,18 @@
         <v>657</v>
       </c>
       <c r="J80" s="8" t="s">
-        <v>894</v>
-      </c>
-      <c r="K80" s="18" t="s">
         <v>895</v>
       </c>
+      <c r="K80" s="16" t="s">
+        <v>896</v>
+      </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A81" s="12" t="s">
-        <v>898</v>
+      <c r="A81" s="11" t="s">
+        <v>899</v>
       </c>
       <c r="B81" s="8" t="s">
-        <v>896</v>
+        <v>897</v>
       </c>
       <c r="C81" s="8" t="s">
         <v>653</v>
@@ -8569,173 +9914,1517 @@
         <v>657</v>
       </c>
       <c r="J81" s="8" t="s">
-        <v>897</v>
-      </c>
-      <c r="K81" s="18" t="s">
         <v>898</v>
       </c>
+      <c r="K81" s="16" t="s">
+        <v>899</v>
+      </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A82" s="12"/>
-      <c r="B82" s="8"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
+      <c r="A82" s="11" t="s">
+        <v>902</v>
+      </c>
+      <c r="B82" s="8" t="s">
+        <v>900</v>
+      </c>
+      <c r="C82" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D82" s="8">
+        <v>680</v>
+      </c>
       <c r="E82" s="8"/>
       <c r="F82" s="8"/>
-      <c r="G82" s="8"/>
-      <c r="H82" s="8"/>
+      <c r="G82" s="8">
+        <v>12</v>
+      </c>
+      <c r="H82" s="8" t="s">
+        <v>43</v>
+      </c>
       <c r="I82" s="8" t="s">
         <v>657</v>
       </c>
-      <c r="J82" s="8"/>
-      <c r="K82" s="18"/>
+      <c r="J82" s="8" t="s">
+        <v>901</v>
+      </c>
+      <c r="K82" s="16" t="s">
+        <v>902</v>
+      </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A83" s="12"/>
-      <c r="B83" s="9"/>
-      <c r="C83" s="9"/>
-      <c r="D83" s="8"/>
+      <c r="A83" s="11" t="s">
+        <v>905</v>
+      </c>
+      <c r="B83" s="8" t="s">
+        <v>903</v>
+      </c>
+      <c r="C83" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D83" s="8">
+        <v>700</v>
+      </c>
       <c r="E83" s="8"/>
       <c r="F83" s="8"/>
-      <c r="G83" s="8"/>
-      <c r="H83" s="8"/>
-      <c r="I83" s="8"/>
-      <c r="J83" s="9"/>
-      <c r="K83" s="15"/>
+      <c r="G83" s="8">
+        <v>16</v>
+      </c>
+      <c r="H83" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I83" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J83" s="8" t="s">
+        <v>904</v>
+      </c>
+      <c r="K83" s="16" t="s">
+        <v>905</v>
+      </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A84" s="12"/>
-      <c r="B84" s="9"/>
-      <c r="C84" s="9"/>
-      <c r="D84" s="8"/>
+      <c r="A84" s="11" t="s">
+        <v>907</v>
+      </c>
+      <c r="B84" s="8" t="s">
+        <v>906</v>
+      </c>
+      <c r="C84" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D84" s="8">
+        <v>700</v>
+      </c>
       <c r="E84" s="8"/>
       <c r="F84" s="8"/>
-      <c r="G84" s="8"/>
-      <c r="H84" s="8"/>
-      <c r="I84" s="8"/>
-      <c r="J84" s="9"/>
-      <c r="K84" s="15"/>
+      <c r="G84" s="8">
+        <v>21</v>
+      </c>
+      <c r="H84" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I84" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J84" s="8" t="s">
+        <v>908</v>
+      </c>
+      <c r="K84" s="16" t="s">
+        <v>907</v>
+      </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A85" s="12"/>
-      <c r="B85" s="9"/>
-      <c r="C85" s="9"/>
-      <c r="D85" s="8"/>
+      <c r="A85" s="11" t="s">
+        <v>910</v>
+      </c>
+      <c r="B85" s="8" t="s">
+        <v>909</v>
+      </c>
+      <c r="C85" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D85" s="8">
+        <v>860</v>
+      </c>
       <c r="E85" s="8"/>
       <c r="F85" s="8"/>
-      <c r="G85" s="8"/>
-      <c r="H85" s="8"/>
-      <c r="I85" s="8"/>
-      <c r="J85" s="9"/>
-      <c r="K85" s="15"/>
+      <c r="G85" s="8">
+        <v>23</v>
+      </c>
+      <c r="H85" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I85" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J85" s="8" t="s">
+        <v>911</v>
+      </c>
+      <c r="K85" s="16" t="s">
+        <v>910</v>
+      </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A86" s="12"/>
-      <c r="B86" s="9"/>
-      <c r="C86" s="9"/>
-      <c r="D86" s="8"/>
+      <c r="A86" s="11" t="s">
+        <v>914</v>
+      </c>
+      <c r="B86" s="8" t="s">
+        <v>912</v>
+      </c>
+      <c r="C86" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D86" s="8">
+        <v>720</v>
+      </c>
       <c r="E86" s="8"/>
       <c r="F86" s="8"/>
-      <c r="G86" s="8"/>
-      <c r="H86" s="8"/>
-      <c r="I86" s="8"/>
-      <c r="J86" s="9"/>
-      <c r="K86" s="15"/>
+      <c r="G86" s="8">
+        <v>24</v>
+      </c>
+      <c r="H86" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I86" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J86" s="8" t="s">
+        <v>913</v>
+      </c>
+      <c r="K86" s="16" t="s">
+        <v>914</v>
+      </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A87" s="12"/>
-      <c r="B87" s="9"/>
-      <c r="C87" s="9"/>
-      <c r="D87" s="8"/>
+      <c r="A87" s="11" t="s">
+        <v>917</v>
+      </c>
+      <c r="B87" s="8" t="s">
+        <v>916</v>
+      </c>
+      <c r="C87" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D87" s="8">
+        <v>1160</v>
+      </c>
       <c r="E87" s="8"/>
       <c r="F87" s="8"/>
-      <c r="G87" s="8"/>
-      <c r="H87" s="8"/>
-      <c r="I87" s="8"/>
-      <c r="J87" s="9"/>
-      <c r="K87" s="15"/>
+      <c r="G87" s="8">
+        <v>17</v>
+      </c>
+      <c r="H87" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I87" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J87" s="8" t="s">
+        <v>915</v>
+      </c>
+      <c r="K87" s="16" t="s">
+        <v>917</v>
+      </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A88" s="12"/>
-      <c r="B88" s="9"/>
-      <c r="C88" s="9"/>
-      <c r="D88" s="8"/>
+      <c r="A88" s="11" t="s">
+        <v>920</v>
+      </c>
+      <c r="B88" s="8" t="s">
+        <v>919</v>
+      </c>
+      <c r="C88" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D88" s="8">
+        <v>680</v>
+      </c>
       <c r="E88" s="8"/>
       <c r="F88" s="8"/>
-      <c r="G88" s="8"/>
-      <c r="H88" s="8"/>
-      <c r="I88" s="8"/>
-      <c r="J88" s="9"/>
-      <c r="K88" s="15"/>
+      <c r="G88" s="8">
+        <v>15</v>
+      </c>
+      <c r="H88" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I88" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J88" s="8" t="s">
+        <v>918</v>
+      </c>
+      <c r="K88" s="16" t="s">
+        <v>920</v>
+      </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A89" s="12"/>
-      <c r="B89" s="9"/>
-      <c r="C89" s="9"/>
-      <c r="D89" s="8"/>
+      <c r="A89" s="11" t="s">
+        <v>923</v>
+      </c>
+      <c r="B89" s="8" t="s">
+        <v>922</v>
+      </c>
+      <c r="C89" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D89" s="8">
+        <v>780</v>
+      </c>
       <c r="E89" s="8"/>
       <c r="F89" s="8"/>
-      <c r="G89" s="8"/>
-      <c r="H89" s="8"/>
-      <c r="I89" s="8"/>
-      <c r="J89" s="9"/>
-      <c r="K89" s="15"/>
+      <c r="G89" s="8">
+        <v>25</v>
+      </c>
+      <c r="H89" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I89" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J89" s="8" t="s">
+        <v>921</v>
+      </c>
+      <c r="K89" s="16" t="s">
+        <v>923</v>
+      </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A90" s="12"/>
-      <c r="B90" s="9"/>
-      <c r="C90" s="9"/>
-      <c r="D90" s="8"/>
+      <c r="A90" s="11" t="s">
+        <v>926</v>
+      </c>
+      <c r="B90" s="8" t="s">
+        <v>924</v>
+      </c>
+      <c r="C90" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D90" s="8">
+        <v>1100</v>
+      </c>
       <c r="E90" s="8"/>
       <c r="F90" s="8"/>
-      <c r="G90" s="8"/>
-      <c r="H90" s="8"/>
-      <c r="I90" s="8"/>
-      <c r="J90" s="9"/>
-      <c r="K90" s="15"/>
+      <c r="G90" s="8">
+        <v>21</v>
+      </c>
+      <c r="H90" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="I90" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J90" s="8" t="s">
+        <v>925</v>
+      </c>
+      <c r="K90" s="16" t="s">
+        <v>926</v>
+      </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A91" s="12"/>
-      <c r="B91" s="9"/>
-      <c r="C91" s="9"/>
-      <c r="D91" s="8"/>
+      <c r="A91" s="11" t="s">
+        <v>930</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>927</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D91" s="8">
+        <v>1440</v>
+      </c>
       <c r="E91" s="8"/>
       <c r="F91" s="8"/>
-      <c r="G91" s="8"/>
-      <c r="H91" s="8"/>
-      <c r="I91" s="8"/>
-      <c r="J91" s="9"/>
-      <c r="K91" s="15"/>
+      <c r="G91" s="8">
+        <v>16</v>
+      </c>
+      <c r="H91" s="8" t="s">
+        <v>928</v>
+      </c>
+      <c r="I91" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J91" s="8" t="s">
+        <v>929</v>
+      </c>
+      <c r="K91" s="16" t="s">
+        <v>930</v>
+      </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A92" s="12"/>
-      <c r="B92" s="9"/>
-      <c r="C92" s="9"/>
-      <c r="D92" s="8"/>
+      <c r="A92" s="11" t="s">
+        <v>934</v>
+      </c>
+      <c r="B92" s="8" t="s">
+        <v>931</v>
+      </c>
+      <c r="C92" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D92" s="8">
+        <v>680</v>
+      </c>
       <c r="E92" s="8"/>
       <c r="F92" s="8"/>
-      <c r="G92" s="8"/>
-      <c r="H92" s="8"/>
-      <c r="I92" s="8"/>
-      <c r="J92" s="9"/>
-      <c r="K92" s="15"/>
+      <c r="G92" s="8">
+        <v>17</v>
+      </c>
+      <c r="H92" s="8" t="s">
+        <v>932</v>
+      </c>
+      <c r="I92" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J92" s="8" t="s">
+        <v>933</v>
+      </c>
+      <c r="K92" s="16" t="s">
+        <v>934</v>
+      </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A93" s="12"/>
-      <c r="B93" s="9"/>
-      <c r="C93" s="9"/>
-      <c r="D93" s="8"/>
+      <c r="A93" s="11" t="s">
+        <v>937</v>
+      </c>
+      <c r="B93" s="8" t="s">
+        <v>935</v>
+      </c>
+      <c r="C93" s="8" t="s">
+        <v>653</v>
+      </c>
+      <c r="D93" s="8">
+        <v>900</v>
+      </c>
       <c r="E93" s="8"/>
-      <c r="F93" s="8"/>
-      <c r="G93" s="8"/>
-      <c r="H93" s="8"/>
-      <c r="I93" s="8"/>
-      <c r="J93" s="9"/>
-      <c r="K93" s="15"/>
+      <c r="F93" s="8" t="s">
+        <v>884</v>
+      </c>
+      <c r="G93" s="8">
+        <v>19</v>
+      </c>
+      <c r="H93" s="8" t="s">
+        <v>672</v>
+      </c>
+      <c r="I93" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J93" s="8" t="s">
+        <v>936</v>
+      </c>
+      <c r="K93" s="16" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A94" s="17" t="s">
+        <v>939</v>
+      </c>
+      <c r="B94" s="18" t="s">
+        <v>938</v>
+      </c>
+      <c r="C94" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D94" s="18">
+        <v>480</v>
+      </c>
+      <c r="E94" s="18"/>
+      <c r="F94" s="18"/>
+      <c r="G94" s="8">
+        <v>16</v>
+      </c>
+      <c r="H94" s="18" t="s">
+        <v>783</v>
+      </c>
+      <c r="I94" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="J94" s="18" t="s">
+        <v>940</v>
+      </c>
+      <c r="K94" s="17" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A95" s="17" t="s">
+        <v>942</v>
+      </c>
+      <c r="B95" s="18" t="s">
+        <v>941</v>
+      </c>
+      <c r="C95" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D95" s="18">
+        <v>1060</v>
+      </c>
+      <c r="E95" s="18"/>
+      <c r="F95" s="18"/>
+      <c r="G95" s="8">
+        <v>15</v>
+      </c>
+      <c r="H95" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="I95" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J95" s="18" t="s">
+        <v>943</v>
+      </c>
+      <c r="K95" s="17" t="s">
+        <v>942</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A96" s="17" t="s">
+        <v>946</v>
+      </c>
+      <c r="B96" s="18" t="s">
+        <v>944</v>
+      </c>
+      <c r="C96" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D96" s="18">
+        <v>1400</v>
+      </c>
+      <c r="E96" s="18">
+        <v>1100</v>
+      </c>
+      <c r="F96" s="18"/>
+      <c r="G96" s="8">
+        <v>25</v>
+      </c>
+      <c r="H96" s="18" t="s">
+        <v>664</v>
+      </c>
+      <c r="I96" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J96" s="18" t="s">
+        <v>945</v>
+      </c>
+      <c r="K96" s="17" t="s">
+        <v>947</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A97" s="17" t="s">
+        <v>951</v>
+      </c>
+      <c r="B97" s="18" t="s">
+        <v>948</v>
+      </c>
+      <c r="C97" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D97" s="18">
+        <v>2500</v>
+      </c>
+      <c r="E97" s="18">
+        <v>2200</v>
+      </c>
+      <c r="F97" s="18"/>
+      <c r="G97" s="8">
+        <v>15</v>
+      </c>
+      <c r="H97" s="18" t="s">
+        <v>928</v>
+      </c>
+      <c r="I97" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J97" s="18" t="s">
+        <v>949</v>
+      </c>
+      <c r="K97" s="17" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A98" s="17" t="s">
+        <v>953</v>
+      </c>
+      <c r="B98" s="18" t="s">
+        <v>952</v>
+      </c>
+      <c r="C98" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D98" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E98" s="18">
+        <v>1460</v>
+      </c>
+      <c r="F98" s="18"/>
+      <c r="G98" s="8">
+        <v>21</v>
+      </c>
+      <c r="H98" s="18" t="s">
+        <v>928</v>
+      </c>
+      <c r="I98" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J98" s="18" t="s">
+        <v>955</v>
+      </c>
+      <c r="K98" s="17" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A99" s="17" t="s">
+        <v>957</v>
+      </c>
+      <c r="B99" s="18" t="s">
+        <v>956</v>
+      </c>
+      <c r="C99" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D99" s="18">
+        <v>1650</v>
+      </c>
+      <c r="E99" s="18">
+        <v>1430</v>
+      </c>
+      <c r="F99" s="18"/>
+      <c r="G99" s="8">
+        <v>26</v>
+      </c>
+      <c r="H99" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="I99" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J99" s="18" t="s">
+        <v>959</v>
+      </c>
+      <c r="K99" s="17" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A100" s="17" t="s">
+        <v>962</v>
+      </c>
+      <c r="B100" s="18" t="s">
+        <v>960</v>
+      </c>
+      <c r="C100" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D100" s="18">
+        <v>2300</v>
+      </c>
+      <c r="E100" s="18">
+        <v>1900</v>
+      </c>
+      <c r="F100" s="18"/>
+      <c r="G100" s="8">
+        <v>17</v>
+      </c>
+      <c r="H100" s="18" t="s">
+        <v>961</v>
+      </c>
+      <c r="I100" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J100" s="18" t="s">
+        <v>964</v>
+      </c>
+      <c r="K100" s="17" t="s">
+        <v>963</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A101" s="17" t="s">
+        <v>967</v>
+      </c>
+      <c r="B101" s="18" t="s">
+        <v>965</v>
+      </c>
+      <c r="C101" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D101" s="18">
+        <v>600</v>
+      </c>
+      <c r="E101" s="18">
+        <v>400</v>
+      </c>
+      <c r="F101" s="18"/>
+      <c r="G101" s="8">
+        <v>25</v>
+      </c>
+      <c r="H101" s="18" t="s">
+        <v>966</v>
+      </c>
+      <c r="I101" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J101" s="18" t="s">
+        <v>969</v>
+      </c>
+      <c r="K101" s="17" t="s">
+        <v>968</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A102" s="17" t="s">
+        <v>972</v>
+      </c>
+      <c r="B102" s="18" t="s">
+        <v>970</v>
+      </c>
+      <c r="C102" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D102" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E102" s="18">
+        <v>1380</v>
+      </c>
+      <c r="F102" s="18"/>
+      <c r="G102" s="8">
+        <v>26</v>
+      </c>
+      <c r="H102" s="18" t="s">
+        <v>971</v>
+      </c>
+      <c r="I102" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J102" s="18" t="s">
+        <v>974</v>
+      </c>
+      <c r="K102" s="17" t="s">
+        <v>973</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A103" s="17" t="s">
+        <v>977</v>
+      </c>
+      <c r="B103" s="18" t="s">
+        <v>975</v>
+      </c>
+      <c r="C103" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D103" s="18">
+        <v>1100</v>
+      </c>
+      <c r="E103" s="18">
+        <v>840</v>
+      </c>
+      <c r="F103" s="18"/>
+      <c r="G103" s="8">
+        <v>17</v>
+      </c>
+      <c r="H103" s="18" t="s">
+        <v>976</v>
+      </c>
+      <c r="I103" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J103" s="18" t="s">
+        <v>979</v>
+      </c>
+      <c r="K103" s="17" t="s">
+        <v>978</v>
+      </c>
+    </row>
+    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A104" s="17" t="s">
+        <v>983</v>
+      </c>
+      <c r="B104" s="18" t="s">
+        <v>981</v>
+      </c>
+      <c r="C104" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D104" s="18">
+        <v>1980</v>
+      </c>
+      <c r="E104" s="18">
+        <v>1640</v>
+      </c>
+      <c r="F104" s="18"/>
+      <c r="G104" s="8">
+        <v>19</v>
+      </c>
+      <c r="H104" s="18" t="s">
+        <v>980</v>
+      </c>
+      <c r="I104" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J104" s="18" t="s">
+        <v>984</v>
+      </c>
+      <c r="K104" s="17" t="s">
+        <v>982</v>
+      </c>
+    </row>
+    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A105" s="17" t="s">
+        <v>987</v>
+      </c>
+      <c r="B105" s="18" t="s">
+        <v>985</v>
+      </c>
+      <c r="C105" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D105" s="18">
+        <v>2100</v>
+      </c>
+      <c r="E105" s="18">
+        <v>1760</v>
+      </c>
+      <c r="F105" s="18"/>
+      <c r="G105" s="8">
+        <v>25</v>
+      </c>
+      <c r="H105" s="18" t="s">
+        <v>928</v>
+      </c>
+      <c r="I105" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J105" s="18" t="s">
+        <v>986</v>
+      </c>
+      <c r="K105" s="17" t="s">
+        <v>988</v>
+      </c>
+    </row>
+    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A106" s="17" t="s">
+        <v>991</v>
+      </c>
+      <c r="B106" s="18" t="s">
+        <v>989</v>
+      </c>
+      <c r="C106" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D106" s="18">
+        <v>2100</v>
+      </c>
+      <c r="E106" s="18">
+        <v>1760</v>
+      </c>
+      <c r="F106" s="18"/>
+      <c r="G106" s="8">
+        <v>18</v>
+      </c>
+      <c r="H106" s="18" t="s">
+        <v>928</v>
+      </c>
+      <c r="I106" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J106" s="18" t="s">
+        <v>990</v>
+      </c>
+      <c r="K106" s="17" t="s">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A107" s="17" t="s">
+        <v>995</v>
+      </c>
+      <c r="B107" s="18" t="s">
+        <v>993</v>
+      </c>
+      <c r="C107" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D107" s="18">
+        <v>2200</v>
+      </c>
+      <c r="E107" s="18">
+        <v>1800</v>
+      </c>
+      <c r="F107" s="18"/>
+      <c r="G107" s="8">
+        <v>9</v>
+      </c>
+      <c r="H107" s="18" t="s">
+        <v>961</v>
+      </c>
+      <c r="I107" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J107" s="18" t="s">
+        <v>996</v>
+      </c>
+      <c r="K107" s="17" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A108" s="17" t="s">
+        <v>999</v>
+      </c>
+      <c r="B108" s="18" t="s">
+        <v>997</v>
+      </c>
+      <c r="C108" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D108" s="18">
+        <v>550</v>
+      </c>
+      <c r="E108" s="18">
+        <v>360</v>
+      </c>
+      <c r="F108" s="18"/>
+      <c r="G108" s="8">
+        <v>26</v>
+      </c>
+      <c r="H108" s="18" t="s">
+        <v>998</v>
+      </c>
+      <c r="I108" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J108" s="18" t="s">
+        <v>1001</v>
+      </c>
+      <c r="K108" s="17" t="s">
+        <v>1000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A109" s="17" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B109" s="18" t="s">
+        <v>1002</v>
+      </c>
+      <c r="C109" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D109" s="18">
+        <v>1500</v>
+      </c>
+      <c r="E109" s="18">
+        <v>1380</v>
+      </c>
+      <c r="F109" s="18"/>
+      <c r="G109" s="8">
+        <v>13</v>
+      </c>
+      <c r="H109" s="18" t="s">
+        <v>971</v>
+      </c>
+      <c r="I109" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J109" s="18" t="s">
+        <v>1003</v>
+      </c>
+      <c r="K109" s="17" t="s">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A110" s="17" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B110" s="18" t="s">
+        <v>1006</v>
+      </c>
+      <c r="C110" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D110" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E110" s="18">
+        <v>1300</v>
+      </c>
+      <c r="F110" s="18"/>
+      <c r="G110" s="8">
+        <v>18</v>
+      </c>
+      <c r="H110" s="18" t="s">
+        <v>971</v>
+      </c>
+      <c r="I110" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J110" s="18" t="s">
+        <v>1007</v>
+      </c>
+      <c r="K110" s="17" t="s">
+        <v>1009</v>
+      </c>
+    </row>
+    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A111" s="17" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B111" s="18" t="s">
+        <v>1010</v>
+      </c>
+      <c r="C111" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D111" s="18">
+        <v>2800</v>
+      </c>
+      <c r="E111" s="18">
+        <v>2500</v>
+      </c>
+      <c r="F111" s="18"/>
+      <c r="G111" s="8">
+        <v>16</v>
+      </c>
+      <c r="H111" s="18" t="s">
+        <v>928</v>
+      </c>
+      <c r="I111" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J111" s="18" t="s">
+        <v>1011</v>
+      </c>
+      <c r="K111" s="17" t="s">
+        <v>1013</v>
+      </c>
+    </row>
+    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A112" s="17"/>
+      <c r="B112" s="18"/>
+      <c r="C112" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D112" s="18"/>
+      <c r="E112" s="18"/>
+      <c r="F112" s="18"/>
+      <c r="G112" s="8"/>
+      <c r="H112" s="18"/>
+      <c r="I112" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J112" s="18"/>
+      <c r="K112" s="17"/>
+    </row>
+    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A113" s="17"/>
+      <c r="B113" s="18"/>
+      <c r="C113" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D113" s="18"/>
+      <c r="E113" s="18"/>
+      <c r="F113" s="18"/>
+      <c r="G113" s="8"/>
+      <c r="H113" s="18"/>
+      <c r="I113" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J113" s="18"/>
+      <c r="K113" s="17"/>
+    </row>
+    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A114" s="17"/>
+      <c r="B114" s="18"/>
+      <c r="C114" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D114" s="18"/>
+      <c r="E114" s="18"/>
+      <c r="F114" s="18"/>
+      <c r="G114" s="8"/>
+      <c r="H114" s="18"/>
+      <c r="I114" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J114" s="18"/>
+      <c r="K114" s="17"/>
+    </row>
+    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A115" s="17"/>
+      <c r="B115" s="18"/>
+      <c r="C115" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D115" s="18"/>
+      <c r="E115" s="18"/>
+      <c r="F115" s="18"/>
+      <c r="G115" s="8"/>
+      <c r="H115" s="18"/>
+      <c r="I115" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J115" s="18"/>
+      <c r="K115" s="17"/>
+    </row>
+    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A116" s="17"/>
+      <c r="B116" s="18"/>
+      <c r="C116" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D116" s="18"/>
+      <c r="E116" s="18"/>
+      <c r="F116" s="18"/>
+      <c r="G116" s="8"/>
+      <c r="H116" s="18"/>
+      <c r="I116" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J116" s="18"/>
+      <c r="K116" s="17"/>
+    </row>
+    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A117" s="17"/>
+      <c r="B117" s="18"/>
+      <c r="C117" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D117" s="18"/>
+      <c r="E117" s="18"/>
+      <c r="F117" s="18"/>
+      <c r="G117" s="8"/>
+      <c r="H117" s="18"/>
+      <c r="I117" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J117" s="18"/>
+      <c r="K117" s="17"/>
+    </row>
+    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A118" s="17"/>
+      <c r="B118" s="18"/>
+      <c r="C118" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D118" s="18"/>
+      <c r="E118" s="18"/>
+      <c r="F118" s="18"/>
+      <c r="G118" s="8"/>
+      <c r="H118" s="18"/>
+      <c r="I118" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J118" s="18"/>
+      <c r="K118" s="17"/>
+    </row>
+    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A119" s="17"/>
+      <c r="B119" s="18"/>
+      <c r="C119" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D119" s="18"/>
+      <c r="E119" s="18"/>
+      <c r="F119" s="18"/>
+      <c r="G119" s="8"/>
+      <c r="H119" s="18"/>
+      <c r="I119" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J119" s="18"/>
+      <c r="K119" s="17"/>
+    </row>
+    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A120" s="17"/>
+      <c r="B120" s="18"/>
+      <c r="C120" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D120" s="18"/>
+      <c r="E120" s="18"/>
+      <c r="F120" s="18"/>
+      <c r="G120" s="8"/>
+      <c r="H120" s="18"/>
+      <c r="I120" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J120" s="18"/>
+      <c r="K120" s="17"/>
+    </row>
+    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A121" s="17"/>
+      <c r="B121" s="18"/>
+      <c r="C121" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D121" s="18"/>
+      <c r="E121" s="18"/>
+      <c r="F121" s="18"/>
+      <c r="G121" s="8"/>
+      <c r="H121" s="18"/>
+      <c r="I121" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J121" s="18"/>
+      <c r="K121" s="17"/>
+    </row>
+    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A122" s="17"/>
+      <c r="B122" s="18"/>
+      <c r="C122" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D122" s="18"/>
+      <c r="E122" s="18"/>
+      <c r="F122" s="18"/>
+      <c r="G122" s="8"/>
+      <c r="H122" s="18"/>
+      <c r="I122" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J122" s="18"/>
+      <c r="K122" s="17"/>
+    </row>
+    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A123" s="17"/>
+      <c r="B123" s="18"/>
+      <c r="C123" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D123" s="18"/>
+      <c r="E123" s="18"/>
+      <c r="F123" s="18"/>
+      <c r="G123" s="8"/>
+      <c r="H123" s="18"/>
+      <c r="I123" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J123" s="18"/>
+      <c r="K123" s="17"/>
+    </row>
+    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A124" s="17"/>
+      <c r="B124" s="18"/>
+      <c r="C124" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D124" s="18"/>
+      <c r="E124" s="18"/>
+      <c r="F124" s="18"/>
+      <c r="G124" s="8"/>
+      <c r="H124" s="18"/>
+      <c r="I124" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J124" s="18"/>
+      <c r="K124" s="17"/>
+    </row>
+    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A125" s="17"/>
+      <c r="B125" s="18"/>
+      <c r="C125" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D125" s="18"/>
+      <c r="E125" s="18"/>
+      <c r="F125" s="18"/>
+      <c r="G125" s="8"/>
+      <c r="H125" s="18"/>
+      <c r="I125" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J125" s="18"/>
+      <c r="K125" s="17"/>
+    </row>
+    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A126" s="17"/>
+      <c r="B126" s="18"/>
+      <c r="C126" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D126" s="18"/>
+      <c r="E126" s="18"/>
+      <c r="F126" s="18"/>
+      <c r="G126" s="8"/>
+      <c r="H126" s="18"/>
+      <c r="I126" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J126" s="18"/>
+      <c r="K126" s="17"/>
+    </row>
+    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A127" s="17"/>
+      <c r="B127" s="18"/>
+      <c r="C127" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D127" s="18"/>
+      <c r="E127" s="18"/>
+      <c r="F127" s="18"/>
+      <c r="G127" s="8"/>
+      <c r="H127" s="18"/>
+      <c r="I127" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J127" s="18"/>
+      <c r="K127" s="17"/>
+    </row>
+    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A128" s="17"/>
+      <c r="B128" s="18"/>
+      <c r="C128" s="18"/>
+      <c r="D128" s="18"/>
+      <c r="E128" s="18"/>
+      <c r="F128" s="18"/>
+      <c r="G128" s="8"/>
+      <c r="H128" s="18"/>
+      <c r="I128" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J128" s="18"/>
+      <c r="K128" s="17"/>
+    </row>
+    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A129" s="17"/>
+      <c r="B129" s="18"/>
+      <c r="C129" s="18"/>
+      <c r="D129" s="18"/>
+      <c r="E129" s="18"/>
+      <c r="F129" s="18"/>
+      <c r="G129" s="8"/>
+      <c r="H129" s="18"/>
+      <c r="I129" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J129" s="18"/>
+      <c r="K129" s="17"/>
+    </row>
+    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A130" s="17"/>
+      <c r="B130" s="18"/>
+      <c r="C130" s="18"/>
+      <c r="D130" s="18"/>
+      <c r="E130" s="18"/>
+      <c r="F130" s="18"/>
+      <c r="G130" s="8"/>
+      <c r="H130" s="18"/>
+      <c r="I130" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J130" s="18"/>
+      <c r="K130" s="17"/>
+    </row>
+    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A131" s="17"/>
+      <c r="B131" s="18"/>
+      <c r="C131" s="18"/>
+      <c r="D131" s="18"/>
+      <c r="E131" s="18"/>
+      <c r="F131" s="18"/>
+      <c r="G131" s="8"/>
+      <c r="H131" s="18"/>
+      <c r="I131" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J131" s="18"/>
+      <c r="K131" s="17"/>
+    </row>
+    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A132" s="17"/>
+      <c r="B132" s="18"/>
+      <c r="C132" s="18"/>
+      <c r="D132" s="18"/>
+      <c r="E132" s="18"/>
+      <c r="F132" s="18"/>
+      <c r="G132" s="8"/>
+      <c r="H132" s="18"/>
+      <c r="I132" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J132" s="18"/>
+      <c r="K132" s="17"/>
+    </row>
+    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A133" s="17"/>
+      <c r="B133" s="18"/>
+      <c r="C133" s="18"/>
+      <c r="D133" s="18"/>
+      <c r="E133" s="18"/>
+      <c r="F133" s="18"/>
+      <c r="G133" s="8"/>
+      <c r="H133" s="18"/>
+      <c r="I133" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J133" s="18"/>
+      <c r="K133" s="17"/>
+    </row>
+    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A134" s="17"/>
+      <c r="B134" s="18"/>
+      <c r="C134" s="18"/>
+      <c r="D134" s="18"/>
+      <c r="E134" s="18"/>
+      <c r="F134" s="18"/>
+      <c r="G134" s="8"/>
+      <c r="H134" s="18"/>
+      <c r="I134" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J134" s="18"/>
+      <c r="K134" s="17"/>
+    </row>
+    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A135" s="17"/>
+      <c r="B135" s="18"/>
+      <c r="C135" s="18"/>
+      <c r="D135" s="18"/>
+      <c r="E135" s="18"/>
+      <c r="F135" s="18"/>
+      <c r="G135" s="8"/>
+      <c r="H135" s="18"/>
+      <c r="I135" s="18" t="s">
+        <v>657</v>
+      </c>
+      <c r="J135" s="18"/>
+      <c r="K135" s="17"/>
+    </row>
+    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G136" s="8"/>
+    </row>
+    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G137" s="8"/>
+    </row>
+    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G138" s="8"/>
+    </row>
+    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G139" s="8"/>
+    </row>
+    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G140" s="8"/>
+    </row>
+    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G141" s="8"/>
+    </row>
+    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G142" s="8"/>
+    </row>
+    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G143" s="8"/>
+    </row>
+    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G144" s="8"/>
+    </row>
+    <row r="145" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G145" s="8"/>
+    </row>
+    <row r="146" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G146" s="8"/>
+    </row>
+    <row r="147" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G147" s="8"/>
+    </row>
+    <row r="148" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G148" s="8"/>
+    </row>
+    <row r="149" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G149" s="8"/>
+    </row>
+    <row r="150" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G150" s="8"/>
+    </row>
+    <row r="151" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G151" s="8"/>
+    </row>
+    <row r="152" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G152" s="8"/>
+    </row>
+    <row r="153" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G153" s="8"/>
+    </row>
+    <row r="154" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G154" s="8"/>
+    </row>
+    <row r="155" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G155" s="8"/>
+    </row>
+    <row r="156" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G156" s="8"/>
+    </row>
+    <row r="157" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G157" s="8"/>
+    </row>
+    <row r="158" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="G158" s="8"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:K93" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="G2:G93">
+    <cfRule type="cellIs" dxfId="23" priority="22" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="23" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="21" priority="24" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G94">
+    <cfRule type="cellIs" dxfId="20" priority="19" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="20" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="21" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G95">
+    <cfRule type="cellIs" dxfId="17" priority="16" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="16" priority="17" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G96">
+    <cfRule type="cellIs" dxfId="14" priority="13" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="13" priority="14" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="15" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G97">
+    <cfRule type="cellIs" dxfId="11" priority="10" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="11" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="12" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G98">
+    <cfRule type="cellIs" dxfId="8" priority="7" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="8" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="9" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G99:G113">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="lessThan">
+      <formula>20</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="greaterThanOrEqual">
+      <formula>20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G114:G158">
     <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>

</xml_diff>

<commit_message>
feat: background-free photos for all catalog products
- generate rembg cutouts for every product (79/80, id 508 has no
  photo) via backend/scripts/make_cutouts.py: trimmed, <=900px WebP,
  filename-safe ids (product "700\703\706\708\711" got sanitized name)
- shared lib/cutouts.ts helper (cutoutName/cutoutSrc) used by home
  page, product detail, cards, brands and chat
- ProductCard/BrandsSection/ChatBubble now load /cutouts/<id>.webp
  first and fall back to the original photo, then placeholder
- category tiles and hero pick cutouts for all four categories
  (Сироватка tile no longer shows a rectangular photo)
- refresh shots/ (errors: 0)
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B16B6B9B-0AC8-4E74-847B-DDFC89E7B5DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE93772-918F-4498-B0F6-AC4F610BE092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-1512" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Зручна таблиця" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2291" uniqueCount="1014">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2296" uniqueCount="1018">
   <si>
     <t>Артикул</t>
   </si>
@@ -6761,6 +6761,49 @@
   </si>
   <si>
     <t>731-1(1)</t>
+  </si>
+  <si>
+    <t>Вдосконалювальний Пептидний крем для періорбітальної зони очей 100 мл</t>
+  </si>
+  <si>
+    <t>✨ Advanced Peptide Eye Cream – технологія “рідких пептидів” для сяючого погляду! ✨
+🌿 Інноваційна формула для делікатної зони навколо очей:
+💎 Ефективно розгладжує тонкі лінії та зморшки
+⚡ Забезпечує миттєвий ліфтинг та моделювання контуру
+🌸 Синхронізує природні процеси відновлення шкіри
+🛡️ Запобігає антиоксидантному стресу
+🚀 Потужні провідникові системи доставляють активні комплекси безпосередньо до клітин
+💚 Результат – свіжий, молодий та сяючий погляд щодня!
+📌 Показання:
+Фото- та хроностаріння
+Зморшки та знижений тонус шкіри
+Гіперпігментація
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Активні компоненти:
+🌱 Декапептиди та олігопептиди – стимуляція синтезу колагену
+💧 Гіалуронат натрію – глибоке зволоження
+🥭 Олія манго та макадамії – живлення та відновлення бар’єру
+🌊 Екстракт фукуса – антиоксидантний захист
+⚡ Аргирелін та нанопептиди – зменшення мімічних зморшок
+🌸 Shadownyl та Agefinity – освітлення та ревіталізація
+🛡️ ПДРН та Inoveol EGCG – регенерація та захист
+📌 Спосіб використання:  
+Нанести невелику кількість крему на чисту шкіру навколо очей. Використовувати щодня вранці та ввечері.
+✔️ Характеристики продукту:
+Тип: Пептидний крем для періорбітальної зони
+Об’єм: 100 мл
+Призначення: Ліфтинг, омолодження, освітлення, зволоження
+Тип шкіри: Чутлива, суха, зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Advanced Peptide Eye Cream – твій must-have для сяючого та молодого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>733</t>
+  </si>
+  <si>
+    <t>733(1)</t>
   </si>
 </sst>
 </file>
@@ -10885,21 +10928,37 @@
       </c>
     </row>
     <row r="112" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A112" s="17"/>
-      <c r="B112" s="18"/>
+      <c r="A112" s="17" t="s">
+        <v>1016</v>
+      </c>
+      <c r="B112" s="18" t="s">
+        <v>1014</v>
+      </c>
       <c r="C112" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D112" s="18"/>
-      <c r="E112" s="18"/>
+      <c r="D112" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E112" s="18">
+        <v>1380</v>
+      </c>
       <c r="F112" s="18"/>
-      <c r="G112" s="8"/>
-      <c r="H112" s="18"/>
+      <c r="G112" s="8">
+        <v>18</v>
+      </c>
+      <c r="H112" s="18" t="s">
+        <v>29</v>
+      </c>
       <c r="I112" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J112" s="18"/>
-      <c r="K112" s="17"/>
+      <c r="J112" s="18" t="s">
+        <v>1015</v>
+      </c>
+      <c r="K112" s="17" t="s">
+        <v>1017</v>
+      </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A113" s="17"/>

</xml_diff>

<commit_message>
﻿feat: automatic cutout generation for new products
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BE93772-918F-4498-B0F6-AC4F610BE092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B311886-7D53-48F6-8509-F47A02FF9192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-1512" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,8 +19,17 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Зручна таблиця'!$A$1:$K$93</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -29,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2296" uniqueCount="1018">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2421" uniqueCount="1101">
   <si>
     <t>Артикул</t>
   </si>
@@ -6804,6 +6813,790 @@
   </si>
   <si>
     <t>733(1)</t>
+  </si>
+  <si>
+    <t>Омолоджуюча маска "Едельвейс" 300 мл</t>
+  </si>
+  <si>
+    <t>✨ Edelweiss Stem Cell Mask – інтелектуальне омолодження! ✨
+🌿 Концентрована формула зі стовбуровими клітинами едельвейсу:
+💎 Розгладжує тонкі лінії та зморшки
+🌸 Забезпечує виражений ліфтинг-ефект
+💧 Стимулює оновлення клітин та підтримує їх структуру
+🛡️ Зміцнює дерма-епідермальне сполучення
+🌟 Має потужну цитопротекторну дію
+💚 Результат – пружна, сяюча та оновлена шкіра з ефектом перетворення!
+📌 Показання:
+Фото- та хроностаріння
+Зморшки та тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Профілактика біостаріння
+Догляд після інвазивних процедур
+📌 Активні компоненти:
+🌱 PhytoStem Cells Edelweiss – стовбурові клітини едельвейсу для омолодження
+🌸 Екстракт Ambiaty – регенерація та захист
+💧 Гіалуронат натрію – глибоке зволоження
+🌿 ПДРН – стимуляція відновлення клітин
+🌺 Alpine Rose Active та екстракт рису – антиоксидантний захист та ревіталізація
+📌 Спосіб використання:  
+Нанести маску на чисту шкіру обличчя, залишити на 10–15 хвилин, після чого змити теплою водою. Використовувати 1–2 рази на тиждень.
+✔️ Характеристики продукту:
+Тип: Омолоджуюча концентрована маска
+Об’єм: 300 мл
+Призначення: Ліфтинг, омолодження, освітлення, зволоження, захист
+Тип шкіри: Зріла, суха, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Edelweiss Stem Cell Mask – твій must-have для миттєвого омолодження та сяючої шкіри!</t>
+  </si>
+  <si>
+    <t>736</t>
+  </si>
+  <si>
+    <t>736(1)</t>
+  </si>
+  <si>
+    <t>Хронобіологічний енергетичний ліфтінг-крем 230 мл</t>
+  </si>
+  <si>
+    <t>✨ ChronoBio Energy Lifting Cream – нічне перезавантаження для твоєї шкіри! ✨
+🌙 Інноваційна хронобіологічна формула з комплексами Chronodyn та DermCom:
+⚡ Максимально стимулює енергообмін у клітинах
+💎 Забезпечує активне відновлення та видимий ліфтинг обличчя, шиї та підборіддя
+🌸 Усуває обвисання та в’ялість (птоз)
+💧 Підвищує пружність і відновлює тонус
+🛡️ Захищає від фото- та хроностаріння
+💚 Результат – підтягнута, сяюча та енергійна шкіра щоранку!
+📌 Показання до застосування:
+Уповільнення старіння без радикальних методів
+Запобігання динамічним та статичним зморшкам
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус та вікова шкіра
+Догляд після інвазивних процедур
+📌 Ключові активні компоненти:
+🌱 Chronodyn + DermCom – стимуляція клітинного обміну та регенерації
+🥥 Олії сезаму, пасіфлори, моної де Таїті – живлення та відновлення бар’єру
+💧 Гіалуронат натрію + Hyaluronic Filling Spheres™ – глибоке зволоження та заповнення зморшок
+🌸 Juveleven™ peptide solution, Replexium, Agefinity™ – омолодження та ревіталізація
+🌿 Фукогель, екстракт цикорію, камедь акації – тонізація та захист
+⚡ Кофеїн та сквален – енергія та антиоксидантний захист
+📌 Спосіб використання:  
+Нанести крем на очищену шкіру обличчя, шиї та підборіддя перед сном. Використовувати регулярно для максимального ефекту ліфтингу та відновлення.
+✔️ Характеристики продукту:
+Тип: Нічний хронобіологічний ліфтинг-крем
+Об’єм: 230 мл
+Призначення: Ліфтинг, омолодження, відновлення тонусу, зволоження
+Тип шкіри: Зріла, суха, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 ChronoBio Energy Lifting Cream – твій must-have для нічного відновлення та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>708-1</t>
+  </si>
+  <si>
+    <t>708-1(1)</t>
+  </si>
+  <si>
+    <t>Передовий денний крем SPF 30 Золоті водорості  230 мл</t>
+  </si>
+  <si>
+    <t>✨ Golden Algae Day Cream SPF 30 – щоденний захист та омолодження! ✨
+🌿 Інноваційна антиоксидантна формула:
+☀️ UVA/UVB-фільтри – надійний захист від сонця та фотостаріння
+🌸 Екстракт золотих водоростей – потужна антиоксидантна дія та відновлення клітин
+💎 Пептидний комплекс – реструктуризація та зміцнення шкіри
+💧 Гіалуронова кислота та олія жожоба – миттєве зволоження та пружність
+💚 Результат – рівний тон, захист від зморшок та сяюча шкіра щодня!
+📌 Основні ефекти:
+Миттєве зволоження та підвищення пружності
+Запобігання динамічним та статичним зморшкам
+Захист від фотостаріння
+Вирівнювання тону обличчя
+Підвищення тонусу вікової шкіри
+📌 Показання:
+Щоденний догляд за віковою шкірою
+Фото- та хроностаріння
+Гіперпігментація та тьмяний колір обличчя
+Догляд після інвазивних процедур та контурної пластики
+📌 Ключові компоненти:
+🌺 ANTILEUKINE™ 6 (екстракт золотих водоростей) – антиоксидантний захист
+🌱 Пептиди (Argireline®, Replexium, Marine Filling Spheres™) – омолодження та ліфтинг
+💧 Hydagen® Aquaporin, гіалуронова кислота – глибоке зволоження
+🥥 Олії жожоба, ши та женьшеня – живлення та відновлення
+🌸 Agefinity™, Sensityl™ – ревіталізація та захист від стресу
+📌 Спосіб використання:  
+Нанести крем на очищену шкіру обличчя щоранку. Рівномірно розподілити по всій поверхні, уникаючи зони навколо очей.
+✔️ Характеристики продукту:
+Тип: Антиоксидантний денний крем з SPF
+Об’єм: 230 мл
+Призначення: Захист SPF 30, омолодження, зволоження, вирівнювання тону
+Тип шкіри: Чутлива, суха, комбінована, вікова
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Golden Algae Day Cream SPF 30 – твій must-have для щоденного захисту та сяйва! 🌟</t>
+  </si>
+  <si>
+    <t>707</t>
+  </si>
+  <si>
+    <t>707(1)</t>
+  </si>
+  <si>
+    <t>Заповнювальна маска-біоміметик з вітаміном С</t>
+  </si>
+  <si>
+    <t>✨ Biomimetic Vitamin C Mask – інноваційне омолодження та сяйво! ✨
+🌿 Ультрасучасна формула з багатоформним вітаміном С та 8 пептидами:
+💎 Помітно омолоджує та коригує всі прояви вікових змін
+🌸 Освітлює пігментні плями та вирівнює тон
+💧 Інтенсивно зволожує завдяки гіалуроновій кислоті
+🛡️ Глибоко ревіталізує та відновлює структуру шкіри
+🌟 Пом’якшує видимість ліній і зморшок
+💚 Результат – гладка, сяюча та оновлена шкіра з ефектом перетворення!
+📌 Показання до застосування:
+Щоденний догляд для уповільнення старіння
+Запобігання динамічним та статичним зморшкам
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Догляд після інвазивних процедур
+📌 Ключові активні компоненти:
+☀️ Вітамін С у кількох формах – антиоксидантний захист та освітлення
+🌱 8 пептидів (Replexium, Juveleven™, Collalift® 18 та ін.) – стимуляція синтезу колагену та омолодження
+💧 Гіалуронат натрію + Hyaluronic Filling Spheres™ – глибоке зволоження та заповнення зморшок
+🌸 Ceramosides™ Hp та олія насіння квітки Алтеї – відновлення бар’єру та захист від втрати вологи
+⚡ Agefinity™, Easyliance, Collamung® Onp – ревіталізація та ліфтинг
+🌿 Екстракт цикорію, амінокислоти (лізин, серин, валін), пантенол – живлення та відновлення
+📌 Спосіб використання:  
+Нанести маску на очищену шкіру обличчя, залишити на 10–15 хвилин, після чого змити теплою водою. Використовувати 1–2 рази на тиждень.
+✔️ Характеристики продукту:
+Тип: Заповнювальна маска-біоміметик
+Об’єм: 50 мл
+Призначення: Омолодження, освітлення, ревіталізація, зволоження
+Тип шкіри: Зріла, суха, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Biomimetic Vitamin C Mask – твій must-have для сяючої та молодої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>713</t>
+  </si>
+  <si>
+    <t>713(1)</t>
+  </si>
+  <si>
+    <t>Реструктурирующая маска для зони навколо очей з екстрактом кави арабіка Smart4Derma Arabica eye mask contour relief 100 мл</t>
+  </si>
+  <si>
+    <t>710(1)</t>
+  </si>
+  <si>
+    <t>710</t>
+  </si>
+  <si>
+    <t>Енерго-генеруючий бустер «Золоті водорослі» Smart4Derma Booster-Elixir Golden Seaweed 10 мл</t>
+  </si>
+  <si>
+    <t>✨ Golden Seaweed Booster – трансдермальна енергія молодості! ✨
+🌿 Інноваційна формула з екстрактом золотих водоростей:
+⚡ Активує мітохондріальний енергообмін у клітинах
+💎 Підвищує реструктуризацію шкірного матриксу
+🌸 Зміцнює дермо-епідермальне з’єднання
+💧 Зменшує пігментні плями та гусячі лапки
+🌟 Розгладжує зморшки в Y-зоні шиї
+💚 Результат – підтягнута, сяюча та оновлена шкіра без ознак втоми!
+📌 Показання до застосування:
+Щоденний догляд для уповільнення старіння
+Профілактика зморшок
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація та знижений тонус
+Вікова шкіра
+Відновлення після інвазивних процедур
+📌 Ключові активні компоненти:
+🌺 Екстракт золотих водоростей (ANTILEUKINE™) – антиоксидантний захист та омолодження
+🌱 Екстракти червоних та японських водоростей, зеленого чаю – ревіталізація та тонізація
+💧 Гіалуронат натрію + Hydagen® Aquaporin – глибоке зволоження
+⚡ Пептиди (Replexium, Agefinity™, Juveleven™, Argireline®) – стимуляція синтезу колагену та ліфтинг
+🌿 ПДРН, біотин трипептид-1, олігопептиди, деекапептид-9 – регенерація та відновлення
+🌸 Амінокислоти (лізин, серин, валін) + пантенол – живлення та захист
+📌 Спосіб використання:  
+Нанести кілька крапель бустера на очищену шкіру обличчя та шиї. Використовувати щодня перед нанесенням крему.
+✔️ Характеристики продукту:
+Тип: Трансдермальний бустер-еліксир
+Об’єм: 30 мл / 50 мл (залежно від упаковки)
+Призначення: Омолодження, освітлення, ліфтинг, зволоження
+Тип шкіри: Зріла, суха, комбінована
+Бренд: Smart Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Golden Seaweed Booster – твій must-have для інтенсивної боротьби зі старінням та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>705</t>
+  </si>
+  <si>
+    <t>705(1)</t>
+  </si>
+  <si>
+    <t>Интеллектуальный заполнительный Гидромист 500 мл</t>
+  </si>
+  <si>
+    <t>✨ Інтелектуальний Гідроміст – багатофункціональне зволоження та anti-age догляд! ✨
+🌿 Формула для інтенсивного відновлення:
+💧 Миттєве та тривале зволоження
+🌸 Нормалізація pH та вирівнювання тону шкіри
+💎 Зменшення глибини зморшок та профілактика їх появи
+🛡️ Захист від сухості та еритеми
+🌟 Ефект сяйва зсередини
+💚 Результат – свіжа, гладка та сяюча шкіра щодня!
+📌 Ключові переваги:
+Морський інгредієнт Antarcticine® з криопротекторними властивостями
+💧 Гіалуронат натрію – глибоке зволоження
+🌱 Hydagen® Aquaporin, SPAR'AGE™, морські мінерали, амінокислоти, пантенол – живлення, захист та відновлення
+📌 Показання до застосування:
+Щоденний догляд за віковою шкірою
+Профілактика старіння
+Відновлення після косметологічних процедур
+Борьба з гіперпігментацією та зниженим тонусом
+✔️ Характеристики продукту:
+Тип: Інтелектуальний заповнювальний гідроміст
+Об’єм: 500 мл
+Призначення: Зволоження, омолодження, освітлення, захист
+Тип шкіри: Всі типи, особливо суха та зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Intelligent HydroMist – твій must-have для сяючої та зволоженої шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>702</t>
+  </si>
+  <si>
+    <t>702(1)</t>
+  </si>
+  <si>
+    <t>Гель для вмивання "Активатор Енергії" з кислотами 500 мл</t>
+  </si>
+  <si>
+    <t>701</t>
+  </si>
+  <si>
+    <t>701(1)</t>
+  </si>
+  <si>
+    <t>✨ Energy Activator Cleansing Gel – перезарядка для твоєї шкіри! ✨
+🌿 Інноваційна формула з кислотами та ензимами:
+⚡ Перезаряджає клітини шкіри на 27%
+💧 Відновлює pH-баланс та підтримує оптимальний рівень зволоження
+🌸 Комплекс із трьох кислот у розчині електролітів – м’яке, але ефективне очищення
+🛡️ Компонент OXY 229 PF активує мітохондріальне дихання для енергії клітин
+💎 Дарує свіжість, сяйво та рівний тон
+💚 Результат – чиста, енергійна та сяюча шкіра після кожного вмивання!
+📌 Ключові активні компоненти:
+🌱 Гліколева, піруватна та ферулова кислоти – ексфоліація та вирівнювання тону
+⚡ OXY 229 PF – активація клітинної енергії
+💧 Гіалуронат натрію, сечовина, Д-пантенол – глибоке зволоження та відновлення
+🌸 Екстракт гібіскуса, морські мінерали – антиоксидантний захист та тонізація
+🌟 Hydagen® Aquaporin, Lys'lastine™ V, Perlaura® – підтримка водного балансу та пружності
+🧬 Амінокислоти (аргінін, лізин, серин) – живлення та регенерація
+📌 Показання до застосування:
+Уповільнення старіння без радикальних методів
+Запобігання появі зморшок
+Фото- та хроностаріння
+Тьмяний колір обличчя
+Гіперпігментація
+Знижений тонус шкіри
+Догляд після інвазивних процедур
+📌 Як застосовувати:  
+Нанести невелику кількість гелю на вологу шкіру, розподілити по масажних лініях, легко промасажувати та змити теплою водою. Використовувати щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Інноваційний гель для вмивання
+Об’єм: 500 мл
+Призначення: Очищення, омолодження, відновлення енергії клітин
+Тип шкіри: Вікова, комбінована, проблемна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Energy Activator Cleansing Gel – твій must-have для щоденного енергетичного догляду! 🌟</t>
+  </si>
+  <si>
+    <t>Розкішний живильний крем з церамідами 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Luxury Ceramide Cream – глибоке живлення та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+💧 Технологія подвійного зволоження – миттєвий та тривалий ефект
+🌸 Церамиди – зміцнення захисного бар’єру шкіри
+🥥 Комплекс Multifeel – інтенсивне живлення та відновлення
+🌟 Пантенол – заспокоює та регенерує
+💎 Бореться з проявами старіння, зменшує глибину зморшок
+💚 Результат – гладка, сяюча та здорова шкіра щодня!
+📌 Підходить для:
+Всі типи шкіри
+Суха та зневоднена шкіра
+Зріла та чутлива шкіра
+Відновлення після косметичних процедур
+✔️ Характеристики продукту:
+Тип: Живильний крем з церамідами
+Об’єм: 50 мл / 100 мл / 230 мл (залежно від упаковки)
+Призначення: Зволоження, живлення, відновлення, омолодження
+Тип шкіри: Всі типи, особливо суха та зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Ceramide Cream – твій must-have для глибокого живлення та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>522</t>
+  </si>
+  <si>
+    <t>522(1)</t>
+  </si>
+  <si>
+    <t>Невагомий Крем-гель SPF 50 - 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Weightless SPF 50 Gel-Cream – щоденний захист та комфорт! ✨
+🌿 Інноваційна формула для щоденного догляду:
+☀️ Потужний УФ-захист: комплекс PolyFructol Plus та X50 Skin Barrier запобігає фотостарінню та передчасним зморшкам
+💧 Глибоке зволоження: технологія PatcH2O та Hydagen® Aquaporine працюють на клітинному рівні
+🛡️ Антиоксидантний захист: DN-Age нейтралізує вільні радикали та стрес
+🌸 Легка текстура: миттєво вбирається без липкості, даруючи комфорт
+💚 Результат – пружна, гладка та захищена шкіра з ефектом свіжості після кожного нанесення!
+📌 Показання до застосування:
+Щоденний догляд для всіх типів шкіри
+Захист від фото- та хроностаріння
+Профілактика зморшок та пігментації
+Зволоження та підтримка клітинного балансу
+📌 Як застосовувати:  
+Наносити на чисту, суху шкіру обличчя за 20 хвилин до виходу на сонце. Використовувати щодня для максимального захисту.
+✔️ Характеристики продукту:
+Тип: Крем-гель з SPF
+Об’єм: 50 мл / 230 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Всі типи
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Weightless SPF 50 Gel-Cream – твій must-have для щоденного захисту та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>523</t>
+  </si>
+  <si>
+    <t>523(1)</t>
+  </si>
+  <si>
+    <t>Сонцезахисний ультразволожувальний крем SPF50 з олією канабісу 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Cannabis Ultra-Hydrating Sunscreen SPF 50 – повний спектр захисту та сяйво! ✨
+🌿 Інноваційна формула для щоденного догляду:
+☀️ SPF50 + широкоспектральний UVA/UVB-захист – профілактика фотостаріння та збереження колагену
+💧 Гіалуронова кислота + PolyFructol Plus – глибоке зволоження та підтримка водного балансу
+🌸 Екстракт азіатської центелли – заспокоює та відновлює бар’єрні функції
+🛡️ Токоферол ацетат та аскорбіл глюкозид – антиоксидантний захист від стресу та вільних радикалів
+🌟 Легка текстура з матуючим ефектом – без відчуття тяжкості
+💚 Результат – пружна, сяюча та захищена шкіра щодня!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Перші ознаки старіння
+Зниження бар’єрної функції
+📌 Спосіб застосування:  
+Наносити на очищену шкіру обличчя вранці, за 20 хвилин до виходу на сонце. Використовувати щодня для максимального ефекту.
+✔️ Характеристики продукту:
+Тип: Сонцезахисний крем з SPF
+Об’єм: 230 мл
+Рівень захисту: SPF 50+ PA++++
+Призначення: Захист, зволоження, антиоксидантний догляд
+Тип шкіри: Суха, чутлива, зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Cannabis Ultra-Hydrating Sunscreen SPF 50 – твій must-have для щоденного захисту та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>516</t>
+  </si>
+  <si>
+    <t>516(1)</t>
+  </si>
+  <si>
+    <t>Крем-маска глибоке зволоження 300 мл</t>
+  </si>
+  <si>
+    <t>✨ Deep Moisture Cream-Mask – миттєве та пролонговане зволоження! ✨
+🌿 Легка пептидна формула з системою доставки X50:
+💧 Створює депо вологи в шкірі для подвійного ефекту гідратації
+🌸 Відновлює бар’єрні функції завдяки комплексу церамідів
+🛡️ Заспокоює подразнення та зменшує сухість
+⚡ Підвищує тонус та еластичність шкіри
+🌟 Дарує свіжість і сяйво вже після першого застосування
+💚 Результат – шкіра стає пружною, гладкою та сяючою!
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист шкіри
+📌 Ключові активні компоненти:
+💧 Hydagen® Aquaporin, гіалуронат натрію, PolyFructol Plus – інтенсивне зволоження
+🌱 Олія авокадо, примули, екстракт центелли – живлення та відновлення
+🌸 Д-пантенол, ніацинамід, бета-глюкан – заспокійливий та регенеруючий ефект
+🛡️ iActive Ceramide, X50 Skin Barrier, токоферол, ферулова кислота, убіхінон – антиоксидантний захист та зміцнення бар’єру
+⚡ Амінокислоти та магнезіум аскорбіл фосфат – стимуляція клітинного оновлення
+✔️ Характеристики продукту:
+Тип: Крем-маска для глибокого зволоження
+Об’єм: 300 мл
+Призначення: Зволоження, живлення, відновлення, антиоксидантний захист
+Тип шкіри: Суха, чутлива, зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Deep Moisture Cream-Mask – твій must-have для миттєвого та тривалого зволоження! 🌟</t>
+  </si>
+  <si>
+    <t>513</t>
+  </si>
+  <si>
+    <t>513(1)</t>
+  </si>
+  <si>
+    <t>Зволожувальний дренажний крем від темних кіл та набряків 100 мл</t>
+  </si>
+  <si>
+    <t>✨ Drainage Moisturizing Eye Cream – сяючий та відпочилий погляд! ✨
+🌿 Активна формула для зони навколо очей:
+💧 Інтенсивне зволоження та відновлення бар’єрної функції
+🌸 Освітлення темних кіл завдяки екстракту водоростей
+🛡️ Зменшення набряків завдяки рутину та ескуліну
+⚡ Комплекс інкапсульованих пептидів – стимуляція синтезу білків для пружності
+🌟 Живлення та захист завдяки олії авокадо та примули
+💚 Результат – світліший тон, менші набряки та пружна шкіра навколо очей!
+📌 Активні компоненти:
+🌱 Екстракт водоростей – покращує кровообіг та освітлює темні кола
+🌸 Рутин + ескулін – протинабрякова дія
+💧 Інулін – підвищує пружність та еластичність
+⚡ Інкапсульовані пептиди – стимулюють синтез кератину, філагрину та лорекину
+🥑 Олія авокадо та примули вечірньої – живлення та захист
+🌟 Токоферол + магнезіум аскорбіл фосфат – антиоксидантний щит
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Зволожувальний дренажний крем для очей
+Об’єм: 100 мл
+Призначення: Зволоження, протинабрякова дія, освітлення темних кіл
+Тип шкіри: Суха, чутлива, зріла
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Drainage Moisturizing Eye Cream – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>507</t>
+  </si>
+  <si>
+    <t>507(1)</t>
+  </si>
+  <si>
+    <t>Дренажна освітлююча маска Глабрідин для очей 100 мл Smart 4 Derma</t>
+  </si>
+  <si>
+    <t>✨ Glabridin Eye Drainage Mask – професійний догляд для сяючого погляду! ✨
+🌿 Інноваційна формула для переорбітальної зони:
+💎 Зміцнює судини та покращує мікроциркуляцію
+⚡ Активізує виведення заліза та білірубіну, зменшуючи тьмяність
+🌸 Освітлює шкіру та зменшує набряки нижніх повік
+💧 Забезпечує глибоке зволоження та підвищує еластичність
+🛡️ Відновлює бар’єрну функцію шкіри
+💚 Результат – свіжий, відпочилий та сяючий погляд!
+📌 Показання до застосування:
+Суха та чутлива шкіра навколо очей
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист
+📌 Активні компоненти:
+🌱 Shadownyl, Рутин, Ескулін – зміцнення судин та протинабрякова дія
+🌸 Inoveol EGCG, екстракти зеленого чаю та каштана – антиоксидантний захист та покращення кровообігу
+💧 PolyFructol Plus, Hydagen® Aquaporin, інулін – глибоке зволоження та підтримка водного балансу
+🛡️ X50® Skin Barrier та комплекс пептидів – стимуляція синтезу кератину та філагрину, відновлення бар’єру
+✔️ Характеристики продукту:
+Тип: Дренажна освітлююча маска для очей
+Об’єм: 100 мл
+Призначення: Зволоження, освітлення, протинабрякова дія, відновлення
+Бренд: Smart4Derma (🇺🇦 Україна + 🇩🇪 Німеччина)
+🌟 Glabridin Eye Mask – твій must-have для сяючого та відпочилого погляду! 🌟</t>
+  </si>
+  <si>
+    <t>511(1)</t>
+  </si>
+  <si>
+    <t>511</t>
+  </si>
+  <si>
+    <t>Зволожуючий гель-тонер для сіяння шкіри 500 мл</t>
+  </si>
+  <si>
+    <t>✨ Polyfructol Toner Bright Skin – професійне сяйво та зволоження! ✨
+🌿 Інноваційна формула для атонічної та зневодненої шкіри:
+💧 Hydagen® Aquaporin + PatcH2O – інтенсивне зволоження та утримання вологи
+🌸 Екстракти ромашки та шавлії – заспокоюють, знімають почервоніння та дискомфорт
+🌟 Ніацинамід – вирівнює тон та додає природне сяйво
+🛡️ Puricare POE LS 9727 + PolyFructol Plus – захист від негативного впливу навколишнього середовища
+⚡ Д-пантенол та натрій гіалуронат – пружність та відчуття свіжості
+💚 Результат – тривале зволоження до 24 годин, свіжий вигляд та сяюча шкіра!
+📌 Результати використання:
+Тривале зволоження на 24 години
+Свіжий та сяючий вигляд шкіри
+Активація процесів оновлення клітин та синтезу колагену
+Захист та покращення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Зволожуючий гель-тонер
+Об’єм: 500 мл
+Призначення: Зволоження, сяйво, захист
+Тип шкіри: Суха, тьмяна, атонічна
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Polyfructol Toner Bright Skin – твій must-have для сяючої та зволоженої шкіри щодня! 🌟</t>
+  </si>
+  <si>
+    <t>502</t>
+  </si>
+  <si>
+    <t>502(1)</t>
+  </si>
+  <si>
+    <t>Smart4Derma Шовкова ензимна пудра з гранулами жожоба 120 г</t>
+  </si>
+  <si>
+    <t>✨ Silk Enzyme Powder – делікатне очищення та сяйво! ✨
+🌿 Унікальна формула для щоденного догляду:
+💎 Ензими ефективно видаляють забруднення та відмерлі клітини
+🌸 Гранули олії жожоба м’яко відлущують, не травмуючи шкіру
+💧 Центелла азіатська покращує текстуру та еластичність
+🛡️ Трегалоза, алантоїн та екстракт ромашки – зволоження та заспокійливий ефект
+🌟 Створює захисну плівку, підтримуючи гідроліпідний баланс
+💚 Результат – чиста, гладка та сяюча шкіра без подразнень!
+📌 Основні переваги:
+Очищення та вирівнювання тону
+Підтримка природного балансу вологи
+Заспокійливий ефект при запаленнях
+Захист від зовнішніх факторів
+✔️ Характеристики продукту:
+Тип: Ензимна пудра для очищення
+Об’єм: 100–120 г (залежно від упаковки)
+Призначення: Очищення, відлущування, зволоження, захист
+Тип шкіри: Чутлива, комбінована, суха
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Silk Enzyme Powder – твій must-have для делікатного очищення та сяючої шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>521</t>
+  </si>
+  <si>
+    <t>521(1)</t>
+  </si>
+  <si>
+    <t>Пінка для сухої та чутливої шкіри з канабісом Hydro Aloe Mousse 480 мл</t>
+  </si>
+  <si>
+    <t>✨ Luxury Gentle Cleansing Foam – делікатне очищення та комфорт! ✨
+🌿 Спеціальна формула для щоденного догляду:
+💧 Легка текстура ефективно видаляє забруднення та макіяж
+🌸 Вирівнює поверхню шкіри без відчуття стягнутості
+🛡️ Заспокоює подразнення та зменшує запалення
+🌟 Відновлює бар’єрні функції та дарує відчуття свіжості
+💚 Результат – чиста, м’яка та сяюча шкіра після кожного очищення!
+📌 Активні компоненти:
+🌱 Олія коноплі та чіа – насичені омега-кислотами, зменшують подразнення
+🌸 Екстракт ромашки – заспокоює чутливу шкіру
+💧 Інулін та Hydagen® Aquaporin – глибоке зволоження та еластичність
+🛡️ Д-пантенол та бетаїн – відновлення та захист бар’єру
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Очищувальна піна для обличчя
+Об’єм: 150 мл / 200 мл (залежно від упаковки)
+Призначення: Делікатне очищення, зволоження, відновлення
+Тип шкіри: Суха, чутлива
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Luxury Gentle Cleansing Foam – твій must-have для щоденного ніжного очищення та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>503</t>
+  </si>
+  <si>
+    <t>503(1)</t>
+  </si>
+  <si>
+    <t>Розкішне молочко для вмивання ОМЕГА  500 мл ніжне очищення</t>
+  </si>
+  <si>
+    <t>✨ Gentle Omega Cleansing – делікатне очищення та регенерація! ✨
+🌿 Багатофункціональна формула для щоденного догляду:
+💧 Ефективно видаляє макіяж та всі типи забруднень (водо- і жиророзчинні)
+🌸 Відновлює та інтенсивно регенерує шкіру
+🛡️ Попереджає подразнення та зневоднення
+⚡ Підтримує водно-ліпідний баланс
+🌟 Активізує кровообіг та покращує тургор
+💚 Результат – чиста, свіжа та сяюча шкіра без відчуття сухості!
+📌 Активні компоненти:
+🌱 Олія коноплі та чіа – насичені омега-кислотами, живлення та протизапальна дія
+🌸 Екстракт ромашки та центелли азіатської – заспокоюють та відновлюють
+💧 Hydagen® Aquaporin, PatcH2O, сечовина – інтенсивне зволоження та утримання вологи
+🛡️ Д-пантенол та натрій аскорбіл фосфат – антиоксидантний захист та регенерація
+📌 Показання до застосування:
+Суха та чутлива шкіра
+Подразнення та зневоднення
+Зниження тонусу
+Перші ознаки старіння
+Відновлення та захист бар’єрної функції
+✔️ Характеристики продукту:
+Тип: Очищуючий засіб для обличчя
+Об’єм: 150 мл / 200 мл (залежно від упаковки)
+Призначення: Очищення, регенерація, зволоження
+Тип шкіри: Суха, чутлива
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Gentle Omega Cleansing – твій must-have для щоденного делікатного очищення та сяйва шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>501</t>
+  </si>
+  <si>
+    <t>501(1)</t>
+  </si>
+  <si>
+    <t>Порозвужувальна себорегулювальна маска «босвелія» 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Boswellia Clay Mask Herbal Pore Control – чиста та збалансована шкіра! ✨
+🌿 Активна формула для проблемної шкіри:
+💧 Зменшує пори та контролює себум
+🌸 Знижує запалення, подразнення та почервоніння
+🛡️ Нормалізує мікробіом шкіри та створює антисептичний бар’єр
+⚡ Має тонізуючу та регенеруючу дію
+🌟 Покращує стан проблемної шкіри та дарує відчуття свіжості
+💚 Результат – матова, рівна та здорова шкіра без надлишку себуму!
+📌 Показання до застосування:
+Акне 1–3 ступеня, постакне
+Розширені пори, нерівний тон
+Атопічний дерматит, екзема, псоріаз
+Подразнення та свербіж
+📌 Активні компоненти:
+🌱 Олії виноградних та персикових кісточок – живлення та відновлення
+🌸 Каолін – глибоке очищення та себорегуляція
+💧 Д-пантенол, гліцерин, ніацинамід – зволоження та регенерація
+🛡️ Екстракти епілобіуму, прополісу, каштану та календули – протизапальна дія
+⚡ Кофеїн, Bosexil, Bix'Activ – контроль себуму та тонізуючий ефект
+🌟 Бісаболол, алантоїн, ацетил тетрапептид-15 – заспокоюють та відновлюють
+✔️ Характеристики продукту:
+Тип: Себорегулююча порозвужуюча маска
+Об’єм: 50 мл
+Призначення: Очищення, себорегуляція, протизапальна дія
+Тип шкіри: Проблемна, жирна, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Boswellia Clay Mask – твій must-have для чистої та збалансованої шкіри без недоліків! 🌟</t>
+  </si>
+  <si>
+    <t>408</t>
+  </si>
+  <si>
+    <t>408(1)</t>
+  </si>
+  <si>
+    <t>Нічний себорегулювальний флюїд «Азеламід» 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Azelamid Night Fluid – нічна терапія проти акне! ✨
+🌿 Лікувальна формула для проблемної шкіри:
+💧 Глибоко очищає пори та зменшує виділення себуму
+🌸 Усуває запалення та почервоніння
+🛡️ Відновлює баланс мікробіому та бар’єрні функції
+⚡ Заспокоює подразнення та прискорює регенерацію
+🌟 Дарує рівний тон та здоровий вигляд шкіри
+💚 Результат – чиста, матова та спокійна шкіра вже після кількох застосувань!
+📌 Активні компоненти:
+🌱 Bix'Activ та прополіс – пригнічують P.Acne, забезпечують антибактеріальний ефект
+🌸 Екстракт епілобіуму – регулює активність сальних залоз та мікробіом
+💧 Азелаїнова та саліцилова кислоти – відлущують та очищають пори
+🛡️ Босвелія – покращує мікроциркуляцію та зменшує почервоніння
+🌟 Ніацинамід та D-пантенол – заспокоюють та стимулюють відновлення
+🌸 Екстракти ромашки, шавлії та каштана – протизапальна та тонізуюча дія
+📌 Показання до застосування:
+Акне 1–3 ступеня
+Постакне та розширені пори
+Нерівний тон шкіри
+Атопічний дерматит, псоріаз, екзема
+Подразнення та свербіж
+✔️ Характеристики продукту:
+Тип: Нічний себорегулюючий флюїд
+Об’єм: 50 мл
+Призначення: Лікування акне, себорегуляція, протизапальна дія
+Тип шкіри: Проблемна, жирна, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Azelamid Night Fluid – твій must-have для нічного догляду та боротьби з акне! 🌟</t>
+  </si>
+  <si>
+    <t>409-1</t>
+  </si>
+  <si>
+    <t>409-1(1)</t>
+  </si>
+  <si>
+    <t>Трансдермальний санблок SPF 30 - 230 мл</t>
+  </si>
+  <si>
+    <t>✨ Therapeutic Sunscreen SPF 30 – захист та лікування! ✨
+🌿 Формула спеціально для проблемної шкіри:
+☀️ SPF 30 широкого спектра – надійний захист від UVA/UVB
+💧 Зменшує пори та контролює себум
+🌸 Лікує акне 1–3 ступеня та постакне
+🛡️ Бореться з дерматитом, псоріазом та екземою
+⚡ Вирівнює тон та зменшує почервоніння
+💚 Результат – здорова, матова та захищена шкіра без недоліків!
+📌 Активні компоненти:
+🌱 Ніацинамід – відновлює мікробіом та регулює себум
+🌸 Екстракт епілобіуму флешері – протизапальна дія
+💧 Бета-глюкан – відновлює та заспокоює
+🛡️ Екстракт бікс орлеана – зменшує пори та жирність
+🌟 Бісаболол, Д-пантенол, пантеніл триацетат – знімають подразнення та почервоніння
+⚡ Екстракт босвелії – ефективний при дерматиті та екземі
+🌸 Додатково: екстракти шавлії, алое, ромашки, прополіс, олії льону та винограду, токоферол ацетат
+📌 Показання до застосування:
+Акне 1–3 ступеня, постакне
+Себорея та розширені пори
+Атопічний дерматит, псоріаз, екзема
+Подразнення та свербіж
+Нерівний тон шкіри
+✔️ Характеристики продукту:
+Тип: Лікувальний сонцезахисний крем
+Об’єм: 50 мл / 100 мл / 230 мл
+Рівень захисту: SPF 30
+Призначення: Захист, лікування акне, себорегуляція, відновлення
+Тип шкіри: Проблемна, жирна, комбінована
+Бренд: Smart4Derma
+Країна виробництва: 🇺🇦 Україна
+🌟 Therapeutic Sunscreen SPF 30 – твій must-have для комплексного догляду та захисту проблемної шкіри! 🌟</t>
+  </si>
+  <si>
+    <t>406</t>
+  </si>
+  <si>
+    <t>406(1)</t>
   </si>
 </sst>
 </file>
@@ -6958,10 +7751,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -10961,354 +11754,704 @@
       </c>
     </row>
     <row r="113" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A113" s="17"/>
-      <c r="B113" s="18"/>
+      <c r="A113" s="17" t="s">
+        <v>1020</v>
+      </c>
+      <c r="B113" s="18" t="s">
+        <v>1018</v>
+      </c>
       <c r="C113" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D113" s="18"/>
-      <c r="E113" s="18"/>
+      <c r="D113" s="18">
+        <v>3200</v>
+      </c>
+      <c r="E113" s="18">
+        <v>2800</v>
+      </c>
       <c r="F113" s="18"/>
-      <c r="G113" s="8"/>
-      <c r="H113" s="18"/>
+      <c r="G113" s="8">
+        <v>21</v>
+      </c>
+      <c r="H113" s="18" t="s">
+        <v>961</v>
+      </c>
       <c r="I113" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J113" s="18"/>
-      <c r="K113" s="17"/>
+      <c r="J113" s="18" t="s">
+        <v>1019</v>
+      </c>
+      <c r="K113" s="17" t="s">
+        <v>1021</v>
+      </c>
     </row>
     <row r="114" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A114" s="17"/>
-      <c r="B114" s="18"/>
+      <c r="A114" s="17" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B114" s="18" t="s">
+        <v>1022</v>
+      </c>
       <c r="C114" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D114" s="18"/>
-      <c r="E114" s="18"/>
+      <c r="D114" s="18">
+        <v>3200</v>
+      </c>
+      <c r="E114" s="18">
+        <v>2740</v>
+      </c>
       <c r="F114" s="18"/>
-      <c r="G114" s="8"/>
-      <c r="H114" s="18"/>
+      <c r="G114" s="8">
+        <v>18</v>
+      </c>
+      <c r="H114" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I114" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J114" s="18"/>
-      <c r="K114" s="17"/>
+      <c r="J114" s="18" t="s">
+        <v>1023</v>
+      </c>
+      <c r="K114" s="17" t="s">
+        <v>1025</v>
+      </c>
     </row>
     <row r="115" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A115" s="17"/>
-      <c r="B115" s="18"/>
+      <c r="A115" s="17" t="s">
+        <v>1028</v>
+      </c>
+      <c r="B115" s="18" t="s">
+        <v>1026</v>
+      </c>
       <c r="C115" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D115" s="18"/>
-      <c r="E115" s="18"/>
+      <c r="D115" s="18">
+        <v>3000</v>
+      </c>
+      <c r="E115" s="18">
+        <v>2500</v>
+      </c>
       <c r="F115" s="18"/>
-      <c r="G115" s="8"/>
-      <c r="H115" s="18"/>
+      <c r="G115" s="8">
+        <v>21</v>
+      </c>
+      <c r="H115" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I115" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J115" s="18"/>
-      <c r="K115" s="17"/>
+      <c r="J115" s="18" t="s">
+        <v>1027</v>
+      </c>
+      <c r="K115" s="17" t="s">
+        <v>1029</v>
+      </c>
     </row>
     <row r="116" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A116" s="17"/>
-      <c r="B116" s="18"/>
+      <c r="A116" s="17" t="s">
+        <v>1032</v>
+      </c>
+      <c r="B116" s="18" t="s">
+        <v>1030</v>
+      </c>
       <c r="C116" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D116" s="18"/>
-      <c r="E116" s="18"/>
+      <c r="D116" s="18">
+        <v>2400</v>
+      </c>
+      <c r="E116" s="18">
+        <v>2000</v>
+      </c>
       <c r="F116" s="18"/>
-      <c r="G116" s="8"/>
-      <c r="H116" s="18"/>
+      <c r="G116" s="8">
+        <v>21</v>
+      </c>
+      <c r="H116" s="18" t="s">
+        <v>961</v>
+      </c>
       <c r="I116" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J116" s="18"/>
-      <c r="K116" s="17"/>
+      <c r="J116" s="18" t="s">
+        <v>1031</v>
+      </c>
+      <c r="K116" s="17" t="s">
+        <v>1033</v>
+      </c>
     </row>
     <row r="117" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A117" s="17"/>
-      <c r="B117" s="18"/>
+      <c r="A117" s="17" t="s">
+        <v>1036</v>
+      </c>
+      <c r="B117" s="18" t="s">
+        <v>1034</v>
+      </c>
       <c r="C117" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D117" s="18"/>
-      <c r="E117" s="18"/>
+      <c r="D117" s="18">
+        <v>2100</v>
+      </c>
+      <c r="E117" s="18">
+        <v>1800</v>
+      </c>
       <c r="F117" s="18"/>
-      <c r="G117" s="8"/>
-      <c r="H117" s="18"/>
+      <c r="G117" s="8">
+        <v>14</v>
+      </c>
+      <c r="H117" s="18" t="s">
+        <v>29</v>
+      </c>
       <c r="I117" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J117" s="18"/>
-      <c r="K117" s="17"/>
+      <c r="J117" s="18" t="s">
+        <v>840</v>
+      </c>
+      <c r="K117" s="17" t="s">
+        <v>1035</v>
+      </c>
     </row>
     <row r="118" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A118" s="17"/>
-      <c r="B118" s="18"/>
+      <c r="A118" s="17" t="s">
+        <v>1039</v>
+      </c>
+      <c r="B118" s="18" t="s">
+        <v>1037</v>
+      </c>
       <c r="C118" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D118" s="18"/>
-      <c r="E118" s="18"/>
+      <c r="D118" s="18">
+        <v>550</v>
+      </c>
+      <c r="E118" s="18">
+        <v>480</v>
+      </c>
       <c r="F118" s="18"/>
-      <c r="G118" s="8"/>
-      <c r="H118" s="18"/>
+      <c r="G118" s="8">
+        <v>16</v>
+      </c>
+      <c r="H118" s="18" t="s">
+        <v>998</v>
+      </c>
       <c r="I118" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J118" s="18"/>
-      <c r="K118" s="17"/>
+      <c r="J118" s="18" t="s">
+        <v>1038</v>
+      </c>
+      <c r="K118" s="17" t="s">
+        <v>1040</v>
+      </c>
     </row>
     <row r="119" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A119" s="17"/>
-      <c r="B119" s="18"/>
+      <c r="A119" s="17" t="s">
+        <v>1043</v>
+      </c>
+      <c r="B119" s="18" t="s">
+        <v>1041</v>
+      </c>
       <c r="C119" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D119" s="18"/>
-      <c r="E119" s="18"/>
+      <c r="D119" s="18">
+        <v>1900</v>
+      </c>
+      <c r="E119" s="18">
+        <v>1600</v>
+      </c>
       <c r="F119" s="18"/>
-      <c r="G119" s="8"/>
-      <c r="H119" s="18"/>
+      <c r="G119" s="8">
+        <v>18</v>
+      </c>
+      <c r="H119" s="18" t="s">
+        <v>971</v>
+      </c>
       <c r="I119" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J119" s="18"/>
-      <c r="K119" s="17"/>
+      <c r="J119" s="18" t="s">
+        <v>1042</v>
+      </c>
+      <c r="K119" s="17" t="s">
+        <v>1044</v>
+      </c>
     </row>
     <row r="120" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A120" s="17"/>
-      <c r="B120" s="18"/>
+      <c r="A120" s="17" t="s">
+        <v>1046</v>
+      </c>
+      <c r="B120" s="18" t="s">
+        <v>1045</v>
+      </c>
       <c r="C120" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D120" s="18"/>
-      <c r="E120" s="18"/>
+      <c r="D120" s="18">
+        <v>1500</v>
+      </c>
+      <c r="E120" s="18">
+        <v>1240</v>
+      </c>
       <c r="F120" s="18"/>
-      <c r="G120" s="8"/>
-      <c r="H120" s="18"/>
+      <c r="G120" s="8">
+        <v>17</v>
+      </c>
+      <c r="H120" s="18" t="s">
+        <v>971</v>
+      </c>
       <c r="I120" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J120" s="18"/>
-      <c r="K120" s="17"/>
+      <c r="J120" s="18" t="s">
+        <v>1048</v>
+      </c>
+      <c r="K120" s="17" t="s">
+        <v>1047</v>
+      </c>
     </row>
     <row r="121" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A121" s="17"/>
-      <c r="B121" s="18"/>
+      <c r="A121" s="17" t="s">
+        <v>1051</v>
+      </c>
+      <c r="B121" s="18" t="s">
+        <v>1049</v>
+      </c>
       <c r="C121" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D121" s="18"/>
-      <c r="E121" s="18"/>
+      <c r="D121" s="18">
+        <v>1700</v>
+      </c>
+      <c r="E121" s="18">
+        <v>1540</v>
+      </c>
       <c r="F121" s="18"/>
-      <c r="G121" s="8"/>
-      <c r="H121" s="18"/>
+      <c r="G121" s="8">
+        <v>15</v>
+      </c>
+      <c r="H121" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I121" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J121" s="18"/>
-      <c r="K121" s="17"/>
+      <c r="J121" s="18" t="s">
+        <v>1050</v>
+      </c>
+      <c r="K121" s="17" t="s">
+        <v>1052</v>
+      </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A122" s="17"/>
-      <c r="B122" s="18"/>
+      <c r="A122" s="17" t="s">
+        <v>1055</v>
+      </c>
+      <c r="B122" s="18" t="s">
+        <v>1053</v>
+      </c>
       <c r="C122" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D122" s="18"/>
-      <c r="E122" s="18"/>
+      <c r="D122" s="18">
+        <v>2400</v>
+      </c>
+      <c r="E122" s="18">
+        <v>2000</v>
+      </c>
       <c r="F122" s="18"/>
-      <c r="G122" s="8"/>
-      <c r="H122" s="18"/>
+      <c r="G122" s="8">
+        <v>24</v>
+      </c>
+      <c r="H122" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I122" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J122" s="18"/>
-      <c r="K122" s="17"/>
+      <c r="J122" s="18" t="s">
+        <v>1054</v>
+      </c>
+      <c r="K122" s="17" t="s">
+        <v>1056</v>
+      </c>
     </row>
     <row r="123" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A123" s="17"/>
-      <c r="B123" s="18"/>
+      <c r="A123" s="17" t="s">
+        <v>1059</v>
+      </c>
+      <c r="B123" s="18" t="s">
+        <v>1057</v>
+      </c>
       <c r="C123" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D123" s="18"/>
-      <c r="E123" s="18"/>
+      <c r="D123" s="18">
+        <v>2400</v>
+      </c>
+      <c r="E123" s="18">
+        <v>2000</v>
+      </c>
       <c r="F123" s="18"/>
-      <c r="G123" s="8"/>
-      <c r="H123" s="18"/>
+      <c r="G123" s="8">
+        <v>25</v>
+      </c>
+      <c r="H123" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I123" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J123" s="18"/>
-      <c r="K123" s="17"/>
+      <c r="J123" s="18" t="s">
+        <v>1058</v>
+      </c>
+      <c r="K123" s="17" t="s">
+        <v>1060</v>
+      </c>
     </row>
     <row r="124" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A124" s="17"/>
-      <c r="B124" s="18"/>
+      <c r="A124" s="17" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B124" s="18" t="s">
+        <v>1061</v>
+      </c>
       <c r="C124" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D124" s="18"/>
-      <c r="E124" s="18"/>
+      <c r="D124" s="18">
+        <v>1500</v>
+      </c>
+      <c r="E124" s="18">
+        <v>1260</v>
+      </c>
       <c r="F124" s="18"/>
-      <c r="G124" s="8"/>
-      <c r="H124" s="18"/>
+      <c r="G124" s="8">
+        <v>21</v>
+      </c>
+      <c r="H124" s="18" t="s">
+        <v>961</v>
+      </c>
       <c r="I124" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J124" s="18"/>
-      <c r="K124" s="17"/>
+      <c r="J124" s="18" t="s">
+        <v>1062</v>
+      </c>
+      <c r="K124" s="17" t="s">
+        <v>1064</v>
+      </c>
     </row>
     <row r="125" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A125" s="17"/>
-      <c r="B125" s="18"/>
+      <c r="A125" s="17" t="s">
+        <v>1067</v>
+      </c>
+      <c r="B125" s="18" t="s">
+        <v>1065</v>
+      </c>
       <c r="C125" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D125" s="18"/>
-      <c r="E125" s="18"/>
+      <c r="D125" s="18">
+        <v>1400</v>
+      </c>
+      <c r="E125" s="18">
+        <v>1220</v>
+      </c>
       <c r="F125" s="18"/>
-      <c r="G125" s="8"/>
-      <c r="H125" s="18"/>
+      <c r="G125" s="8">
+        <v>25</v>
+      </c>
+      <c r="H125" s="18" t="s">
+        <v>29</v>
+      </c>
       <c r="I125" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J125" s="18"/>
-      <c r="K125" s="17"/>
+      <c r="J125" s="18" t="s">
+        <v>1066</v>
+      </c>
+      <c r="K125" s="17" t="s">
+        <v>1068</v>
+      </c>
     </row>
     <row r="126" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A126" s="17"/>
-      <c r="B126" s="18"/>
+      <c r="A126" s="17" t="s">
+        <v>1072</v>
+      </c>
+      <c r="B126" s="18" t="s">
+        <v>1069</v>
+      </c>
       <c r="C126" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D126" s="18"/>
-      <c r="E126" s="18"/>
+      <c r="D126" s="18">
+        <v>1500</v>
+      </c>
+      <c r="E126" s="18">
+        <v>1300</v>
+      </c>
       <c r="F126" s="18"/>
-      <c r="G126" s="8"/>
-      <c r="H126" s="18"/>
+      <c r="G126" s="8">
+        <v>21</v>
+      </c>
+      <c r="H126" s="18" t="s">
+        <v>29</v>
+      </c>
       <c r="I126" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J126" s="18"/>
-      <c r="K126" s="17"/>
+      <c r="J126" s="18" t="s">
+        <v>1070</v>
+      </c>
+      <c r="K126" s="17" t="s">
+        <v>1071</v>
+      </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A127" s="17"/>
-      <c r="B127" s="18"/>
+      <c r="A127" s="17" t="s">
+        <v>1075</v>
+      </c>
+      <c r="B127" s="18" t="s">
+        <v>1073</v>
+      </c>
       <c r="C127" s="18" t="s">
         <v>653</v>
       </c>
-      <c r="D127" s="18"/>
-      <c r="E127" s="18"/>
+      <c r="D127" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E127" s="18">
+        <v>1440</v>
+      </c>
       <c r="F127" s="18"/>
-      <c r="G127" s="8"/>
-      <c r="H127" s="18"/>
+      <c r="G127" s="8">
+        <v>15</v>
+      </c>
+      <c r="H127" s="18" t="s">
+        <v>971</v>
+      </c>
       <c r="I127" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J127" s="18"/>
-      <c r="K127" s="17"/>
+      <c r="J127" s="18" t="s">
+        <v>1074</v>
+      </c>
+      <c r="K127" s="17" t="s">
+        <v>1076</v>
+      </c>
     </row>
     <row r="128" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A128" s="17"/>
-      <c r="B128" s="18"/>
-      <c r="C128" s="18"/>
-      <c r="D128" s="18"/>
-      <c r="E128" s="18"/>
+      <c r="A128" s="17" t="s">
+        <v>1079</v>
+      </c>
+      <c r="B128" s="18" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C128" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D128" s="18">
+        <v>1100</v>
+      </c>
+      <c r="E128" s="18">
+        <v>750</v>
+      </c>
       <c r="F128" s="18"/>
-      <c r="G128" s="8"/>
-      <c r="H128" s="18"/>
+      <c r="G128" s="8">
+        <v>18</v>
+      </c>
+      <c r="H128" s="18" t="s">
+        <v>932</v>
+      </c>
       <c r="I128" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J128" s="18"/>
-      <c r="K128" s="17"/>
+      <c r="J128" s="18" t="s">
+        <v>1078</v>
+      </c>
+      <c r="K128" s="17" t="s">
+        <v>1080</v>
+      </c>
     </row>
     <row r="129" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A129" s="17"/>
-      <c r="B129" s="18"/>
-      <c r="C129" s="18"/>
-      <c r="D129" s="18"/>
-      <c r="E129" s="18"/>
+      <c r="A129" s="17" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B129" s="18" t="s">
+        <v>1081</v>
+      </c>
+      <c r="C129" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D129" s="18">
+        <v>1600</v>
+      </c>
+      <c r="E129" s="18">
+        <v>1300</v>
+      </c>
       <c r="F129" s="18"/>
-      <c r="G129" s="8"/>
-      <c r="H129" s="18"/>
+      <c r="G129" s="8">
+        <v>12</v>
+      </c>
+      <c r="H129" s="18" t="s">
+        <v>980</v>
+      </c>
       <c r="I129" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J129" s="18"/>
-      <c r="K129" s="17"/>
+      <c r="J129" s="18" t="s">
+        <v>1082</v>
+      </c>
+      <c r="K129" s="17" t="s">
+        <v>1084</v>
+      </c>
     </row>
     <row r="130" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A130" s="17"/>
-      <c r="B130" s="18"/>
-      <c r="C130" s="18"/>
-      <c r="D130" s="18"/>
-      <c r="E130" s="18"/>
+      <c r="A130" s="17" t="s">
+        <v>1087</v>
+      </c>
+      <c r="B130" s="18" t="s">
+        <v>1085</v>
+      </c>
+      <c r="C130" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D130" s="18">
+        <v>1300</v>
+      </c>
+      <c r="E130" s="18">
+        <v>1140</v>
+      </c>
       <c r="F130" s="18"/>
-      <c r="G130" s="8"/>
-      <c r="H130" s="18"/>
+      <c r="G130" s="8">
+        <v>15</v>
+      </c>
+      <c r="H130" s="18" t="s">
+        <v>971</v>
+      </c>
       <c r="I130" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J130" s="18"/>
-      <c r="K130" s="17"/>
+      <c r="J130" s="18" t="s">
+        <v>1086</v>
+      </c>
+      <c r="K130" s="17" t="s">
+        <v>1088</v>
+      </c>
     </row>
     <row r="131" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A131" s="17"/>
-      <c r="B131" s="18"/>
-      <c r="C131" s="18"/>
-      <c r="D131" s="18"/>
-      <c r="E131" s="18"/>
+      <c r="A131" s="17" t="s">
+        <v>1091</v>
+      </c>
+      <c r="B131" s="18" t="s">
+        <v>1089</v>
+      </c>
+      <c r="C131" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D131" s="18">
+        <v>1400</v>
+      </c>
+      <c r="E131" s="18">
+        <v>1240</v>
+      </c>
       <c r="F131" s="18"/>
-      <c r="G131" s="8"/>
-      <c r="H131" s="18"/>
+      <c r="G131" s="8">
+        <v>19</v>
+      </c>
+      <c r="H131" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I131" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J131" s="18"/>
-      <c r="K131" s="17"/>
+      <c r="J131" s="18" t="s">
+        <v>1090</v>
+      </c>
+      <c r="K131" s="17" t="s">
+        <v>1092</v>
+      </c>
     </row>
     <row r="132" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A132" s="17"/>
-      <c r="B132" s="18"/>
-      <c r="C132" s="18"/>
-      <c r="D132" s="18"/>
-      <c r="E132" s="18"/>
+      <c r="A132" s="17" t="s">
+        <v>1095</v>
+      </c>
+      <c r="B132" s="18" t="s">
+        <v>1093</v>
+      </c>
+      <c r="C132" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D132" s="18">
+        <v>2500</v>
+      </c>
+      <c r="E132" s="18">
+        <v>2200</v>
+      </c>
       <c r="F132" s="18"/>
-      <c r="G132" s="8"/>
-      <c r="H132" s="18"/>
+      <c r="G132" s="8">
+        <v>25</v>
+      </c>
+      <c r="H132" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I132" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J132" s="18"/>
-      <c r="K132" s="17"/>
+      <c r="J132" s="18" t="s">
+        <v>1094</v>
+      </c>
+      <c r="K132" s="17" t="s">
+        <v>1096</v>
+      </c>
     </row>
     <row r="133" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A133" s="17"/>
-      <c r="B133" s="18"/>
-      <c r="C133" s="18"/>
-      <c r="D133" s="18"/>
-      <c r="E133" s="18"/>
+      <c r="A133" s="17" t="s">
+        <v>1099</v>
+      </c>
+      <c r="B133" s="18" t="s">
+        <v>1097</v>
+      </c>
+      <c r="C133" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D133" s="18">
+        <v>1800</v>
+      </c>
+      <c r="E133" s="18">
+        <v>1440</v>
+      </c>
       <c r="F133" s="18"/>
-      <c r="G133" s="8"/>
-      <c r="H133" s="18"/>
+      <c r="G133" s="8">
+        <v>16</v>
+      </c>
+      <c r="H133" s="18" t="s">
+        <v>928</v>
+      </c>
       <c r="I133" s="18" t="s">
         <v>657</v>
       </c>
-      <c r="J133" s="18"/>
-      <c r="K133" s="17"/>
+      <c r="J133" s="18" t="s">
+        <v>1098</v>
+      </c>
+      <c r="K133" s="17" t="s">
+        <v>1100</v>
+      </c>
     </row>
     <row r="134" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A134" s="17"/>
       <c r="B134" s="18"/>
-      <c r="C134" s="18"/>
+      <c r="C134" s="18" t="s">
+        <v>653</v>
+      </c>
       <c r="D134" s="18"/>
       <c r="E134" s="18"/>
       <c r="F134" s="18"/>
@@ -11323,7 +12466,9 @@
     <row r="135" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A135" s="17"/>
       <c r="B135" s="18"/>
-      <c r="C135" s="18"/>
+      <c r="C135" s="18" t="s">
+        <v>653</v>
+      </c>
       <c r="D135" s="18"/>
       <c r="E135" s="18"/>
       <c r="F135" s="18"/>
@@ -11336,72 +12481,216 @@
       <c r="K135" s="17"/>
     </row>
     <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A136" s="17"/>
+      <c r="B136" s="18"/>
+      <c r="C136" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D136" s="18"/>
+      <c r="E136" s="18"/>
+      <c r="F136" s="18"/>
       <c r="G136" s="8"/>
+      <c r="H136" s="18"/>
+      <c r="I136" s="18"/>
+      <c r="J136" s="18"/>
+      <c r="K136" s="17"/>
     </row>
     <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A137" s="17"/>
+      <c r="B137" s="18"/>
+      <c r="C137" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D137" s="18"/>
+      <c r="E137" s="18"/>
+      <c r="F137" s="18"/>
       <c r="G137" s="8"/>
+      <c r="H137" s="18"/>
+      <c r="I137" s="18"/>
+      <c r="J137" s="18"/>
+      <c r="K137" s="17"/>
     </row>
     <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A138" s="17"/>
+      <c r="B138" s="18"/>
+      <c r="C138" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D138" s="18"/>
+      <c r="E138" s="18"/>
+      <c r="F138" s="18"/>
       <c r="G138" s="8"/>
+      <c r="H138" s="18"/>
+      <c r="I138" s="18"/>
+      <c r="J138" s="18"/>
+      <c r="K138" s="17"/>
     </row>
     <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A139" s="17"/>
+      <c r="B139" s="18"/>
+      <c r="C139" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D139" s="18"/>
+      <c r="E139" s="18"/>
+      <c r="F139" s="18"/>
       <c r="G139" s="8"/>
+      <c r="H139" s="18"/>
+      <c r="I139" s="18"/>
+      <c r="J139" s="18"/>
+      <c r="K139" s="17"/>
     </row>
     <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A140" s="17"/>
+      <c r="B140" s="18"/>
+      <c r="C140" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D140" s="18"/>
+      <c r="E140" s="18"/>
+      <c r="F140" s="18"/>
       <c r="G140" s="8"/>
+      <c r="H140" s="18"/>
+      <c r="I140" s="18"/>
+      <c r="J140" s="18"/>
+      <c r="K140" s="17"/>
     </row>
     <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A141" s="17"/>
+      <c r="B141" s="18"/>
+      <c r="C141" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D141" s="18"/>
+      <c r="E141" s="18"/>
+      <c r="F141" s="18"/>
       <c r="G141" s="8"/>
+      <c r="H141" s="18"/>
+      <c r="I141" s="18"/>
+      <c r="J141" s="18"/>
+      <c r="K141" s="17"/>
     </row>
     <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A142" s="17"/>
+      <c r="B142" s="18"/>
+      <c r="C142" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D142" s="18"/>
+      <c r="E142" s="18"/>
+      <c r="F142" s="18"/>
       <c r="G142" s="8"/>
+      <c r="H142" s="18"/>
+      <c r="I142" s="18"/>
+      <c r="J142" s="18"/>
+      <c r="K142" s="17"/>
     </row>
     <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A143" s="17"/>
+      <c r="B143" s="18"/>
+      <c r="C143" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D143" s="18"/>
+      <c r="E143" s="18"/>
+      <c r="F143" s="18"/>
       <c r="G143" s="8"/>
+      <c r="H143" s="18"/>
+      <c r="I143" s="18"/>
+      <c r="J143" s="18"/>
+      <c r="K143" s="17"/>
     </row>
     <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A144" s="17"/>
+      <c r="B144" s="18"/>
+      <c r="C144" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D144" s="18"/>
+      <c r="E144" s="18"/>
+      <c r="F144" s="18"/>
       <c r="G144" s="8"/>
-    </row>
-    <row r="145" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="H144" s="18"/>
+      <c r="I144" s="18"/>
+      <c r="J144" s="18"/>
+      <c r="K144" s="17"/>
+    </row>
+    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A145" s="17"/>
+      <c r="B145" s="18"/>
+      <c r="C145" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D145" s="18"/>
+      <c r="E145" s="18"/>
+      <c r="F145" s="18"/>
       <c r="G145" s="8"/>
-    </row>
-    <row r="146" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="H145" s="18"/>
+      <c r="I145" s="18"/>
+      <c r="J145" s="18"/>
+      <c r="K145" s="17"/>
+    </row>
+    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A146" s="17"/>
+      <c r="B146" s="18"/>
+      <c r="C146" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D146" s="18"/>
+      <c r="E146" s="18"/>
+      <c r="F146" s="18"/>
       <c r="G146" s="8"/>
-    </row>
-    <row r="147" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="H146" s="18"/>
+      <c r="I146" s="18"/>
+      <c r="J146" s="18"/>
+      <c r="K146" s="17"/>
+    </row>
+    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A147" s="17"/>
+      <c r="B147" s="18"/>
+      <c r="C147" s="18" t="s">
+        <v>653</v>
+      </c>
+      <c r="D147" s="18"/>
+      <c r="E147" s="18"/>
+      <c r="F147" s="18"/>
       <c r="G147" s="8"/>
-    </row>
-    <row r="148" spans="7:7" x14ac:dyDescent="0.3">
+      <c r="H147" s="18"/>
+      <c r="I147" s="18"/>
+      <c r="J147" s="18"/>
+      <c r="K147" s="17"/>
+    </row>
+    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G148" s="8"/>
     </row>
-    <row r="149" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G149" s="8"/>
     </row>
-    <row r="150" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G150" s="8"/>
     </row>
-    <row r="151" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G151" s="8"/>
     </row>
-    <row r="152" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G152" s="8"/>
     </row>
-    <row r="153" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G153" s="8"/>
     </row>
-    <row r="154" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G154" s="8"/>
     </row>
-    <row r="155" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G155" s="8"/>
     </row>
-    <row r="156" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G156" s="8"/>
     </row>
-    <row r="157" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G157" s="8"/>
     </row>
-    <row r="158" spans="7:7" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G158" s="8"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: gift sets tab + support mark-format sets sheet
- backend: sets sheet now also accepts a plain Артикул list (mark mode):
  listed SKUs become is_set with category Набори; composition format kept
- catalog: "Набори" tab via /catalog?sets=1 (header link, 🎁 chip, footer link)
</commit_message>
<xml_diff>
--- a/price.xlsx
+++ b/price.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ПРОЕКТ AI\ЛИЧНЫЕ НАРАБОТКИ\AI Skin Lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84258969-3C80-4057-88E3-80AA2C0BB7BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED556DBF-94AA-4499-AE67-7D5227448194}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Зручна таблиця" sheetId="1" r:id="rId1"/>

</xml_diff>